<commit_message>
Added simulations script and other items
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -9,10 +9,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9516"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9516" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Project Planner" sheetId="1" r:id="rId1"/>
+    <sheet name="Task List" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="Actual">(PeriodInActual*('Project Planner'!$E1&gt;0))*PeriodInPlan</definedName>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -232,21 +233,139 @@
   <si>
     <t>Eternal Inflation Project Planner</t>
   </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Assigned</t>
+  </si>
+  <si>
+    <t>Due</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Create task list and project planner spreadsheets</t>
+  </si>
+  <si>
+    <t>Test limiting gravity case</t>
+  </si>
+  <si>
+    <t>Check limiting case of gravitational instanton (where there should be no gravitational effects).</t>
+  </si>
+  <si>
+    <t>Set up a git repository for eternal inflation code</t>
+  </si>
+  <si>
+    <t>Email STR notifying leave of absence</t>
+  </si>
+  <si>
+    <t>Follow-up with Cathy regarding TA availability</t>
+  </si>
+  <si>
+    <t>Instanton approximation</t>
+  </si>
+  <si>
+    <t>Tunneling rate cutoff</t>
+  </si>
+  <si>
+    <t>What is a sensible order-of-magnitude cutoff for tunneling rate given by approximations?</t>
+  </si>
+  <si>
+    <t>Instanton write-up</t>
+  </si>
+  <si>
+    <t>Write up existing work on instantons in style of hybrid inflation notes.</t>
+  </si>
+  <si>
+    <t>Enroll in Independent Study and Seminars</t>
+  </si>
+  <si>
+    <t>Cosmology (just talks) or something else? (Particle Physics?)</t>
+  </si>
+  <si>
+    <t>Check thresholds &amp; units for all quantities in code</t>
+  </si>
+  <si>
+    <t>Gather to-date references for paper</t>
+  </si>
+  <si>
+    <t>Give Anthony permissions for git repo</t>
+  </si>
+  <si>
+    <t>Write scripts to run simulation</t>
+  </si>
+  <si>
+    <t>Finalize output structure from simulation</t>
+  </si>
+  <si>
+    <t>Which quantities should I record from the simulation?  How should I record them?</t>
+  </si>
+  <si>
+    <t>Write up description of false vacuum procedure</t>
+  </si>
+  <si>
+    <t>Locate gravitational and non-gravitational approximations to instanton action.</t>
+  </si>
+  <si>
+    <t>Submit teaching preferences</t>
+  </si>
+  <si>
+    <t>Enforce parameters</t>
+  </si>
+  <si>
+    <t>Populate "Code" appendix</t>
+  </si>
+  <si>
+    <t>Create an appendix to describe workings of the code in detail</t>
+  </si>
+  <si>
+    <t>Get proper references for code borrowed from Max Tegmark, Max Wainwright</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
+    <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="14"/>
@@ -479,101 +598,102 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="19">
+  <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="13" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="16" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="13" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="16" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -591,49 +711,60 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -648,8 +779,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="19">
+  <cellStyles count="20">
     <cellStyle name="% complete" xfId="16"/>
     <cellStyle name="% complete (beyond plan) legend" xfId="18"/>
     <cellStyle name="Activity" xfId="2"/>
@@ -662,6 +797,7 @@
     <cellStyle name="Heading 4" xfId="11" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Label" xfId="5"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
+    <cellStyle name="Normal 2" xfId="19"/>
     <cellStyle name="Percent Complete" xfId="6"/>
     <cellStyle name="Period Headers" xfId="3"/>
     <cellStyle name="Period Highlight Control" xfId="7"/>
@@ -670,7 +806,11 @@
     <cellStyle name="Project Headers" xfId="4"/>
     <cellStyle name="Title" xfId="8" builtinId="15" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
+    <dxf>
+      <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -829,6 +969,24 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F27" totalsRowShown="0">
+  <autoFilter ref="A1:F27"/>
+  <sortState ref="A2:F27">
+    <sortCondition ref="C1:C27"/>
+  </sortState>
+  <tableColumns count="6">
+    <tableColumn id="1" name="Task"/>
+    <tableColumn id="2" name="Assigned"/>
+    <tableColumn id="3" name="Due"/>
+    <tableColumn id="6" name=" " dataDxfId="0"/>
+    <tableColumn id="4" name="Review"/>
+    <tableColumn id="5" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1086,13 +1244,13 @@
       <c r="G1" s="10"/>
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
@@ -1100,66 +1258,66 @@
         <v>1</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="29" t="s">
+      <c r="K2" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="31"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="36"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="29" t="s">
+      <c r="Q2" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="32"/>
-      <c r="S2" s="32"/>
-      <c r="T2" s="31"/>
+      <c r="R2" s="37"/>
+      <c r="S2" s="37"/>
+      <c r="T2" s="36"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="21" t="s">
+      <c r="V2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
-      <c r="Y2" s="33"/>
+      <c r="W2" s="27"/>
+      <c r="X2" s="27"/>
+      <c r="Y2" s="38"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="34" t="s">
+      <c r="AA2" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="35"/>
-      <c r="AC2" s="35"/>
-      <c r="AD2" s="35"/>
-      <c r="AE2" s="35"/>
-      <c r="AF2" s="35"/>
-      <c r="AG2" s="36"/>
+      <c r="AB2" s="40"/>
+      <c r="AC2" s="40"/>
+      <c r="AD2" s="40"/>
+      <c r="AE2" s="40"/>
+      <c r="AF2" s="40"/>
+      <c r="AG2" s="41"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="21" t="s">
+      <c r="AI2" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="22"/>
-      <c r="AK2" s="22"/>
-      <c r="AL2" s="22"/>
-      <c r="AM2" s="22"/>
-      <c r="AN2" s="22"/>
-      <c r="AO2" s="22"/>
-      <c r="AP2" s="22"/>
+      <c r="AJ2" s="27"/>
+      <c r="AK2" s="27"/>
+      <c r="AL2" s="27"/>
+      <c r="AM2" s="27"/>
+      <c r="AN2" s="27"/>
+      <c r="AO2" s="27"/>
+      <c r="AP2" s="27"/>
     </row>
     <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="26" t="s">
+      <c r="B3" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="33" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -1288,12 +1446,12 @@
       <c r="AW3" s="18"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="25"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -1489,7 +1647,7 @@
         <v>3</v>
       </c>
       <c r="D7" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" s="7">
         <v>0</v>
@@ -2008,38 +2166,38 @@
     <mergeCell ref="AA2:AG2"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:BO31">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="10" priority="1">
       <formula>PercentComplete</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>PercentCompleteBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>Actual</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>ActualBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="6">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>Plan</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="7">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>H$4=period_selected</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="11">
+    <cfRule type="expression" dxfId="4" priority="11">
       <formula>MOD(COLUMN(),2)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="12">
+    <cfRule type="expression" dxfId="3" priority="12">
       <formula>MOD(COLUMN(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:BO32">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:BO4">
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule type="expression" dxfId="1" priority="8">
       <formula>H$4=period_selected</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2075,4 +2233,419 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="43.5546875" style="21" customWidth="1"/>
+    <col min="2" max="3" width="9.77734375" style="21" customWidth="1"/>
+    <col min="4" max="4" width="5.21875" style="21" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" style="21" customWidth="1"/>
+    <col min="6" max="6" width="80.88671875" style="21" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="21" hidden="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C2" s="23">
+        <v>42983</v>
+      </c>
+      <c r="D2" s="24">
+        <v>1</v>
+      </c>
+      <c r="E2" s="23">
+        <v>42984</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C3" s="23">
+        <v>42983</v>
+      </c>
+      <c r="D3" s="24">
+        <v>1</v>
+      </c>
+      <c r="E3" s="23">
+        <v>42992</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C4" s="23">
+        <v>42983</v>
+      </c>
+      <c r="D4" s="24">
+        <v>1</v>
+      </c>
+      <c r="E4" s="23">
+        <v>42984</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C5" s="23">
+        <v>42984</v>
+      </c>
+      <c r="D5" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E5" s="23">
+        <v>42986</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C6" s="23">
+        <v>42984</v>
+      </c>
+      <c r="D6" s="24">
+        <v>1</v>
+      </c>
+      <c r="E6" s="23">
+        <v>42987</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C7" s="23">
+        <v>42986</v>
+      </c>
+      <c r="D7" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E7" s="23">
+        <v>42992</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C8" s="23">
+        <v>42990</v>
+      </c>
+      <c r="D8" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="23">
+        <v>42992</v>
+      </c>
+      <c r="F8" s="25" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C9" s="23">
+        <v>42990</v>
+      </c>
+      <c r="D9" s="24">
+        <v>0</v>
+      </c>
+      <c r="E9" s="23">
+        <v>42992</v>
+      </c>
+      <c r="F9" s="21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="23">
+        <v>42984</v>
+      </c>
+      <c r="C10" s="23">
+        <v>42992</v>
+      </c>
+      <c r="D10" s="24">
+        <v>0</v>
+      </c>
+      <c r="E10" s="23">
+        <v>42992</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C11" s="23">
+        <v>42992</v>
+      </c>
+      <c r="D11" s="24">
+        <v>1</v>
+      </c>
+      <c r="E11" s="23">
+        <v>42992</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="23">
+        <v>42984</v>
+      </c>
+      <c r="C12" s="23">
+        <v>42992</v>
+      </c>
+      <c r="D12" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="E12" s="23">
+        <v>42992</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C13" s="23">
+        <v>42999</v>
+      </c>
+      <c r="D13" s="24">
+        <v>0</v>
+      </c>
+      <c r="E13" s="23">
+        <v>42999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="23">
+        <v>42984</v>
+      </c>
+      <c r="C14" s="23">
+        <v>42999</v>
+      </c>
+      <c r="D14" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="23">
+        <v>42999</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="42" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" s="23">
+        <v>42986</v>
+      </c>
+      <c r="C15" s="23">
+        <v>42999</v>
+      </c>
+      <c r="D15" s="23">
+        <v>0</v>
+      </c>
+      <c r="E15" s="23">
+        <v>42999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="23">
+        <v>42984</v>
+      </c>
+      <c r="C16" s="23">
+        <v>43003</v>
+      </c>
+      <c r="D16" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="E16" s="23">
+        <v>43006</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C17" s="23">
+        <v>43006</v>
+      </c>
+      <c r="D17" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E17" s="23">
+        <v>43006</v>
+      </c>
+      <c r="F17" s="42" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="23">
+        <v>42986</v>
+      </c>
+      <c r="C18" s="23">
+        <v>43060</v>
+      </c>
+      <c r="D18" s="23">
+        <v>0.25</v>
+      </c>
+      <c r="E18" s="43">
+        <v>43060</v>
+      </c>
+      <c r="F18" s="42" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="23"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="23"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+  </sheetData>
+  <conditionalFormatting sqref="D2:D25">
+    <cfRule type="iconSet" priority="14">
+      <iconSet iconSet="5Quarters" showValue="0">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="num" val="0.2"/>
+        <cfvo type="num" val="0.4"/>
+        <cfvo type="num" val="0.6"/>
+        <cfvo type="num" val="0.8"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed action calculation with gravity
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="17726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="18201"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9516" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12324" windowHeight="8724" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Project Planner" sheetId="1" r:id="rId1"/>
@@ -28,16 +28,12 @@
     <definedName name="TitleRegion..BO60">'Project Planner'!$B$3:$B$4</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
-      <mx:ArchID Flags="2"/>
-    </ext>
-  </extLst>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -276,15 +272,9 @@
     <t>Tunneling rate cutoff</t>
   </si>
   <si>
-    <t>What is a sensible order-of-magnitude cutoff for tunneling rate given by approximations?</t>
-  </si>
-  <si>
     <t>Instanton write-up</t>
   </si>
   <si>
-    <t>Write up existing work on instantons in style of hybrid inflation notes.</t>
-  </si>
-  <si>
     <t>Enroll in Independent Study and Seminars</t>
   </si>
   <si>
@@ -312,9 +302,6 @@
     <t>Write up description of false vacuum procedure</t>
   </si>
   <si>
-    <t>Locate gravitational and non-gravitational approximations to instanton action.</t>
-  </si>
-  <si>
     <t>Submit teaching preferences</t>
   </si>
   <si>
@@ -328,6 +315,54 @@
   </si>
   <si>
     <t>Get proper references for code borrowed from Max Tegmark, Max Wainwright</t>
+  </si>
+  <si>
+    <t>Or decide he doesn't need them now.</t>
+  </si>
+  <si>
+    <t>A brief overview in the text of the paper, rather than an in-depth appendix</t>
+  </si>
+  <si>
+    <t>Write up notes on CDL instantons and prefactor calculation in style of hybrid inflation notes.</t>
+  </si>
+  <si>
+    <t>Clarify sections of instanton notes</t>
+  </si>
+  <si>
+    <t>Zero modes, rework/scrap beginning section</t>
+  </si>
+  <si>
+    <t>Thin wall criteria</t>
+  </si>
+  <si>
+    <t>Write down heuristic criteria for thin wall approximation to be valid</t>
+  </si>
+  <si>
+    <t>Find expression for bubble tension in TWA</t>
+  </si>
+  <si>
+    <t>Show equivalence of thin wall results</t>
+  </si>
+  <si>
+    <t>Check that Garriga and Matt Johnson's thesis agree</t>
+  </si>
+  <si>
+    <t>Look at Anthony's articles</t>
+  </si>
+  <si>
+    <t>Write up and incorporate "deep well approximation"</t>
+  </si>
+  <si>
+    <t>Figure out how gravity should be included in S_E</t>
+  </si>
+  <si>
+    <t>Review slicings of de Sitter space</t>
+  </si>
+  <si>
+    <t>Explain factor of 2</t>
+  </si>
+  <si>
+    <t>Settle issues with initial conditions</t>
   </si>
 </sst>
 </file>
@@ -338,13 +373,62 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -602,98 +686,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="16" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="23" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="16" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="23" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -711,60 +795,68 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="20" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -778,10 +870,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="20">
@@ -973,8 +1061,17 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F27" totalsRowShown="0">
-  <autoFilter ref="A1:F27"/>
-  <sortState ref="A2:F27">
+  <autoFilter ref="A1:F27">
+    <filterColumn colId="3">
+      <filters blank="1">
+        <filter val="0"/>
+        <filter val="0.25"/>
+        <filter val="0.5"/>
+        <filter val="0.75"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <sortState ref="A8:F27">
     <sortCondition ref="C1:C27"/>
   </sortState>
   <tableColumns count="6">
@@ -1244,80 +1341,80 @@
       <c r="G1" s="10"/>
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
       <c r="H2" s="12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="34" t="s">
+      <c r="K2" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="36"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="44"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="34" t="s">
+      <c r="Q2" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="37"/>
-      <c r="S2" s="37"/>
-      <c r="T2" s="36"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="44"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="26" t="s">
+      <c r="V2" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="27"/>
-      <c r="X2" s="27"/>
-      <c r="Y2" s="38"/>
+      <c r="W2" s="35"/>
+      <c r="X2" s="35"/>
+      <c r="Y2" s="46"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="39" t="s">
+      <c r="AA2" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="40"/>
-      <c r="AC2" s="40"/>
-      <c r="AD2" s="40"/>
-      <c r="AE2" s="40"/>
-      <c r="AF2" s="40"/>
-      <c r="AG2" s="41"/>
+      <c r="AB2" s="48"/>
+      <c r="AC2" s="48"/>
+      <c r="AD2" s="48"/>
+      <c r="AE2" s="48"/>
+      <c r="AF2" s="48"/>
+      <c r="AG2" s="49"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="26" t="s">
+      <c r="AI2" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="27"/>
-      <c r="AK2" s="27"/>
-      <c r="AL2" s="27"/>
-      <c r="AM2" s="27"/>
-      <c r="AN2" s="27"/>
-      <c r="AO2" s="27"/>
-      <c r="AP2" s="27"/>
+      <c r="AJ2" s="35"/>
+      <c r="AK2" s="35"/>
+      <c r="AL2" s="35"/>
+      <c r="AM2" s="35"/>
+      <c r="AN2" s="35"/>
+      <c r="AO2" s="35"/>
+      <c r="AP2" s="35"/>
     </row>
     <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="29" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="31" t="s">
+      <c r="B3" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="31" t="s">
+      <c r="D3" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="31" t="s">
+      <c r="E3" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="31" t="s">
+      <c r="F3" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="33" t="s">
+      <c r="G3" s="41" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -1446,12 +1543,12 @@
       <c r="AW3" s="18"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="30"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -1609,7 +1706,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G5" s="8">
         <v>0.2</v>
@@ -1758,7 +1855,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G12" s="8">
         <v>0.2</v>
@@ -2227,11 +2324,6 @@
   <headerFooter differentFirst="1">
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -2240,8 +2332,9 @@
   <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.5546875" style="21" customWidth="1"/>
-    <col min="2" max="3" width="9.77734375" style="21" customWidth="1"/>
+    <col min="1" max="1" width="46.5546875" style="21" customWidth="1"/>
+    <col min="2" max="2" width="9.77734375" style="21" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" style="21" customWidth="1"/>
     <col min="4" max="4" width="5.21875" style="21" customWidth="1"/>
     <col min="5" max="5" width="9.77734375" style="21" customWidth="1"/>
     <col min="6" max="6" width="80.88671875" style="21" customWidth="1"/>
@@ -2268,7 +2361,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
         <v>47</v>
       </c>
@@ -2285,7 +2378,7 @@
         <v>42984</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
         <v>48</v>
       </c>
@@ -2305,7 +2398,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>50</v>
       </c>
@@ -2322,9 +2415,9 @@
         <v>42984</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B5" s="23">
         <v>42983</v>
@@ -2333,95 +2426,95 @@
         <v>42984</v>
       </c>
       <c r="D5" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E5" s="23">
         <v>42986</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F5" s="25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B6" s="23">
         <v>42983</v>
       </c>
       <c r="C6" s="23">
-        <v>42984</v>
+        <v>42990</v>
       </c>
       <c r="D6" s="24">
         <v>1</v>
       </c>
       <c r="E6" s="23">
-        <v>42987</v>
-      </c>
-      <c r="F6" s="25" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>42990</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" s="23">
         <v>42983</v>
       </c>
       <c r="C7" s="23">
-        <v>42986</v>
+        <v>42990</v>
       </c>
       <c r="D7" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E7" s="23">
-        <v>42992</v>
-      </c>
-      <c r="F7" s="21" t="s">
-        <v>57</v>
+        <v>42991</v>
+      </c>
+      <c r="F7" s="27" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="21" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="B8" s="23">
-        <v>42983</v>
+        <v>42984</v>
       </c>
       <c r="C8" s="23">
-        <v>42990</v>
+        <v>42992</v>
       </c>
       <c r="D8" s="24">
         <v>0.25</v>
       </c>
       <c r="E8" s="23">
+        <v>43006</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" s="23">
+        <v>42990</v>
+      </c>
+      <c r="C9" s="23">
         <v>42992</v>
       </c>
-      <c r="F8" s="25" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="23">
-        <v>42983</v>
-      </c>
-      <c r="C9" s="23">
-        <v>42990</v>
-      </c>
       <c r="D9" s="24">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="E9" s="23">
-        <v>42992</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+        <v>43006</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B10" s="23">
         <v>42984</v>
@@ -2430,15 +2523,18 @@
         <v>42992</v>
       </c>
       <c r="D10" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="23">
         <v>42992</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F10" s="26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B11" s="23">
         <v>42983</v>
@@ -2453,92 +2549,98 @@
         <v>42992</v>
       </c>
       <c r="F11" s="21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="21" t="s">
-        <v>66</v>
+      <c r="A12" s="29" t="s">
+        <v>78</v>
       </c>
       <c r="B12" s="23">
-        <v>42984</v>
+        <v>42992</v>
       </c>
       <c r="C12" s="23">
         <v>42992</v>
       </c>
       <c r="D12" s="24">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="E12" s="23">
+        <v>43006</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="23">
+        <v>42990</v>
+      </c>
+      <c r="C13" s="23">
+        <v>42993</v>
+      </c>
+      <c r="D13" s="24">
+        <v>1</v>
+      </c>
+      <c r="E13" s="23">
+        <v>43006</v>
+      </c>
+      <c r="F13" s="27" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" s="23">
+        <v>42991</v>
+      </c>
+      <c r="C14" s="23">
+        <v>42993</v>
+      </c>
+      <c r="D14" s="24">
+        <v>0</v>
+      </c>
+      <c r="E14" s="23">
+        <v>43006</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="23">
         <v>42992</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="B13" s="23">
-        <v>42983</v>
-      </c>
-      <c r="C13" s="23">
-        <v>42999</v>
-      </c>
-      <c r="D13" s="24">
-        <v>0</v>
-      </c>
-      <c r="E13" s="23">
-        <v>42999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="23">
-        <v>42984</v>
-      </c>
-      <c r="C14" s="23">
-        <v>42999</v>
-      </c>
-      <c r="D14" s="24">
-        <v>0.5</v>
-      </c>
-      <c r="E14" s="23">
-        <v>42999</v>
-      </c>
-      <c r="F14" s="21" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="42" t="s">
-        <v>69</v>
-      </c>
-      <c r="B15" s="23">
-        <v>42986</v>
-      </c>
       <c r="C15" s="23">
-        <v>42999</v>
-      </c>
-      <c r="D15" s="23">
+        <v>42993</v>
+      </c>
+      <c r="D15" s="24">
         <v>0</v>
       </c>
       <c r="E15" s="23">
-        <v>42999</v>
+        <v>43006</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
-        <v>63</v>
+      <c r="A16" s="31" t="s">
+        <v>83</v>
       </c>
       <c r="B16" s="23">
-        <v>42984</v>
+        <v>42998</v>
       </c>
       <c r="C16" s="23">
-        <v>43003</v>
+        <v>42998</v>
       </c>
       <c r="D16" s="24">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E16" s="23">
         <v>43006</v>
@@ -2546,92 +2648,180 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B17" s="23">
         <v>42983</v>
       </c>
       <c r="C17" s="23">
-        <v>43006</v>
+        <v>42999</v>
       </c>
       <c r="D17" s="24">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E17" s="23">
         <v>43006</v>
       </c>
-      <c r="F17" s="42" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="42" t="s">
-        <v>70</v>
+      <c r="A18" s="21" t="s">
+        <v>62</v>
       </c>
       <c r="B18" s="23">
+        <v>42984</v>
+      </c>
+      <c r="C18" s="23">
+        <v>42999</v>
+      </c>
+      <c r="D18" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E18" s="23">
+        <v>43006</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="23">
         <v>42986</v>
       </c>
-      <c r="C18" s="23">
+      <c r="C19" s="23">
+        <v>42999</v>
+      </c>
+      <c r="D19" s="24">
+        <v>0</v>
+      </c>
+      <c r="E19" s="23">
+        <v>43006</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="23">
+        <v>42984</v>
+      </c>
+      <c r="C20" s="23">
+        <v>43003</v>
+      </c>
+      <c r="D20" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="E20" s="23">
+        <v>43006</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C21" s="23">
+        <v>43006</v>
+      </c>
+      <c r="D21" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E21" s="23">
+        <v>43006</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C22" s="23">
+        <v>42991</v>
+      </c>
+      <c r="D22" s="24">
+        <v>1</v>
+      </c>
+      <c r="E22" s="23">
+        <v>42999</v>
+      </c>
+      <c r="F22" s="29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C23" s="23">
+        <v>42991</v>
+      </c>
+      <c r="D23" s="24">
+        <v>1</v>
+      </c>
+      <c r="E23" s="23">
+        <v>42999</v>
+      </c>
+      <c r="F23" s="29" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" s="23">
+        <v>42986</v>
+      </c>
+      <c r="C24" s="23">
         <v>43060</v>
       </c>
-      <c r="D18" s="23">
-        <v>0.25</v>
-      </c>
-      <c r="E18" s="43">
-        <v>43060</v>
-      </c>
-      <c r="F18" s="42" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="23"/>
+      <c r="D24" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E24" s="23">
+        <v>43062</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="23"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3"/>
+      <c r="A25" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" s="23">
+        <v>43017</v>
+      </c>
+      <c r="C25" s="23">
+        <v>43020</v>
+      </c>
+      <c r="D25" s="24">
+        <v>0</v>
+      </c>
+      <c r="E25" s="23">
+        <v>43020</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D26" s="24"/>
+    </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3"/>
     <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3"/>
     <row r="29" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <conditionalFormatting sqref="D2:D25">
+  <conditionalFormatting sqref="D2:D26">
     <cfRule type="iconSet" priority="14">
       <iconSet iconSet="5Quarters" showValue="0">
         <cfvo type="percent" val="0"/>

</xml_diff>

<commit_message>
Fixed ODE solver with Jacobian and events
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -28,12 +28,11 @@
     <definedName name="TitleRegion..BO60">'Project Planner'!$B$3:$B$4</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -362,7 +361,52 @@
     <t>Explain factor of 2</t>
   </si>
   <si>
-    <t>Settle issues with initial conditions</t>
+    <t>Figure out why reduced action doesn't match</t>
+  </si>
+  <si>
+    <t>Shelf for now</t>
+  </si>
+  <si>
+    <t>Are Measures A and B implemented correctly in the code?</t>
+  </si>
+  <si>
+    <t>Check initial conditions</t>
+  </si>
+  <si>
+    <t>Can we impose constraints that select for observed quantities? Shelf for now?</t>
+  </si>
+  <si>
+    <t>Make sure all units are correct</t>
+  </si>
+  <si>
+    <t>Generate a script that loops over all cases we're interested in</t>
+  </si>
+  <si>
+    <t>Add volume terms for bubble interior to gravity action</t>
+  </si>
+  <si>
+    <t>Fix volume terms if missing surface term</t>
+  </si>
+  <si>
+    <t>Volume terms as they are might not take into account boundary term in integration by parts</t>
+  </si>
+  <si>
+    <t>Speed up numerical integration for instanton code</t>
+  </si>
+  <si>
+    <t>Avoid stiff diff eq. issues.  Q: Do we need to integrate twice?</t>
+  </si>
+  <si>
+    <t>Automate selection of tolerances</t>
+  </si>
+  <si>
+    <t>Specify Jacobian in ODE solver</t>
+  </si>
+  <si>
+    <t>Replace step solver with ODE events</t>
+  </si>
+  <si>
+    <t>Troubleshoot integration failures</t>
   </si>
 </sst>
 </file>
@@ -373,13 +417,27 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -686,98 +744,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="23" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="25" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="18" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="23" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="25" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -795,25 +853,27 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="22" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -822,41 +882,40 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -871,6 +930,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
   </cellXfs>
   <cellStyles count="20">
     <cellStyle name="% complete" xfId="16"/>
@@ -895,10 +955,6 @@
     <cellStyle name="Title" xfId="8" builtinId="15" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="11">
-    <dxf>
-      <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1041,6 +1097,10 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1060,25 +1120,31 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F27" totalsRowShown="0">
-  <autoFilter ref="A1:F27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F34" totalsRowShown="0">
+  <autoFilter ref="A1:F34">
     <filterColumn colId="3">
       <filters blank="1">
         <filter val="0"/>
         <filter val="0.25"/>
         <filter val="0.5"/>
-        <filter val="0.75"/>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters blank="1">
+        <dateGroupItem year="2017" month="10" dateTimeGrouping="month"/>
+        <dateGroupItem year="2017" month="11" dateTimeGrouping="month"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState ref="A8:F27">
-    <sortCondition ref="C1:C27"/>
+  <sortState ref="A10:F34">
+    <sortCondition descending="1" ref="D1:D34"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" name="Task"/>
     <tableColumn id="2" name="Assigned"/>
     <tableColumn id="3" name="Due"/>
-    <tableColumn id="6" name=" " dataDxfId="0"/>
+    <tableColumn id="6" name=" " dataDxfId="10"/>
     <tableColumn id="4" name="Review"/>
     <tableColumn id="5" name="Notes"/>
   </tableColumns>
@@ -1341,13 +1407,13 @@
       <c r="G1" s="10"/>
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
@@ -1355,66 +1421,66 @@
         <v>3</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="42" t="s">
+      <c r="K2" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="45"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="42" t="s">
+      <c r="Q2" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="45"/>
-      <c r="S2" s="45"/>
-      <c r="T2" s="44"/>
+      <c r="R2" s="46"/>
+      <c r="S2" s="46"/>
+      <c r="T2" s="45"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="34" t="s">
+      <c r="V2" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="35"/>
-      <c r="X2" s="35"/>
-      <c r="Y2" s="46"/>
+      <c r="W2" s="36"/>
+      <c r="X2" s="36"/>
+      <c r="Y2" s="47"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="47" t="s">
+      <c r="AA2" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="48"/>
-      <c r="AC2" s="48"/>
-      <c r="AD2" s="48"/>
-      <c r="AE2" s="48"/>
-      <c r="AF2" s="48"/>
-      <c r="AG2" s="49"/>
+      <c r="AB2" s="49"/>
+      <c r="AC2" s="49"/>
+      <c r="AD2" s="49"/>
+      <c r="AE2" s="49"/>
+      <c r="AF2" s="49"/>
+      <c r="AG2" s="50"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="34" t="s">
+      <c r="AI2" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="35"/>
-      <c r="AK2" s="35"/>
-      <c r="AL2" s="35"/>
-      <c r="AM2" s="35"/>
-      <c r="AN2" s="35"/>
-      <c r="AO2" s="35"/>
-      <c r="AP2" s="35"/>
+      <c r="AJ2" s="36"/>
+      <c r="AK2" s="36"/>
+      <c r="AL2" s="36"/>
+      <c r="AM2" s="36"/>
+      <c r="AN2" s="36"/>
+      <c r="AO2" s="36"/>
+      <c r="AP2" s="36"/>
     </row>
     <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="37" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="39" t="s">
+      <c r="B3" s="38" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="39" t="s">
+      <c r="E3" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="39" t="s">
+      <c r="F3" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="41" t="s">
+      <c r="G3" s="42" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -1543,12 +1609,12 @@
       <c r="AW3" s="18"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="38"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -2263,38 +2329,38 @@
     <mergeCell ref="AA2:AG2"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:BO31">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>PercentComplete</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="3">
+    <cfRule type="expression" dxfId="8" priority="3">
       <formula>PercentCompleteBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="4">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>Actual</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>ActualBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>Plan</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="7">
+    <cfRule type="expression" dxfId="4" priority="7">
       <formula>H$4=period_selected</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="11">
+    <cfRule type="expression" dxfId="3" priority="11">
       <formula>MOD(COLUMN(),2)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="12">
+    <cfRule type="expression" dxfId="2" priority="12">
       <formula>MOD(COLUMN(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:BO32">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:BO4">
-    <cfRule type="expression" dxfId="1" priority="8">
+    <cfRule type="expression" dxfId="0" priority="8">
       <formula>H$4=period_selected</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2329,7 +2395,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46.5546875" style="21" customWidth="1"/>
@@ -2362,45 +2428,48 @@
       </c>
     </row>
     <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
-        <v>47</v>
+      <c r="A2" s="29" t="s">
+        <v>81</v>
       </c>
       <c r="B2" s="23">
-        <v>42983</v>
+        <v>42992</v>
       </c>
       <c r="C2" s="23">
-        <v>42983</v>
+        <v>42993</v>
       </c>
       <c r="D2" s="24">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E2" s="23">
-        <v>42984</v>
+        <v>43006</v>
+      </c>
+      <c r="F2" s="33" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
-        <v>48</v>
+      <c r="A3" s="26" t="s">
+        <v>66</v>
       </c>
       <c r="B3" s="23">
-        <v>42983</v>
+        <v>42986</v>
       </c>
       <c r="C3" s="23">
-        <v>42983</v>
+        <v>42999</v>
       </c>
       <c r="D3" s="24">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E3" s="23">
-        <v>42992</v>
-      </c>
-      <c r="F3" s="21" t="s">
-        <v>49</v>
+        <v>43006</v>
+      </c>
+      <c r="F3" s="33" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B4" s="23">
         <v>42983</v>
@@ -2417,107 +2486,104 @@
     </row>
     <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B5" s="23">
         <v>42983</v>
       </c>
       <c r="C5" s="23">
-        <v>42984</v>
+        <v>42983</v>
       </c>
       <c r="D5" s="24">
         <v>1</v>
       </c>
       <c r="E5" s="23">
-        <v>42986</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>65</v>
+        <v>42992</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="23">
         <v>42983</v>
       </c>
       <c r="C6" s="23">
-        <v>42990</v>
+        <v>42983</v>
       </c>
       <c r="D6" s="24">
         <v>1</v>
       </c>
       <c r="E6" s="23">
-        <v>42990</v>
+        <v>42984</v>
       </c>
     </row>
     <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B7" s="23">
         <v>42983</v>
       </c>
       <c r="C7" s="23">
-        <v>42990</v>
+        <v>42984</v>
       </c>
       <c r="D7" s="24">
         <v>1</v>
       </c>
       <c r="E7" s="23">
+        <v>42986</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C8" s="23">
+        <v>42990</v>
+      </c>
+      <c r="D8" s="24">
+        <v>1</v>
+      </c>
+      <c r="E8" s="23">
+        <v>42990</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C9" s="23">
+        <v>42990</v>
+      </c>
+      <c r="D9" s="24">
+        <v>1</v>
+      </c>
+      <c r="E9" s="23">
         <v>42991</v>
       </c>
-      <c r="F7" s="27" t="s">
+      <c r="F9" s="27" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="B8" s="23">
-        <v>42984</v>
-      </c>
-      <c r="C8" s="23">
-        <v>42992</v>
-      </c>
-      <c r="D8" s="24">
-        <v>0.25</v>
-      </c>
-      <c r="E8" s="23">
-        <v>43006</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="30" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B10" s="23">
         <v>42990</v>
-      </c>
-      <c r="C9" s="23">
-        <v>42992</v>
-      </c>
-      <c r="D9" s="24">
-        <v>0.75</v>
-      </c>
-      <c r="E9" s="23">
-        <v>43006</v>
-      </c>
-      <c r="F9" s="32" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="23">
-        <v>42984</v>
       </c>
       <c r="C10" s="23">
         <v>42992</v>
@@ -2526,18 +2592,18 @@
         <v>1</v>
       </c>
       <c r="E10" s="23">
-        <v>42992</v>
-      </c>
-      <c r="F10" s="26" t="s">
-        <v>70</v>
+        <v>43027</v>
+      </c>
+      <c r="F10" s="32" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B11" s="23">
-        <v>42983</v>
+        <v>42984</v>
       </c>
       <c r="C11" s="23">
         <v>42992</v>
@@ -2548,28 +2614,28 @@
       <c r="E11" s="23">
         <v>42992</v>
       </c>
-      <c r="F11" s="21" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="29" t="s">
-        <v>78</v>
+      <c r="F11" s="26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="21" t="s">
+        <v>56</v>
       </c>
       <c r="B12" s="23">
-        <v>42992</v>
+        <v>42983</v>
       </c>
       <c r="C12" s="23">
         <v>42992</v>
       </c>
       <c r="D12" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E12" s="23">
-        <v>43006</v>
-      </c>
-      <c r="F12" s="29" t="s">
-        <v>79</v>
+        <v>42992</v>
+      </c>
+      <c r="F12" s="21" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -2592,236 +2658,400 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
-        <v>75</v>
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="31" t="s">
+        <v>83</v>
       </c>
       <c r="B14" s="23">
-        <v>42991</v>
+        <v>42998</v>
       </c>
       <c r="C14" s="23">
-        <v>42993</v>
+        <v>42998</v>
       </c>
       <c r="D14" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="23">
         <v>43006</v>
       </c>
-      <c r="F14" s="28" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="29" t="s">
-        <v>81</v>
+    </row>
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="21" t="s">
+        <v>53</v>
       </c>
       <c r="B15" s="23">
-        <v>42992</v>
+        <v>42983</v>
       </c>
       <c r="C15" s="23">
-        <v>42993</v>
+        <v>42991</v>
       </c>
       <c r="D15" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="23">
-        <v>43006</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="31" t="s">
-        <v>83</v>
+        <v>42999</v>
+      </c>
+      <c r="F15" s="29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
+        <v>54</v>
       </c>
       <c r="B16" s="23">
-        <v>42998</v>
+        <v>42983</v>
       </c>
       <c r="C16" s="23">
-        <v>42998</v>
+        <v>42991</v>
       </c>
       <c r="D16" s="24">
         <v>1</v>
       </c>
       <c r="E16" s="23">
+        <v>42999</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="23">
+        <v>43021</v>
+      </c>
+      <c r="C17" s="23">
+        <v>43021</v>
+      </c>
+      <c r="D17" s="24">
+        <v>1</v>
+      </c>
+      <c r="E17" s="23">
+        <v>43027</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" s="23">
+        <v>43021</v>
+      </c>
+      <c r="C18" s="23">
+        <v>43021</v>
+      </c>
+      <c r="D18" s="24">
+        <v>1</v>
+      </c>
+      <c r="E18" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F18" s="33"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="23">
+        <v>43021</v>
+      </c>
+      <c r="C19" s="23">
+        <v>43024</v>
+      </c>
+      <c r="D19" s="24">
+        <v>1</v>
+      </c>
+      <c r="E19" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F19" s="33" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="51" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="23">
+        <v>43021</v>
+      </c>
+      <c r="C20" s="23">
+        <v>43024</v>
+      </c>
+      <c r="D20" s="24">
+        <v>1</v>
+      </c>
+      <c r="E20" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F20" s="33"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="51" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" s="23">
+        <v>43021</v>
+      </c>
+      <c r="C21" s="23">
+        <v>43027</v>
+      </c>
+      <c r="D21" s="24">
+        <v>1</v>
+      </c>
+      <c r="E21" s="23">
+        <v>43023</v>
+      </c>
+      <c r="F21" s="33"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="23">
+        <v>42992</v>
+      </c>
+      <c r="C22" s="23">
+        <v>42992</v>
+      </c>
+      <c r="D22" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E22" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F22" s="29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="23">
+        <v>42984</v>
+      </c>
+      <c r="C23" s="23">
+        <v>42999</v>
+      </c>
+      <c r="D23" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E23" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F23" s="21" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C24" s="23">
         <v>43006</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="23">
-        <v>42983</v>
-      </c>
-      <c r="C17" s="23">
-        <v>42999</v>
-      </c>
-      <c r="D17" s="24">
-        <v>0</v>
-      </c>
-      <c r="E17" s="23">
-        <v>43006</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" s="23">
-        <v>42984</v>
-      </c>
-      <c r="C18" s="23">
-        <v>42999</v>
-      </c>
-      <c r="D18" s="24">
-        <v>0.5</v>
-      </c>
-      <c r="E18" s="23">
-        <v>43006</v>
-      </c>
-      <c r="F18" s="21" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="B19" s="23">
-        <v>42986</v>
-      </c>
-      <c r="C19" s="23">
-        <v>42999</v>
-      </c>
-      <c r="D19" s="24">
-        <v>0</v>
-      </c>
-      <c r="E19" s="23">
-        <v>43006</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" s="23">
-        <v>42984</v>
-      </c>
-      <c r="C20" s="23">
-        <v>43003</v>
-      </c>
-      <c r="D20" s="24">
-        <v>0.25</v>
-      </c>
-      <c r="E20" s="23">
-        <v>43006</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="B21" s="23">
-        <v>42983</v>
-      </c>
-      <c r="C21" s="23">
-        <v>43006</v>
-      </c>
-      <c r="D21" s="24">
-        <v>0.5</v>
-      </c>
-      <c r="E21" s="23">
-        <v>43006</v>
-      </c>
-      <c r="F21" s="26" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="23">
-        <v>42983</v>
-      </c>
-      <c r="C22" s="23">
-        <v>42991</v>
-      </c>
-      <c r="D22" s="24">
-        <v>1</v>
-      </c>
-      <c r="E22" s="23">
-        <v>42999</v>
-      </c>
-      <c r="F22" s="29" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="B23" s="23">
-        <v>42983</v>
-      </c>
-      <c r="C23" s="23">
-        <v>42991</v>
-      </c>
-      <c r="D23" s="24">
-        <v>1</v>
-      </c>
-      <c r="E23" s="23">
-        <v>42999</v>
-      </c>
-      <c r="F23" s="29" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="B24" s="23">
-        <v>42986</v>
-      </c>
-      <c r="C24" s="23">
-        <v>43060</v>
       </c>
       <c r="D24" s="24">
         <v>0.5</v>
       </c>
       <c r="E24" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="23">
+        <v>42986</v>
+      </c>
+      <c r="C25" s="23">
+        <v>43060</v>
+      </c>
+      <c r="D25" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E25" s="23">
         <v>43062</v>
       </c>
-      <c r="F24" s="26" t="s">
+      <c r="F25" s="26" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="B25" s="23">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="51" t="s">
+        <v>100</v>
+      </c>
+      <c r="B26" s="23">
+        <v>43021</v>
+      </c>
+      <c r="C26" s="23">
+        <v>43024</v>
+      </c>
+      <c r="D26" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E26" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F26" s="33"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="23">
+        <v>42984</v>
+      </c>
+      <c r="C27" s="23">
+        <v>42992</v>
+      </c>
+      <c r="D27" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="E27" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" s="23">
+        <v>42984</v>
+      </c>
+      <c r="C28" s="23">
+        <v>43003</v>
+      </c>
+      <c r="D28" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="E28" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F28" s="33" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="B29" s="23">
+        <v>43021</v>
+      </c>
+      <c r="C29" s="23">
+        <v>43027</v>
+      </c>
+      <c r="D29" s="24">
+        <v>0</v>
+      </c>
+      <c r="E29" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F29" s="34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="B30" s="23">
+        <v>42991</v>
+      </c>
+      <c r="C30" s="23">
+        <v>42993</v>
+      </c>
+      <c r="D30" s="24">
+        <v>0</v>
+      </c>
+      <c r="E30" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F30" s="28" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="23">
+        <v>42983</v>
+      </c>
+      <c r="C31" s="23">
+        <v>42999</v>
+      </c>
+      <c r="D31" s="24">
+        <v>0</v>
+      </c>
+      <c r="E31" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F31" s="33" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32" s="23">
         <v>43017</v>
       </c>
-      <c r="C25" s="23">
+      <c r="C32" s="23">
         <v>43020</v>
       </c>
-      <c r="D25" s="24">
-        <v>0</v>
-      </c>
-      <c r="E25" s="23">
-        <v>43020</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="D26" s="24"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="D32" s="24">
+        <v>0</v>
+      </c>
+      <c r="E32" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F32" s="33" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="51" t="s">
+        <v>97</v>
+      </c>
+      <c r="B33" s="23">
+        <v>43021</v>
+      </c>
+      <c r="C33" s="23">
+        <v>43027</v>
+      </c>
+      <c r="D33" s="24">
+        <v>0</v>
+      </c>
+      <c r="E33" s="23">
+        <v>43027</v>
+      </c>
+      <c r="F33" s="33"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="23"/>
+    </row>
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="36" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <conditionalFormatting sqref="D2:D26">
+  <conditionalFormatting sqref="D2:D34">
     <cfRule type="iconSet" priority="14">
       <iconSet iconSet="5Quarters" showValue="0">
         <cfvo type="percent" val="0"/>

</xml_diff>

<commit_message>
Added preemptive check for inflation in neighboring basin
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -30,12 +30,11 @@
     <definedName name="TitleRegion..BO60">'Project Planner'!$B$3:$B$4</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="160">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -564,6 +563,30 @@
   <si>
     <t>Check for inflation on other side of barrier</t>
   </si>
+  <si>
+    <t>What is flagStartAtMaximum?</t>
+  </si>
+  <si>
+    <t>Scan param files in script</t>
+  </si>
+  <si>
+    <t>Precompute N_max e-foldings in neighboring basins</t>
+  </si>
+  <si>
+    <t>Make a table of all status codes</t>
+  </si>
+  <si>
+    <t>Line</t>
+  </si>
+  <si>
+    <t>Deprecated?</t>
+  </si>
+  <si>
+    <t>Email Matt Johnson</t>
+  </si>
+  <si>
+    <t>Optimize find_phistart</t>
+  </si>
 </sst>
 </file>
 
@@ -573,13 +596,27 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="37" x14ac:knownFonts="1">
+  <fonts count="39" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -977,98 +1014,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="32" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="34" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="25" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="27" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="35" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="37" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="35" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="35" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="32" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="34" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="25" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="27" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="33" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="28" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="30" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="35" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="37" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -1086,25 +1123,27 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="34" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -1119,61 +1158,85 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -1188,6 +1251,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
   </cellXfs>
   <cellStyles count="20">
@@ -1212,7 +1276,7 @@
     <cellStyle name="Project Headers" xfId="4"/>
     <cellStyle name="Title" xfId="8" builtinId="15" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="31">
+  <dxfs count="32">
     <dxf>
       <fill>
         <patternFill>
@@ -1704,6 +1768,24 @@
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1723,9 +1805,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F44" totalsRowShown="0">
-  <autoFilter ref="A1:F44">
-    <filterColumn colId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:G49" totalsRowShown="0">
+  <autoFilter ref="A1:G49">
+    <filterColumn colId="4">
       <filters blank="1">
         <filter val="0"/>
         <filter val="0.25"/>
@@ -1734,11 +1816,12 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState ref="A27:F44">
-    <sortCondition descending="1" ref="D1:D44"/>
+  <sortState ref="A27:G49">
+    <sortCondition descending="1" ref="E1:E49"/>
   </sortState>
-  <tableColumns count="6">
+  <tableColumns count="7">
     <tableColumn id="1" name="Task"/>
+    <tableColumn id="7" name="Line" dataDxfId="31" dataCellStyle="Normal 2"/>
     <tableColumn id="2" name="Assigned"/>
     <tableColumn id="3" name="Due"/>
     <tableColumn id="6" name=" " dataDxfId="30"/>
@@ -2043,13 +2126,13 @@
       <c r="G1" s="10"/>
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
@@ -2057,66 +2140,66 @@
         <v>8</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="58" t="s">
+      <c r="K2" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="60"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="70"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="58" t="s">
+      <c r="Q2" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="61"/>
-      <c r="S2" s="61"/>
-      <c r="T2" s="60"/>
+      <c r="R2" s="71"/>
+      <c r="S2" s="71"/>
+      <c r="T2" s="70"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="50" t="s">
+      <c r="V2" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="51"/>
-      <c r="X2" s="51"/>
-      <c r="Y2" s="62"/>
+      <c r="W2" s="61"/>
+      <c r="X2" s="61"/>
+      <c r="Y2" s="72"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="63" t="s">
+      <c r="AA2" s="73" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="64"/>
-      <c r="AC2" s="64"/>
-      <c r="AD2" s="64"/>
-      <c r="AE2" s="64"/>
-      <c r="AF2" s="64"/>
-      <c r="AG2" s="65"/>
+      <c r="AB2" s="74"/>
+      <c r="AC2" s="74"/>
+      <c r="AD2" s="74"/>
+      <c r="AE2" s="74"/>
+      <c r="AF2" s="74"/>
+      <c r="AG2" s="75"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="50" t="s">
+      <c r="AI2" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="51"/>
-      <c r="AK2" s="51"/>
-      <c r="AL2" s="51"/>
-      <c r="AM2" s="51"/>
-      <c r="AN2" s="51"/>
-      <c r="AO2" s="51"/>
-      <c r="AP2" s="51"/>
+      <c r="AJ2" s="61"/>
+      <c r="AK2" s="61"/>
+      <c r="AL2" s="61"/>
+      <c r="AM2" s="61"/>
+      <c r="AN2" s="61"/>
+      <c r="AO2" s="61"/>
+      <c r="AP2" s="61"/>
     </row>
     <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="53" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="55" t="s">
+      <c r="B3" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="55" t="s">
+      <c r="D3" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="55" t="s">
+      <c r="F3" s="65" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="57" t="s">
+      <c r="G3" s="67" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -2245,12 +2328,12 @@
       <c r="AW3" s="18"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="54"/>
-      <c r="C4" s="56"/>
-      <c r="D4" s="56"/>
-      <c r="E4" s="56"/>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -3035,846 +3118,980 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46.5546875" style="21" customWidth="1"/>
-    <col min="2" max="2" width="9.77734375" style="21" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" style="21" customWidth="1"/>
-    <col min="4" max="4" width="5.21875" style="21" customWidth="1"/>
-    <col min="5" max="5" width="9.77734375" style="21" customWidth="1"/>
-    <col min="6" max="6" width="80.88671875" style="21" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="21" hidden="1"/>
+    <col min="2" max="2" width="6" style="21" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" style="21" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" style="21" customWidth="1"/>
+    <col min="5" max="5" width="5.21875" style="21" customWidth="1"/>
+    <col min="6" max="6" width="9.77734375" style="21" customWidth="1"/>
+    <col min="7" max="7" width="80.88671875" style="21" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="21" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="52" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="D1" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="E1" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="F1" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="G1" s="21" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="23">
+      <c r="B2" s="29"/>
+      <c r="C2" s="23">
         <v>42992</v>
       </c>
-      <c r="C2" s="23">
+      <c r="D2" s="23">
         <v>42993</v>
       </c>
-      <c r="D2" s="24">
+      <c r="E2" s="24">
         <v>1.5</v>
       </c>
-      <c r="E2" s="23">
+      <c r="F2" s="23">
         <v>43006</v>
       </c>
-      <c r="F2" s="33" t="s">
+      <c r="G2" s="33" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="26"/>
+      <c r="C3" s="23">
         <v>42986</v>
       </c>
-      <c r="C3" s="23">
+      <c r="D3" s="23">
         <v>42999</v>
       </c>
-      <c r="D3" s="24">
+      <c r="E3" s="24">
         <v>1.5</v>
       </c>
-      <c r="E3" s="23">
+      <c r="F3" s="23">
         <v>43006</v>
       </c>
-      <c r="F3" s="33" t="s">
+      <c r="G3" s="33" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="23">
-        <v>42983</v>
-      </c>
       <c r="C4" s="23">
         <v>42983</v>
       </c>
-      <c r="D4" s="24">
-        <v>1</v>
-      </c>
-      <c r="E4" s="23">
+      <c r="D4" s="23">
+        <v>42983</v>
+      </c>
+      <c r="E4" s="24">
+        <v>1</v>
+      </c>
+      <c r="F4" s="23">
         <v>42984</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="23">
-        <v>42983</v>
-      </c>
       <c r="C5" s="23">
         <v>42983</v>
       </c>
-      <c r="D5" s="24">
-        <v>1</v>
-      </c>
-      <c r="E5" s="23">
+      <c r="D5" s="23">
+        <v>42983</v>
+      </c>
+      <c r="E5" s="24">
+        <v>1</v>
+      </c>
+      <c r="F5" s="23">
         <v>42992</v>
       </c>
-      <c r="F5" s="21" t="s">
+      <c r="G5" s="21" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="23">
-        <v>42983</v>
-      </c>
       <c r="C6" s="23">
         <v>42983</v>
       </c>
-      <c r="D6" s="24">
-        <v>1</v>
-      </c>
-      <c r="E6" s="23">
+      <c r="D6" s="23">
+        <v>42983</v>
+      </c>
+      <c r="E6" s="24">
+        <v>1</v>
+      </c>
+      <c r="F6" s="23">
         <v>42984</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="23">
+      <c r="C7" s="23">
         <v>42983</v>
       </c>
-      <c r="C7" s="23">
+      <c r="D7" s="23">
         <v>42984</v>
       </c>
-      <c r="D7" s="24">
-        <v>1</v>
-      </c>
-      <c r="E7" s="23">
+      <c r="E7" s="24">
+        <v>1</v>
+      </c>
+      <c r="F7" s="23">
         <v>42986</v>
       </c>
-      <c r="F7" s="25" t="s">
+      <c r="G7" s="25" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="23">
+      <c r="C8" s="23">
         <v>42983</v>
       </c>
-      <c r="C8" s="23">
+      <c r="D8" s="23">
         <v>42990</v>
       </c>
-      <c r="D8" s="24">
-        <v>1</v>
-      </c>
-      <c r="E8" s="23">
+      <c r="E8" s="24">
+        <v>1</v>
+      </c>
+      <c r="F8" s="23">
         <v>42990</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="23">
+      <c r="C9" s="23">
         <v>42983</v>
       </c>
-      <c r="C9" s="23">
+      <c r="D9" s="23">
         <v>42990</v>
       </c>
-      <c r="D9" s="24">
-        <v>1</v>
-      </c>
-      <c r="E9" s="23">
+      <c r="E9" s="24">
+        <v>1</v>
+      </c>
+      <c r="F9" s="23">
         <v>42991</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="G9" s="27" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="B10" s="23">
+      <c r="B10" s="30"/>
+      <c r="C10" s="23">
         <v>42990</v>
       </c>
-      <c r="C10" s="23">
+      <c r="D10" s="23">
         <v>42992</v>
       </c>
-      <c r="D10" s="24">
-        <v>1</v>
-      </c>
-      <c r="E10" s="23">
+      <c r="E10" s="24">
+        <v>1</v>
+      </c>
+      <c r="F10" s="23">
         <v>43027</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="G10" s="32" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="23">
+      <c r="C11" s="23">
         <v>42984</v>
       </c>
-      <c r="C11" s="23">
+      <c r="D11" s="23">
         <v>42992</v>
       </c>
-      <c r="D11" s="24">
-        <v>1</v>
-      </c>
-      <c r="E11" s="23">
+      <c r="E11" s="24">
+        <v>1</v>
+      </c>
+      <c r="F11" s="23">
         <v>42992</v>
       </c>
-      <c r="F11" s="26" t="s">
+      <c r="G11" s="26" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="23">
+      <c r="C12" s="23">
         <v>42983</v>
       </c>
-      <c r="C12" s="23">
+      <c r="D12" s="23">
         <v>42992</v>
       </c>
-      <c r="D12" s="24">
-        <v>1</v>
-      </c>
-      <c r="E12" s="23">
+      <c r="E12" s="24">
+        <v>1</v>
+      </c>
+      <c r="F12" s="23">
         <v>42992</v>
       </c>
-      <c r="F12" s="21" t="s">
+      <c r="G12" s="21" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="23">
+      <c r="B13" s="27"/>
+      <c r="C13" s="23">
         <v>42990</v>
       </c>
-      <c r="C13" s="23">
+      <c r="D13" s="23">
         <v>42993</v>
       </c>
-      <c r="D13" s="24">
-        <v>1</v>
-      </c>
-      <c r="E13" s="23">
+      <c r="E13" s="24">
+        <v>1</v>
+      </c>
+      <c r="F13" s="23">
         <v>43006</v>
       </c>
-      <c r="F13" s="27" t="s">
+      <c r="G13" s="27" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="B14" s="23">
-        <v>42998</v>
-      </c>
+      <c r="B14" s="31"/>
       <c r="C14" s="23">
         <v>42998</v>
       </c>
-      <c r="D14" s="24">
-        <v>1</v>
-      </c>
-      <c r="E14" s="23">
+      <c r="D14" s="23">
+        <v>42998</v>
+      </c>
+      <c r="E14" s="24">
+        <v>1</v>
+      </c>
+      <c r="F14" s="23">
         <v>43006</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="23">
+      <c r="C15" s="23">
         <v>42983</v>
       </c>
-      <c r="C15" s="23">
+      <c r="D15" s="23">
         <v>42991</v>
       </c>
-      <c r="D15" s="24">
-        <v>1</v>
-      </c>
-      <c r="E15" s="23">
+      <c r="E15" s="24">
+        <v>1</v>
+      </c>
+      <c r="F15" s="23">
         <v>42999</v>
       </c>
-      <c r="F15" s="29" t="s">
+      <c r="G15" s="29" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="23">
+      <c r="C16" s="23">
         <v>42983</v>
       </c>
-      <c r="C16" s="23">
+      <c r="D16" s="23">
         <v>42991</v>
       </c>
-      <c r="D16" s="24">
-        <v>1</v>
-      </c>
-      <c r="E16" s="23">
+      <c r="E16" s="24">
+        <v>1</v>
+      </c>
+      <c r="F16" s="23">
         <v>42999</v>
       </c>
-      <c r="F16" s="29" t="s">
+      <c r="G16" s="29" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="B17" s="23">
-        <v>43021</v>
-      </c>
+      <c r="B17" s="33"/>
       <c r="C17" s="23">
         <v>43021</v>
       </c>
-      <c r="D17" s="24">
-        <v>1</v>
-      </c>
-      <c r="E17" s="23">
+      <c r="D17" s="23">
+        <v>43021</v>
+      </c>
+      <c r="E17" s="24">
+        <v>1</v>
+      </c>
+      <c r="F17" s="23">
         <v>43027</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="23">
-        <v>43021</v>
-      </c>
+      <c r="B18" s="33"/>
       <c r="C18" s="23">
         <v>43021</v>
       </c>
-      <c r="D18" s="24">
-        <v>1</v>
-      </c>
-      <c r="E18" s="23">
+      <c r="D18" s="23">
+        <v>43021</v>
+      </c>
+      <c r="E18" s="24">
+        <v>1</v>
+      </c>
+      <c r="F18" s="23">
         <v>43027</v>
       </c>
-      <c r="F18" s="33"/>
-    </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G18" s="33"/>
+    </row>
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="B19" s="23">
+      <c r="B19" s="33"/>
+      <c r="C19" s="23">
         <v>43021</v>
       </c>
-      <c r="C19" s="23">
+      <c r="D19" s="23">
         <v>43024</v>
       </c>
-      <c r="D19" s="24">
-        <v>1</v>
-      </c>
-      <c r="E19" s="23">
+      <c r="E19" s="24">
+        <v>1</v>
+      </c>
+      <c r="F19" s="23">
         <v>43027</v>
       </c>
-      <c r="F19" s="33" t="s">
+      <c r="G19" s="33" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="B20" s="23">
+      <c r="B20" s="35"/>
+      <c r="C20" s="23">
         <v>43021</v>
       </c>
-      <c r="C20" s="23">
+      <c r="D20" s="23">
         <v>43024</v>
       </c>
-      <c r="D20" s="24">
-        <v>1</v>
-      </c>
-      <c r="E20" s="23">
+      <c r="E20" s="24">
+        <v>1</v>
+      </c>
+      <c r="F20" s="23">
         <v>43027</v>
       </c>
-      <c r="F20" s="33"/>
-    </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G20" s="33"/>
+    </row>
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="B21" s="23">
+      <c r="B21" s="35"/>
+      <c r="C21" s="23">
         <v>43021</v>
       </c>
-      <c r="C21" s="23">
+      <c r="D21" s="23">
         <v>43027</v>
       </c>
-      <c r="D21" s="24">
-        <v>1</v>
-      </c>
-      <c r="E21" s="23">
+      <c r="E21" s="24">
+        <v>1</v>
+      </c>
+      <c r="F21" s="23">
         <v>43023</v>
       </c>
-      <c r="F21" s="33"/>
-    </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G21" s="33"/>
+    </row>
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="B22" s="23">
+      <c r="B22" s="34"/>
+      <c r="C22" s="23">
         <v>43021</v>
       </c>
-      <c r="C22" s="23">
+      <c r="D22" s="23">
         <v>43027</v>
       </c>
-      <c r="D22" s="24">
-        <v>1</v>
-      </c>
-      <c r="E22" s="23">
+      <c r="E22" s="24">
+        <v>1</v>
+      </c>
+      <c r="F22" s="23">
         <v>43027</v>
       </c>
-      <c r="F22" s="34" t="s">
+      <c r="G22" s="34" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="B23" s="23">
+      <c r="B23" s="36"/>
+      <c r="C23" s="23">
         <v>43024</v>
       </c>
-      <c r="C23" s="23">
+      <c r="D23" s="23">
         <v>43025</v>
       </c>
-      <c r="D23" s="24">
-        <v>1</v>
-      </c>
-      <c r="E23" s="23">
+      <c r="E23" s="24">
+        <v>1</v>
+      </c>
+      <c r="F23" s="23">
         <v>43034</v>
       </c>
-      <c r="F23" s="37" t="s">
+      <c r="G23" s="37" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="B24" s="23">
+      <c r="B24" s="38"/>
+      <c r="C24" s="23">
         <v>43026</v>
       </c>
-      <c r="C24" s="23">
+      <c r="D24" s="23">
         <v>43027</v>
       </c>
-      <c r="D24" s="24">
-        <v>1</v>
-      </c>
-      <c r="E24" s="23">
+      <c r="E24" s="24">
+        <v>1</v>
+      </c>
+      <c r="F24" s="23">
         <v>43034</v>
       </c>
-      <c r="F24" s="39" t="s">
+      <c r="G24" s="39" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="23">
+      <c r="B25" s="36"/>
+      <c r="C25" s="23">
         <v>43024</v>
       </c>
-      <c r="C25" s="23">
+      <c r="D25" s="23">
         <v>43026</v>
       </c>
-      <c r="D25" s="24">
-        <v>1</v>
-      </c>
-      <c r="E25" s="23">
+      <c r="E25" s="24">
+        <v>1</v>
+      </c>
+      <c r="F25" s="23">
         <v>43034</v>
       </c>
-      <c r="F25" s="33"/>
-    </row>
-    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G25" s="33"/>
+    </row>
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="35" t="s">
         <v>97</v>
       </c>
-      <c r="B26" s="23">
+      <c r="B26" s="35"/>
+      <c r="C26" s="23">
         <v>43021</v>
       </c>
-      <c r="C26" s="23">
+      <c r="D26" s="23">
         <v>43024</v>
       </c>
-      <c r="D26" s="24">
-        <v>1</v>
-      </c>
-      <c r="E26" s="23">
+      <c r="E26" s="24">
+        <v>1</v>
+      </c>
+      <c r="F26" s="23">
         <v>43027</v>
       </c>
-      <c r="F26" s="33"/>
-    </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G26" s="33"/>
+    </row>
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="46" t="s">
         <v>147</v>
       </c>
-      <c r="B27" s="23">
+      <c r="B27" s="46"/>
+      <c r="C27" s="23">
         <v>43109</v>
       </c>
-      <c r="C27" s="23">
+      <c r="D27" s="23">
         <v>43118</v>
       </c>
-      <c r="D27" s="24">
-        <v>1</v>
-      </c>
-      <c r="E27" s="23">
+      <c r="E27" s="24">
+        <v>1</v>
+      </c>
+      <c r="F27" s="23">
         <v>43118</v>
       </c>
-      <c r="F27" s="33"/>
-    </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G27" s="33"/>
+    </row>
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="39" t="s">
         <v>103</v>
       </c>
-      <c r="B28" s="23">
+      <c r="B28" s="39"/>
+      <c r="C28" s="23">
         <v>43109</v>
       </c>
-      <c r="C28" s="23">
+      <c r="D28" s="23">
         <v>43118</v>
       </c>
-      <c r="D28" s="24">
-        <v>1</v>
-      </c>
-      <c r="E28" s="23">
+      <c r="E28" s="24">
+        <v>1</v>
+      </c>
+      <c r="F28" s="23">
         <v>43118</v>
       </c>
-      <c r="F28" s="33"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G28" s="33"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="B29" s="23">
+      <c r="B29" s="53"/>
+      <c r="C29" s="23">
         <v>43109</v>
       </c>
-      <c r="C29" s="23">
+      <c r="D29" s="23">
         <v>43118</v>
       </c>
-      <c r="D29" s="24">
+      <c r="E29" s="24">
         <v>0.75</v>
       </c>
-      <c r="E29" s="23">
+      <c r="F29" s="23">
         <v>43118</v>
       </c>
-      <c r="F29" s="48"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G29" s="48"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="23">
+      <c r="B30" s="22"/>
+      <c r="C30" s="23">
         <v>43109</v>
       </c>
-      <c r="C30" s="23">
+      <c r="D30" s="23">
         <v>43118</v>
       </c>
-      <c r="D30" s="24">
+      <c r="E30" s="24">
         <v>0.75</v>
       </c>
-      <c r="E30" s="23">
+      <c r="F30" s="23">
         <v>43118</v>
       </c>
-      <c r="F30" s="46" t="s">
+      <c r="G30" s="46" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="B31" s="23">
+      <c r="B31" s="26"/>
+      <c r="C31" s="23">
         <v>42986</v>
       </c>
-      <c r="C31" s="23">
+      <c r="D31" s="23">
         <v>43060</v>
       </c>
-      <c r="D31" s="24">
+      <c r="E31" s="24">
         <v>1.5</v>
       </c>
-      <c r="E31" s="23">
+      <c r="F31" s="23">
         <v>43040</v>
       </c>
-      <c r="F31" s="26" t="s">
+      <c r="G31" s="26" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="B32" s="23">
+      <c r="B32" s="54"/>
+      <c r="C32" s="23">
         <v>43109</v>
       </c>
-      <c r="C32" s="23">
+      <c r="D32" s="23">
         <v>43118</v>
       </c>
-      <c r="D32" s="24">
+      <c r="E32" s="24">
         <v>0.5</v>
       </c>
-      <c r="E32" s="23">
+      <c r="F32" s="23">
         <v>43118</v>
       </c>
-      <c r="F32" s="29" t="s">
+      <c r="G32" s="29" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="B33" s="23">
+      <c r="B33" s="22"/>
+      <c r="C33" s="23">
         <v>43109</v>
       </c>
-      <c r="C33" s="23">
+      <c r="D33" s="23">
         <v>43118</v>
       </c>
-      <c r="D33" s="24">
+      <c r="E33" s="24">
         <v>0.5</v>
       </c>
-      <c r="E33" s="23">
+      <c r="F33" s="23">
         <v>43118</v>
       </c>
-      <c r="F33" s="21" t="s">
+      <c r="G33" s="21" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="23">
+      <c r="B34" s="22"/>
+      <c r="C34" s="23">
         <v>43109</v>
       </c>
-      <c r="C34" s="23">
+      <c r="D34" s="23">
         <v>43118</v>
       </c>
-      <c r="D34" s="24">
+      <c r="E34" s="24">
         <v>0.5</v>
       </c>
-      <c r="E34" s="23">
+      <c r="F34" s="23">
         <v>43118</v>
       </c>
-      <c r="F34" s="26" t="s">
+      <c r="G34" s="26" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="B35" s="23">
+      <c r="B35" s="22"/>
+      <c r="C35" s="23">
         <v>43109</v>
       </c>
-      <c r="C35" s="23">
+      <c r="D35" s="23">
         <v>43118</v>
       </c>
-      <c r="D35" s="24">
+      <c r="E35" s="24">
         <v>0.25</v>
       </c>
-      <c r="E35" s="23">
+      <c r="F35" s="23">
         <v>43118</v>
       </c>
-      <c r="F35" s="26" t="s">
+      <c r="G35" s="26" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="B36" s="23">
+      <c r="B36" s="22"/>
+      <c r="C36" s="23">
         <v>43109</v>
       </c>
-      <c r="C36" s="23">
+      <c r="D36" s="23">
         <v>43118</v>
       </c>
-      <c r="D36" s="24">
+      <c r="E36" s="24">
         <v>0.25</v>
       </c>
-      <c r="E36" s="23">
+      <c r="F36" s="23">
         <v>43118</v>
       </c>
-      <c r="F36" s="33" t="s">
+      <c r="G36" s="33" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="B37" s="23">
+      <c r="B37" s="55"/>
+      <c r="C37" s="23">
         <v>43109</v>
       </c>
-      <c r="C37" s="23">
+      <c r="D37" s="23">
         <v>43118</v>
       </c>
-      <c r="D37" s="24">
+      <c r="E37" s="24">
         <v>0.25</v>
       </c>
-      <c r="E37" s="23">
+      <c r="F37" s="23">
         <v>43118</v>
       </c>
-      <c r="F37" s="33" t="s">
+      <c r="G37" s="33" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="B38" s="23">
+      <c r="B38" s="56"/>
+      <c r="C38" s="23">
         <v>43109</v>
       </c>
-      <c r="C38" s="23">
+      <c r="D38" s="23">
         <v>43118</v>
       </c>
-      <c r="D38" s="24">
-        <v>0</v>
-      </c>
-      <c r="E38" s="23">
+      <c r="E38" s="24">
+        <v>0</v>
+      </c>
+      <c r="F38" s="23">
         <v>43118</v>
       </c>
-      <c r="F38" s="33"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G38" s="51" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="40" t="s">
         <v>105</v>
       </c>
-      <c r="B39" s="23">
+      <c r="B39" s="56"/>
+      <c r="C39" s="23">
         <v>43109</v>
       </c>
-      <c r="C39" s="23">
+      <c r="D39" s="23">
         <v>43118</v>
       </c>
-      <c r="D39" s="24">
-        <v>0</v>
-      </c>
-      <c r="E39" s="23">
+      <c r="E39" s="24">
+        <v>0</v>
+      </c>
+      <c r="F39" s="23">
         <v>43118</v>
       </c>
-      <c r="F39" s="33"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G39" s="33"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="47" t="s">
         <v>148</v>
       </c>
-      <c r="B40" s="23">
+      <c r="B40" s="57"/>
+      <c r="C40" s="23">
         <v>43109</v>
       </c>
-      <c r="C40" s="23">
+      <c r="D40" s="23">
         <v>43118</v>
       </c>
-      <c r="D40" s="24">
+      <c r="E40" s="24">
         <v>0.25</v>
       </c>
-      <c r="E40" s="23">
+      <c r="F40" s="23">
         <v>43118</v>
       </c>
-      <c r="F40" s="33"/>
-    </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G40" s="33"/>
+    </row>
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="49" t="s">
         <v>149</v>
       </c>
-      <c r="B41" s="23">
+      <c r="B41" s="49"/>
+      <c r="C41" s="23">
         <v>43109</v>
       </c>
-      <c r="C41" s="23">
+      <c r="D41" s="23">
         <v>43118</v>
       </c>
-      <c r="D41" s="24">
-        <v>1</v>
-      </c>
-      <c r="E41" s="23">
+      <c r="E41" s="24">
+        <v>1</v>
+      </c>
+      <c r="F41" s="23">
         <v>43118</v>
       </c>
-      <c r="F41" s="33"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G41" s="33"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="49" t="s">
         <v>150</v>
       </c>
-      <c r="B42" s="23">
+      <c r="B42" s="58"/>
+      <c r="C42" s="23">
         <v>43109</v>
       </c>
-      <c r="C42" s="23">
+      <c r="D42" s="23">
         <v>43118</v>
       </c>
-      <c r="D42" s="24">
+      <c r="E42" s="24">
         <v>0.25</v>
       </c>
-      <c r="E42" s="23">
+      <c r="F42" s="23">
         <v>43118</v>
       </c>
-      <c r="F42" s="33"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="66" t="s">
+      <c r="G42" s="33"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" s="50" t="s">
         <v>151</v>
       </c>
-      <c r="B43" s="23">
+      <c r="B43" s="59"/>
+      <c r="C43" s="23">
         <f ca="1">TODAY()</f>
-        <v>43110</v>
-      </c>
-      <c r="C43" s="23">
+        <v>43112</v>
+      </c>
+      <c r="D43" s="23">
         <v>43118</v>
       </c>
-      <c r="D43" s="24">
-        <v>0</v>
-      </c>
-      <c r="E43" s="23">
+      <c r="E43" s="24">
+        <v>0</v>
+      </c>
+      <c r="F43" s="23">
         <v>43118</v>
       </c>
-      <c r="F43" s="33"/>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B44" s="23"/>
-      <c r="C44" s="23"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="23"/>
-    </row>
-    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.3"/>
-    <row r="46" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="G43" s="33"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="51" t="s">
+        <v>152</v>
+      </c>
+      <c r="B44" s="52"/>
+      <c r="C44" s="23">
+        <f ca="1">TODAY()</f>
+        <v>43112</v>
+      </c>
+      <c r="D44" s="23">
+        <v>43118</v>
+      </c>
+      <c r="E44" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="F44" s="23">
+        <v>41292</v>
+      </c>
+      <c r="G44" s="51" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" s="51" t="s">
+        <v>153</v>
+      </c>
+      <c r="B45" s="52"/>
+      <c r="C45" s="23">
+        <f ca="1">TODAY()</f>
+        <v>43112</v>
+      </c>
+      <c r="D45" s="23">
+        <v>43118</v>
+      </c>
+      <c r="E45" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="F45" s="23">
+        <v>41292</v>
+      </c>
+      <c r="G45" s="33"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="51" t="s">
+        <v>154</v>
+      </c>
+      <c r="B46" s="52">
+        <v>680</v>
+      </c>
+      <c r="C46" s="23">
+        <f t="shared" ref="C46:C47" ca="1" si="0">TODAY()</f>
+        <v>43112</v>
+      </c>
+      <c r="D46" s="23">
+        <v>43118</v>
+      </c>
+      <c r="E46" s="24">
+        <v>0.75</v>
+      </c>
+      <c r="F46" s="23">
+        <v>41292</v>
+      </c>
+      <c r="G46" s="33"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="51" t="s">
+        <v>155</v>
+      </c>
+      <c r="B47" s="52"/>
+      <c r="C47" s="23">
+        <f t="shared" ca="1" si="0"/>
+        <v>43112</v>
+      </c>
+      <c r="D47" s="23">
+        <v>43118</v>
+      </c>
+      <c r="E47" s="24">
+        <v>1</v>
+      </c>
+      <c r="F47" s="23">
+        <v>41292</v>
+      </c>
+      <c r="G47" s="33"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="77" t="s">
+        <v>159</v>
+      </c>
+      <c r="B48" s="76"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="33"/>
+    </row>
+    <row r="49" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B49" s="22"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="23"/>
+      <c r="E49" s="24"/>
+      <c r="F49" s="23"/>
+    </row>
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="51" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <conditionalFormatting sqref="D2:D44">
+  <conditionalFormatting sqref="E2:E49">
     <cfRule type="iconSet" priority="14">
       <iconSet iconSet="5Quarters" showValue="0">
         <cfvo type="percent" val="0"/>

</xml_diff>

<commit_message>
Speed-ups and multiprocessing integration
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="8649" windowHeight="8451" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="8652" windowHeight="8448" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Project Planner" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="184">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -369,9 +369,6 @@
     <t>Are Measures A and B implemented correctly in the code?</t>
   </si>
   <si>
-    <t>Check initial conditions</t>
-  </si>
-  <si>
     <t>Can we impose constraints that select for observed quantities? Shelf for now?</t>
   </si>
   <si>
@@ -552,21 +549,12 @@
     <t>Rescale the potential in instanton code</t>
   </si>
   <si>
-    <t>Check find_phistart_A</t>
-  </si>
-  <si>
     <t>Speed up non-false-vacuum code</t>
   </si>
   <si>
-    <t>Fix issue with fv code related to field scale</t>
-  </si>
-  <si>
     <t>Check for inflation on other side of barrier</t>
   </si>
   <si>
-    <t>What is flagStartAtMaximum?</t>
-  </si>
-  <si>
     <t>Scan param files in script</t>
   </si>
   <si>
@@ -576,9 +564,6 @@
     <t>Make a table of all status codes</t>
   </si>
   <si>
-    <t>Deprecated?</t>
-  </si>
-  <si>
     <t>Email Matt Johnson</t>
   </si>
   <si>
@@ -622,6 +607,57 @@
   </si>
   <si>
     <t>Get multiprocessing to work with Matlab functions</t>
+  </si>
+  <si>
+    <t>Get started with hummingbird</t>
+  </si>
+  <si>
+    <t>Learn SLURM</t>
+  </si>
+  <si>
+    <t>Allow reheating in the true vacuum</t>
+  </si>
+  <si>
+    <t>Convert to function</t>
+  </si>
+  <si>
+    <t>No speedup resulted</t>
+  </si>
+  <si>
+    <t>Allow for looking ahead to multiple true minima</t>
+  </si>
+  <si>
+    <t>Pre-compute Hawking-Moss tunneling rate</t>
+  </si>
+  <si>
+    <t>Add remaining parameters to Python script</t>
+  </si>
+  <si>
+    <t>Solve "Minimum step size reached" problem</t>
+  </si>
+  <si>
+    <t>Related to field scale?</t>
+  </si>
+  <si>
+    <t>Fix issue with false vacuum code</t>
+  </si>
+  <si>
+    <t>Does it matter after all?</t>
+  </si>
+  <si>
+    <t>Check initial conditions for measure A</t>
+  </si>
+  <si>
+    <t>Make find_phipeak always land on the starting side</t>
+  </si>
+  <si>
+    <t>Make stochastic and topological checks compatible with A</t>
+  </si>
+  <si>
+    <t>Add lower bound on potential for initiating FV check</t>
+  </si>
+  <si>
+    <t>Make find_next_minimum also return phipeak</t>
   </si>
 </sst>
 </file>
@@ -632,13 +668,27 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="46" x14ac:knownFonts="1">
+  <fonts count="48" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1099,98 +1149,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="41" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="43" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="34" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="44" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="46" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="44" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="44" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="44" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="44" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="44" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="41" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="43" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="34" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="36" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="42" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="37" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="39" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="44" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="46" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -1208,25 +1258,27 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="43" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="41" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="43" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="31" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="33" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -1241,58 +1293,61 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="18" fontId="24" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="18" fontId="22" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1303,34 +1358,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -1346,6 +1401,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="20">
     <cellStyle name="% complete" xfId="16"/>
@@ -1370,6 +1428,148 @@
     <cellStyle name="Title" xfId="8" builtinId="15" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="31">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="9" tint="-0.24994659260841701"/>
+        </left>
+        <right style="thin">
+          <color theme="9" tint="-0.24994659260841701"/>
+        </right>
+        <bottom style="thin">
+          <color theme="7"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color theme="7"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="9" tint="-0.24994659260841701"/>
+        </left>
+        <right style="thin">
+          <color theme="9" tint="-0.24994659260841701"/>
+        </right>
+        <bottom style="thin">
+          <color theme="9" tint="0.59996337778862885"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor theme="7"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor theme="7"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor theme="7"/>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1719,148 +1919,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="9" tint="-0.24994659260841701"/>
-        </left>
-        <right style="thin">
-          <color theme="9" tint="-0.24994659260841701"/>
-        </right>
-        <bottom style="thin">
-          <color theme="7"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="7"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="9" tint="-0.24994659260841701"/>
-        </left>
-        <right style="thin">
-          <color theme="9" tint="-0.24994659260841701"/>
-        </right>
-        <bottom style="thin">
-          <color theme="9" tint="0.59996337778862885"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp">
-          <fgColor theme="7"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp">
-          <fgColor theme="7"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp">
-          <fgColor theme="7"/>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1880,8 +1938,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F73" totalsRowShown="0">
-  <autoFilter ref="A1:F73">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F81" totalsRowShown="0">
+  <autoFilter ref="A1:F81">
     <filterColumn colId="3">
       <filters blank="1">
         <filter val="0"/>
@@ -1891,14 +1949,14 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState ref="A27:F73">
-    <sortCondition descending="1" ref="D1:D73"/>
+  <sortState ref="A30:F81">
+    <sortCondition descending="1" ref="C1:C81"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" name="Task"/>
     <tableColumn id="2" name="Assigned"/>
     <tableColumn id="3" name="Due"/>
-    <tableColumn id="6" name=" " dataDxfId="20"/>
+    <tableColumn id="6" name=" " dataDxfId="30"/>
     <tableColumn id="4" name="Review"/>
     <tableColumn id="5" name="Notes"/>
   </tableColumns>
@@ -1907,26 +1965,26 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:Q33" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:Q33" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
   <autoFilter ref="A1:Q33"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="Test ID" dataDxfId="17"/>
-    <tableColumn id="2" name="log10(mv)" dataDxfId="16"/>
-    <tableColumn id="3" name="mh" dataDxfId="15"/>
-    <tableColumn id="4" name="log10(n_iter)" dataDxfId="14"/>
-    <tableColumn id="5" name="lambda_screen" dataDxfId="13"/>
-    <tableColumn id="6" name="fix_Lambda" dataDxfId="12"/>
-    <tableColumn id="7" name="fix_Q" dataDxfId="11"/>
-    <tableColumn id="8" name="measure" dataDxfId="10"/>
-    <tableColumn id="9" name="n_tunnel_max" dataDxfId="9"/>
-    <tableColumn id="10" name="End Date" dataDxfId="8"/>
-    <tableColumn id="11" name="Runtime" dataDxfId="7"/>
-    <tableColumn id="12" name="File name" dataDxfId="6"/>
-    <tableColumn id="13" name="Column13" dataDxfId="5"/>
-    <tableColumn id="14" name="Column14" dataDxfId="4"/>
-    <tableColumn id="15" name="Column15" dataDxfId="3"/>
-    <tableColumn id="16" name="Column16" dataDxfId="2"/>
-    <tableColumn id="17" name="Column17" dataDxfId="1"/>
+    <tableColumn id="1" name="Test ID" dataDxfId="27"/>
+    <tableColumn id="2" name="log10(mv)" dataDxfId="26"/>
+    <tableColumn id="3" name="mh" dataDxfId="25"/>
+    <tableColumn id="4" name="log10(n_iter)" dataDxfId="24"/>
+    <tableColumn id="5" name="lambda_screen" dataDxfId="23"/>
+    <tableColumn id="6" name="fix_Lambda" dataDxfId="22"/>
+    <tableColumn id="7" name="fix_Q" dataDxfId="21"/>
+    <tableColumn id="8" name="measure" dataDxfId="20"/>
+    <tableColumn id="9" name="n_tunnel_max" dataDxfId="19"/>
+    <tableColumn id="10" name="End Date" dataDxfId="18"/>
+    <tableColumn id="11" name="Runtime" dataDxfId="17"/>
+    <tableColumn id="12" name="File name" dataDxfId="16"/>
+    <tableColumn id="13" name="Column13" dataDxfId="15"/>
+    <tableColumn id="14" name="Column14" dataDxfId="14"/>
+    <tableColumn id="15" name="Column15" dataDxfId="13"/>
+    <tableColumn id="16" name="Column16" dataDxfId="12"/>
+    <tableColumn id="17" name="Column17" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1939,7 +1997,7 @@
     <tableColumn id="1" name="Quantity"/>
     <tableColumn id="2" name="Dimensions"/>
     <tableColumn id="3" name="Units"/>
-    <tableColumn id="4" name="Description" dataDxfId="0"/>
+    <tableColumn id="4" name="Description" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2177,19 +2235,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BO31"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.640625" customWidth="1"/>
-    <col min="2" max="2" width="15.640625" style="2" customWidth="1"/>
-    <col min="3" max="6" width="11.640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.640625" style="4" customWidth="1"/>
-    <col min="8" max="27" width="3.5703125" style="1" customWidth="1"/>
-    <col min="28" max="48" width="3.5703125" customWidth="1"/>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="2" customWidth="1"/>
+    <col min="3" max="6" width="11.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="4" customWidth="1"/>
+    <col min="8" max="27" width="3.5546875" style="1" customWidth="1"/>
+    <col min="28" max="48" width="3.5546875" customWidth="1"/>
     <col min="49" max="67" width="0" hidden="1" customWidth="1"/>
-    <col min="68" max="16384" width="2.78515625" hidden="1"/>
+    <col min="68" max="16384" width="2.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.4">
+    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.05">
       <c r="B1" s="11" t="s">
         <v>40</v>
       </c>
@@ -2199,14 +2257,14 @@
       <c r="F1" s="10"/>
       <c r="G1" s="10"/>
     </row>
-    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="69" t="s">
+    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="72" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
@@ -2214,66 +2272,66 @@
         <v>8</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="75" t="s">
+      <c r="K2" s="78" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="76"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="76"/>
-      <c r="O2" s="77"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="79"/>
+      <c r="O2" s="80"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="75" t="s">
+      <c r="Q2" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="78"/>
-      <c r="S2" s="78"/>
-      <c r="T2" s="77"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="80"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="67" t="s">
+      <c r="V2" s="70" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="68"/>
-      <c r="X2" s="68"/>
-      <c r="Y2" s="79"/>
+      <c r="W2" s="71"/>
+      <c r="X2" s="71"/>
+      <c r="Y2" s="82"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="80" t="s">
+      <c r="AA2" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="81"/>
-      <c r="AC2" s="81"/>
-      <c r="AD2" s="81"/>
-      <c r="AE2" s="81"/>
-      <c r="AF2" s="81"/>
-      <c r="AG2" s="82"/>
+      <c r="AB2" s="84"/>
+      <c r="AC2" s="84"/>
+      <c r="AD2" s="84"/>
+      <c r="AE2" s="84"/>
+      <c r="AF2" s="84"/>
+      <c r="AG2" s="85"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="67" t="s">
+      <c r="AI2" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="68"/>
-      <c r="AK2" s="68"/>
-      <c r="AL2" s="68"/>
-      <c r="AM2" s="68"/>
-      <c r="AN2" s="68"/>
-      <c r="AO2" s="68"/>
-      <c r="AP2" s="68"/>
-    </row>
-    <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="70" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="72" t="s">
+      <c r="AJ2" s="71"/>
+      <c r="AK2" s="71"/>
+      <c r="AL2" s="71"/>
+      <c r="AM2" s="71"/>
+      <c r="AN2" s="71"/>
+      <c r="AO2" s="71"/>
+      <c r="AP2" s="71"/>
+    </row>
+    <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="73" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="75" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="72" t="s">
+      <c r="D3" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="72" t="s">
+      <c r="E3" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="72" t="s">
+      <c r="F3" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="74" t="s">
+      <c r="G3" s="77" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -2401,13 +2459,13 @@
       </c>
       <c r="AW3" s="18"/>
     </row>
-    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="71"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
+    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="74"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -2551,7 +2609,7 @@
       <c r="BN4" s="3"/>
       <c r="BO4" s="3"/>
     </row>
-    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6" t="s">
         <v>38</v>
       </c>
@@ -2574,7 +2632,7 @@
       <c r="X5" s="19"/>
       <c r="Y5" s="19"/>
     </row>
-    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>35</v>
       </c>
@@ -2597,7 +2655,7 @@
       <c r="X6" s="19"/>
       <c r="Y6" s="19"/>
     </row>
-    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6" t="s">
         <v>29</v>
       </c>
@@ -2620,7 +2678,7 @@
       <c r="X7" s="19"/>
       <c r="Y7" s="19"/>
     </row>
-    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>32</v>
       </c>
@@ -2641,7 +2699,7 @@
       <c r="X8" s="19"/>
       <c r="Y8" s="19"/>
     </row>
-    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="6" t="s">
         <v>33</v>
       </c>
@@ -2662,7 +2720,7 @@
       <c r="X9" s="19"/>
       <c r="Y9" s="19"/>
     </row>
-    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="6" t="s">
         <v>34</v>
       </c>
@@ -2683,7 +2741,7 @@
       <c r="X10" s="19"/>
       <c r="Y10" s="19"/>
     </row>
-    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="6" t="s">
         <v>39</v>
       </c>
@@ -2704,7 +2762,7 @@
       <c r="X11" s="19"/>
       <c r="Y11" s="19"/>
     </row>
-    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
@@ -2727,7 +2785,7 @@
       <c r="X12" s="19"/>
       <c r="Y12" s="19"/>
     </row>
-    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="6" t="s">
         <v>31</v>
       </c>
@@ -2748,7 +2806,7 @@
       <c r="X13" s="19"/>
       <c r="Y13" s="19"/>
     </row>
-    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>36</v>
       </c>
@@ -2769,7 +2827,7 @@
       <c r="X14" s="19"/>
       <c r="Y14" s="19"/>
     </row>
-    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="6" t="s">
         <v>37</v>
       </c>
@@ -2790,7 +2848,7 @@
       <c r="X15" s="19"/>
       <c r="Y15" s="19"/>
     </row>
-    <row r="16" spans="2:67" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:67" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="6" t="s">
         <v>1</v>
       </c>
@@ -2810,7 +2868,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="6" t="s">
         <v>2</v>
       </c>
@@ -2830,7 +2888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="6" t="s">
         <v>3</v>
       </c>
@@ -2850,7 +2908,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="6" t="s">
         <v>4</v>
       </c>
@@ -2870,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="6" t="s">
         <v>5</v>
       </c>
@@ -2890,7 +2948,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="6" t="s">
         <v>6</v>
       </c>
@@ -2910,7 +2968,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="6" t="s">
         <v>7</v>
       </c>
@@ -2930,7 +2988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="6" t="s">
         <v>8</v>
       </c>
@@ -2950,7 +3008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="6" t="s">
         <v>9</v>
       </c>
@@ -2970,7 +3028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="6" t="s">
         <v>10</v>
       </c>
@@ -2990,7 +3048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="6" t="s">
         <v>11</v>
       </c>
@@ -3010,7 +3068,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="6" t="s">
         <v>12</v>
       </c>
@@ -3030,7 +3088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="6" t="s">
         <v>13</v>
       </c>
@@ -3050,7 +3108,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="6" t="s">
         <v>14</v>
       </c>
@@ -3070,7 +3128,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="6" t="s">
         <v>15</v>
       </c>
@@ -3090,7 +3148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="6" t="s">
         <v>16</v>
       </c>
@@ -3126,38 +3184,38 @@
     <mergeCell ref="AA2:AG2"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:BO31">
-    <cfRule type="expression" dxfId="30" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>PercentComplete</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="3">
+    <cfRule type="expression" dxfId="8" priority="3">
       <formula>PercentCompleteBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="4">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>Actual</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>ActualBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>Plan</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="7">
+    <cfRule type="expression" dxfId="4" priority="7">
       <formula>H$4=period_selected</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="11">
+    <cfRule type="expression" dxfId="3" priority="11">
       <formula>MOD(COLUMN(),2)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="12">
+    <cfRule type="expression" dxfId="2" priority="12">
       <formula>MOD(COLUMN(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:BO32">
-    <cfRule type="expression" dxfId="22" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:BO4">
-    <cfRule type="expression" dxfId="21" priority="8">
+    <cfRule type="expression" dxfId="0" priority="8">
       <formula>H$4=period_selected</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3192,20 +3250,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G75"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:G85"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="51.2109375" style="21" customWidth="1"/>
-    <col min="2" max="2" width="9.78515625" style="21" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" style="21" customWidth="1"/>
-    <col min="4" max="4" width="5.2109375" style="21" customWidth="1"/>
-    <col min="5" max="5" width="9.78515625" style="21" customWidth="1"/>
-    <col min="6" max="6" width="80.85546875" style="21" customWidth="1"/>
+    <col min="1" max="1" width="51.21875" style="21" customWidth="1"/>
+    <col min="2" max="2" width="9.77734375" style="21" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" style="21" customWidth="1"/>
+    <col min="4" max="4" width="5.21875" style="21" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" style="21" customWidth="1"/>
+    <col min="6" max="6" width="80.88671875" style="21" customWidth="1"/>
     <col min="7" max="7" width="0" style="21" hidden="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.85546875" style="21" hidden="1"/>
+    <col min="8" max="16384" width="8.88671875" style="21" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
         <v>41</v>
       </c>
@@ -3225,7 +3283,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>80</v>
       </c>
@@ -3245,7 +3303,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
         <v>66</v>
       </c>
@@ -3262,10 +3320,10 @@
         <v>43006</v>
       </c>
       <c r="F3" s="33" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>47</v>
       </c>
@@ -3282,7 +3340,7 @@
         <v>42984</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
         <v>48</v>
       </c>
@@ -3302,7 +3360,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
         <v>50</v>
       </c>
@@ -3319,7 +3377,7 @@
         <v>42984</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
         <v>52</v>
       </c>
@@ -3339,7 +3397,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="21" t="s">
         <v>51</v>
       </c>
@@ -3356,7 +3414,7 @@
         <v>42990</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
         <v>55</v>
       </c>
@@ -3376,7 +3434,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
         <v>81</v>
       </c>
@@ -3396,7 +3454,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
         <v>60</v>
       </c>
@@ -3416,7 +3474,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
         <v>56</v>
       </c>
@@ -3436,7 +3494,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="27" t="s">
         <v>73</v>
       </c>
@@ -3456,7 +3514,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="31" t="s">
         <v>82</v>
       </c>
@@ -3473,7 +3531,7 @@
         <v>43006</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
         <v>53</v>
       </c>
@@ -3493,7 +3551,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>54</v>
       </c>
@@ -3513,7 +3571,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
         <v>84</v>
       </c>
@@ -3530,9 +3588,9 @@
         <v>43027</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B18" s="23">
         <v>43021</v>
@@ -3548,9 +3606,9 @@
       </c>
       <c r="F18" s="33"/>
     </row>
-    <row r="19" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B19" s="23">
         <v>43021</v>
@@ -3565,12 +3623,12 @@
         <v>43027</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B20" s="23">
         <v>43021</v>
@@ -3586,9 +3644,9 @@
       </c>
       <c r="F20" s="33"/>
     </row>
-    <row r="21" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="35" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B21" s="23">
         <v>43021</v>
@@ -3604,9 +3662,9 @@
       </c>
       <c r="F21" s="33"/>
     </row>
-    <row r="22" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="34" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B22" s="23">
         <v>43021</v>
@@ -3621,12 +3679,12 @@
         <v>43027</v>
       </c>
       <c r="F22" s="34" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B23" s="23">
         <v>43024</v>
@@ -3641,12 +3699,12 @@
         <v>43034</v>
       </c>
       <c r="F23" s="37" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="38" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="38" t="s">
-        <v>101</v>
       </c>
       <c r="B24" s="23">
         <v>43026</v>
@@ -3661,12 +3719,12 @@
         <v>43034</v>
       </c>
       <c r="F24" s="39" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B25" s="23">
         <v>43024</v>
@@ -3682,9 +3740,9 @@
       </c>
       <c r="F25" s="33"/>
     </row>
-    <row r="26" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="35" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B26" s="23">
         <v>43021</v>
@@ -3700,9 +3758,9 @@
       </c>
       <c r="F26" s="33"/>
     </row>
-    <row r="27" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="46" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B27" s="23">
         <v>43109</v>
@@ -3718,9 +3776,9 @@
       </c>
       <c r="F27" s="33"/>
     </row>
-    <row r="28" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="39" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B28" s="23">
         <v>43109</v>
@@ -3736,7 +3794,7 @@
       </c>
       <c r="F28" s="33"/>
     </row>
-    <row r="29" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="28" t="s">
         <v>75</v>
       </c>
@@ -3747,34 +3805,34 @@
         <v>43118</v>
       </c>
       <c r="D29" s="24">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="E29" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F29" s="57"/>
-    </row>
-    <row r="30" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+        <v>43125</v>
+      </c>
+      <c r="F29" s="56"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="21" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B30" s="23">
-        <v>43109</v>
+        <v>43124</v>
       </c>
       <c r="C30" s="23">
-        <v>43118</v>
+        <v>43130</v>
       </c>
       <c r="D30" s="24">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="E30" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F30" s="58" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+        <v>43132</v>
+      </c>
+      <c r="F30" s="59" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="26" t="s">
         <v>67</v>
       </c>
@@ -3794,7 +3852,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="29" t="s">
         <v>77</v>
       </c>
@@ -3805,118 +3863,112 @@
         <v>43118</v>
       </c>
       <c r="D32" s="24">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E32" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F32" s="59" t="s">
+        <v>43125</v>
+      </c>
+      <c r="F32" s="58" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="21" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B33" s="23">
-        <v>43109</v>
+        <v>43124</v>
       </c>
       <c r="C33" s="23">
-        <v>43118</v>
+        <v>43130</v>
       </c>
       <c r="D33" s="24">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="E33" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F33" s="60" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A34" s="21" t="s">
-        <v>59</v>
+        <v>43132</v>
+      </c>
+      <c r="F33" s="57" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="67" t="s">
+        <v>168</v>
       </c>
       <c r="B34" s="23">
-        <v>43109</v>
+        <v>43119</v>
       </c>
       <c r="C34" s="23">
-        <v>43118</v>
+        <v>43126</v>
       </c>
       <c r="D34" s="24">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="E34" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F34" s="61" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+        <v>43125</v>
+      </c>
+      <c r="F34" s="61"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="21" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B35" s="23">
-        <v>43109</v>
+        <v>43124</v>
       </c>
       <c r="C35" s="23">
-        <v>43118</v>
+        <v>43126</v>
       </c>
       <c r="D35" s="24">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="E35" s="23">
-        <v>43118</v>
+        <v>43125</v>
       </c>
       <c r="F35" s="61" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A36" s="21" t="s">
-        <v>61</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="86" t="s">
+        <v>182</v>
       </c>
       <c r="B36" s="23">
-        <v>43109</v>
+        <v>43124</v>
       </c>
       <c r="C36" s="23">
-        <v>43118</v>
+        <v>43125</v>
       </c>
       <c r="D36" s="24">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E36" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F36" s="62" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A37" s="33" t="s">
-        <v>87</v>
+        <v>43125</v>
+      </c>
+      <c r="F36" s="61"/>
+    </row>
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="86" t="s">
+        <v>175</v>
       </c>
       <c r="B37" s="23">
-        <v>43109</v>
+        <v>43124</v>
       </c>
       <c r="C37" s="23">
-        <v>43118</v>
+        <v>43124</v>
       </c>
       <c r="D37" s="24">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E37" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F37" s="62" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+        <v>43125</v>
+      </c>
+      <c r="F37" s="61"/>
+    </row>
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="40" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B38" s="23">
         <v>43109</v>
@@ -3925,36 +3977,38 @@
         <v>43118</v>
       </c>
       <c r="D38" s="24">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E38" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F38" s="63" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A39" s="40" t="s">
-        <v>105</v>
+        <v>43125</v>
+      </c>
+      <c r="F38" s="62" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="86" t="s">
+        <v>177</v>
       </c>
       <c r="B39" s="23">
-        <v>43109</v>
+        <v>43124</v>
       </c>
       <c r="C39" s="23">
-        <v>43118</v>
+        <v>43125</v>
       </c>
       <c r="D39" s="24">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E39" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F39" s="62"/>
-    </row>
-    <row r="40" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+        <v>43125</v>
+      </c>
+      <c r="F39" s="87" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="47" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B40" s="23">
         <v>43109</v>
@@ -3963,115 +4017,114 @@
         <v>43118</v>
       </c>
       <c r="D40" s="24">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E40" s="23">
         <v>43118</v>
       </c>
-      <c r="F40" s="62"/>
-    </row>
-    <row r="41" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="48" t="s">
-        <v>149</v>
+      <c r="F40" s="33"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="40" t="s">
+        <v>104</v>
       </c>
       <c r="B41" s="23">
-        <v>43109</v>
+        <v>43124</v>
       </c>
       <c r="C41" s="23">
-        <v>43118</v>
+        <v>43124</v>
       </c>
       <c r="D41" s="24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E41" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F41" s="33"/>
-    </row>
-    <row r="42" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+        <v>43125</v>
+      </c>
+      <c r="F41" s="87" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="48" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B42" s="23">
-        <v>43109</v>
+        <f ca="1">TODAY()</f>
+        <v>43124</v>
       </c>
       <c r="C42" s="23">
         <v>43118</v>
       </c>
       <c r="D42" s="24">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E42" s="23">
         <v>43118</v>
       </c>
-      <c r="F42" s="62"/>
-    </row>
-    <row r="43" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="49" t="s">
-        <v>151</v>
+      <c r="F42" s="33"/>
+    </row>
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="69" t="s">
+        <v>174</v>
       </c>
       <c r="B43" s="23">
+        <v>43122</v>
+      </c>
+      <c r="C43" s="23">
+        <v>43122</v>
+      </c>
+      <c r="D43" s="24">
+        <v>1</v>
+      </c>
+      <c r="E43" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F43" s="61"/>
+    </row>
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="49" t="s">
+        <v>150</v>
+      </c>
+      <c r="B44" s="23">
         <f ca="1">TODAY()</f>
-        <v>43117</v>
-      </c>
-      <c r="C43" s="23">
-        <v>43118</v>
-      </c>
-      <c r="D43" s="24">
-        <v>1</v>
-      </c>
-      <c r="E43" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F43" s="33"/>
-    </row>
-    <row r="44" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A44" s="50" t="s">
-        <v>152</v>
-      </c>
-      <c r="B44" s="23">
-        <v>43112</v>
+        <v>43124</v>
       </c>
       <c r="C44" s="23">
         <v>43118</v>
       </c>
       <c r="D44" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E44" s="23">
         <v>43118</v>
       </c>
-      <c r="F44" s="63" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A45" s="50" t="s">
-        <v>153</v>
+      <c r="F44" s="33"/>
+    </row>
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="49" t="s">
+        <v>151</v>
       </c>
       <c r="B45" s="23">
-        <v>43112</v>
+        <f ca="1">TODAY()</f>
+        <v>43124</v>
       </c>
       <c r="C45" s="23">
         <v>43118</v>
       </c>
       <c r="D45" s="24">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E45" s="23">
         <v>43118</v>
       </c>
-      <c r="F45" s="65" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="F45" s="33"/>
+    </row>
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="50" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B46" s="23">
-        <f t="shared" ref="B46:B47" ca="1" si="0">TODAY()</f>
-        <v>43117</v>
+        <v>43112</v>
       </c>
       <c r="C46" s="23">
         <v>43118</v>
@@ -4080,21 +4133,19 @@
         <v>1</v>
       </c>
       <c r="E46" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F46" s="33"/>
-    </row>
-    <row r="47" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+        <v>43125</v>
+      </c>
+      <c r="F46" s="61"/>
+    </row>
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="50" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B47" s="23">
-        <f t="shared" ca="1" si="0"/>
-        <v>43117</v>
-      </c>
-      <c r="C47" s="23">
-        <v>43118</v>
-      </c>
+        <f ca="1">TODAY()</f>
+        <v>43124</v>
+      </c>
+      <c r="C47" s="23"/>
       <c r="D47" s="24">
         <v>1</v>
       </c>
@@ -4103,33 +4154,30 @@
       </c>
       <c r="F47" s="33"/>
     </row>
-    <row r="48" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A48" s="51" t="s">
-        <v>158</v>
-      </c>
-      <c r="B48" s="23">
-        <v>43112</v>
-      </c>
-      <c r="C48" s="23">
-        <v>43118</v>
-      </c>
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="50" t="s">
+        <v>155</v>
+      </c>
+      <c r="B48" s="23"/>
+      <c r="C48" s="23"/>
       <c r="D48" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E48" s="23">
         <v>43118</v>
       </c>
-      <c r="F48" s="62"/>
-    </row>
-    <row r="49" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="F48" s="33"/>
+    </row>
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="51" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B49" s="23">
-        <f ca="1">TODAY()</f>
-        <v>43117</v>
-      </c>
-      <c r="C49" s="23"/>
+        <v>43112</v>
+      </c>
+      <c r="C49" s="23">
+        <v>43118</v>
+      </c>
       <c r="D49" s="24">
         <v>1</v>
       </c>
@@ -4138,26 +4186,32 @@
       </c>
       <c r="F49" s="33"/>
     </row>
-    <row r="50" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A50" s="51" t="s">
-        <v>160</v>
-      </c>
-      <c r="B50" s="23"/>
-      <c r="C50" s="23"/>
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="52" t="s">
+        <v>157</v>
+      </c>
+      <c r="B50" s="23">
+        <v>43115</v>
+      </c>
+      <c r="C50" s="23">
+        <v>43117</v>
+      </c>
       <c r="D50" s="24">
         <v>1</v>
       </c>
       <c r="E50" s="23">
         <v>43118</v>
       </c>
-      <c r="F50" s="33"/>
-    </row>
-    <row r="51" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A51" s="52" t="s">
-        <v>161</v>
+      <c r="F50" s="63">
+        <v>0.60416666666666663</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="53" t="s">
+        <v>158</v>
       </c>
       <c r="B51" s="23">
-        <v>43112</v>
+        <v>43115</v>
       </c>
       <c r="C51" s="23">
         <v>43118</v>
@@ -4168,49 +4222,43 @@
       <c r="E51" s="23">
         <v>43118</v>
       </c>
-      <c r="F51" s="33"/>
-    </row>
-    <row r="52" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="F51" s="61"/>
+    </row>
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="53" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B52" s="23">
-        <v>43115</v>
+        <v>43116</v>
       </c>
       <c r="C52" s="23">
-        <v>43117</v>
+        <v>43116</v>
       </c>
       <c r="D52" s="24">
-        <v>0</v>
-      </c>
-      <c r="E52" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F52" s="64">
-        <v>0.60416666666666663</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+        <v>1</v>
+      </c>
+      <c r="E52" s="23"/>
+      <c r="F52" s="33"/>
+    </row>
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="54" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B53" s="23">
-        <v>43115</v>
+        <v>43116</v>
       </c>
       <c r="C53" s="23">
-        <v>43118</v>
+        <v>43116</v>
       </c>
       <c r="D53" s="24">
-        <v>0</v>
-      </c>
-      <c r="E53" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F53" s="62"/>
-    </row>
-    <row r="54" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+        <v>1</v>
+      </c>
+      <c r="E53" s="23"/>
+      <c r="F53" s="33"/>
+    </row>
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="54" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B54" s="23">
         <v>43116</v>
@@ -4224,218 +4272,397 @@
       <c r="E54" s="23"/>
       <c r="F54" s="33"/>
     </row>
-    <row r="55" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="55" t="s">
+        <v>162</v>
+      </c>
+      <c r="B55" s="23">
+        <v>43117</v>
+      </c>
+      <c r="C55" s="23">
+        <v>43117</v>
+      </c>
+      <c r="D55" s="24">
+        <v>1</v>
+      </c>
+      <c r="E55" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F55" s="61"/>
+    </row>
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="B56" s="23">
+        <v>43117</v>
+      </c>
+      <c r="C56" s="23">
+        <v>43118</v>
+      </c>
+      <c r="D56" s="24">
+        <v>1</v>
+      </c>
+      <c r="E56" s="23">
+        <v>43118</v>
+      </c>
+      <c r="F56" s="61"/>
+    </row>
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="65" t="s">
         <v>165</v>
-      </c>
-      <c r="B55" s="23">
-        <v>43116</v>
-      </c>
-      <c r="C55" s="23">
-        <v>43116</v>
-      </c>
-      <c r="D55" s="24">
-        <v>1</v>
-      </c>
-      <c r="E55" s="23"/>
-      <c r="F55" s="33"/>
-    </row>
-    <row r="56" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A56" s="55" t="s">
-        <v>166</v>
-      </c>
-      <c r="B56" s="23">
-        <v>43116</v>
-      </c>
-      <c r="C56" s="23">
-        <v>43116</v>
-      </c>
-      <c r="D56" s="24">
-        <v>1</v>
-      </c>
-      <c r="E56" s="23"/>
-      <c r="F56" s="33"/>
-    </row>
-    <row r="57" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A57" s="56" t="s">
-        <v>167</v>
       </c>
       <c r="B57" s="23">
         <v>43117</v>
       </c>
       <c r="C57" s="23">
-        <v>43117</v>
+        <v>43118</v>
       </c>
       <c r="D57" s="24">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E57" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F57" s="62"/>
-    </row>
-    <row r="58" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A58" s="56" t="s">
-        <v>168</v>
+        <v>43125</v>
+      </c>
+      <c r="F57" s="61"/>
+    </row>
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="66" t="s">
+        <v>166</v>
       </c>
       <c r="B58" s="23">
         <v>43117</v>
       </c>
       <c r="C58" s="23">
-        <v>43118</v>
+        <v>43117</v>
       </c>
       <c r="D58" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E58" s="23">
         <v>43118</v>
       </c>
-      <c r="F58" s="62"/>
-    </row>
-    <row r="59" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A59" s="66" t="s">
+      <c r="F58" s="61"/>
+    </row>
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="67" t="s">
+        <v>167</v>
+      </c>
+      <c r="B59" s="23">
+        <v>43119</v>
+      </c>
+      <c r="C59" s="23">
+        <v>43122</v>
+      </c>
+      <c r="D59" s="24">
+        <v>1</v>
+      </c>
+      <c r="E59" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F59" s="61"/>
+    </row>
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B60" s="23">
+        <v>43109</v>
+      </c>
+      <c r="C60" s="23">
+        <v>43118</v>
+      </c>
+      <c r="D60" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="E60" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F60" s="60" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="68" t="s">
+        <v>169</v>
+      </c>
+      <c r="B61" s="23">
+        <v>43119</v>
+      </c>
+      <c r="C61" s="23">
+        <v>43122</v>
+      </c>
+      <c r="D61" s="24">
+        <v>1</v>
+      </c>
+      <c r="E61" s="23">
+        <v>43125</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="67" t="s">
         <v>170</v>
       </c>
-      <c r="B59" s="23">
-        <v>43117</v>
-      </c>
-      <c r="C59" s="23">
+      <c r="B62" s="23">
+        <v>43119</v>
+      </c>
+      <c r="C62" s="23">
+        <v>43119</v>
+      </c>
+      <c r="D62" s="24">
+        <v>1</v>
+      </c>
+      <c r="E62" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F62" s="68" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="69" t="s">
+        <v>172</v>
+      </c>
+      <c r="B63" s="23">
+        <v>43122</v>
+      </c>
+      <c r="C63" s="23">
+        <v>43122</v>
+      </c>
+      <c r="D63" s="24">
+        <v>1</v>
+      </c>
+      <c r="E63" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F63" s="61"/>
+    </row>
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B64" s="23">
+        <v>43109</v>
+      </c>
+      <c r="C64" s="23">
         <v>43118</v>
       </c>
-      <c r="D59" s="24">
-        <v>0.5</v>
-      </c>
-      <c r="E59" s="23">
+      <c r="D64" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="E64" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F64" s="60" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="86" t="s">
+        <v>181</v>
+      </c>
+      <c r="B65" s="23">
+        <v>43124</v>
+      </c>
+      <c r="C65" s="23">
+        <v>43124</v>
+      </c>
+      <c r="D65" s="24">
+        <v>0</v>
+      </c>
+      <c r="E65" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F65" s="61"/>
+    </row>
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="49" t="s">
+        <v>149</v>
+      </c>
+      <c r="B66" s="23">
+        <v>43112</v>
+      </c>
+      <c r="C66" s="23">
         <v>43118</v>
       </c>
-      <c r="F59" s="62"/>
-    </row>
-    <row r="60" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A60" s="83" t="s">
-        <v>171</v>
-      </c>
-      <c r="B60" s="23">
-        <v>43117</v>
-      </c>
-      <c r="C60" s="23">
-        <v>43117</v>
-      </c>
-      <c r="D60" s="24">
-        <v>1</v>
-      </c>
-      <c r="E60" s="23">
-        <v>43118</v>
-      </c>
-      <c r="F60" s="62"/>
-    </row>
-    <row r="61" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A61" s="51"/>
-      <c r="B61" s="23"/>
-      <c r="C61" s="23"/>
-      <c r="D61" s="24"/>
-      <c r="E61" s="23"/>
-      <c r="F61" s="62"/>
-    </row>
-    <row r="62" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A62" s="51"/>
-      <c r="B62" s="23"/>
-      <c r="C62" s="23"/>
-      <c r="D62" s="24"/>
-      <c r="E62" s="23"/>
-      <c r="F62" s="62"/>
-    </row>
-    <row r="63" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A63" s="51"/>
-      <c r="B63" s="23"/>
-      <c r="C63" s="23"/>
-      <c r="D63" s="24"/>
-      <c r="E63" s="23"/>
-      <c r="F63" s="62"/>
-    </row>
-    <row r="64" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A64" s="51"/>
-      <c r="B64" s="23"/>
-      <c r="C64" s="23"/>
-      <c r="D64" s="24"/>
-      <c r="E64" s="23"/>
-      <c r="F64" s="62"/>
-    </row>
-    <row r="65" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A65" s="51"/>
-      <c r="B65" s="23"/>
-      <c r="C65" s="23"/>
-      <c r="D65" s="24"/>
-      <c r="E65" s="23"/>
-      <c r="F65" s="62"/>
-    </row>
-    <row r="66" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A66" s="51"/>
-      <c r="B66" s="23"/>
-      <c r="C66" s="23"/>
-      <c r="D66" s="24"/>
-      <c r="E66" s="23"/>
-      <c r="F66" s="62"/>
-    </row>
-    <row r="67" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A67" s="51"/>
-      <c r="B67" s="23"/>
-      <c r="C67" s="23"/>
-      <c r="D67" s="24"/>
-      <c r="E67" s="23"/>
-      <c r="F67" s="62"/>
-    </row>
-    <row r="68" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A68" s="51"/>
-      <c r="B68" s="23"/>
-      <c r="C68" s="23"/>
-      <c r="D68" s="24"/>
-      <c r="E68" s="23"/>
-      <c r="F68" s="62"/>
-    </row>
-    <row r="69" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A69" s="51"/>
-      <c r="B69" s="23"/>
-      <c r="C69" s="23"/>
-      <c r="D69" s="24"/>
-      <c r="E69" s="23"/>
-      <c r="F69" s="62"/>
-    </row>
-    <row r="70" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A70" s="51"/>
-      <c r="B70" s="23"/>
-      <c r="C70" s="23"/>
-      <c r="D70" s="24"/>
-      <c r="E70" s="23"/>
-      <c r="F70" s="62"/>
-    </row>
-    <row r="71" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A71" s="51"/>
+      <c r="D66" s="24">
+        <v>1</v>
+      </c>
+      <c r="E66" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F66" s="64" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="86" t="s">
+        <v>183</v>
+      </c>
+      <c r="B67" s="23">
+        <v>43124</v>
+      </c>
+      <c r="C67" s="23">
+        <v>43124</v>
+      </c>
+      <c r="D67" s="24">
+        <v>1</v>
+      </c>
+      <c r="E67" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F67" s="61"/>
+    </row>
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="86" t="s">
+        <v>179</v>
+      </c>
+      <c r="B68" s="23">
+        <v>43124</v>
+      </c>
+      <c r="C68" s="23">
+        <v>43124</v>
+      </c>
+      <c r="D68" s="24">
+        <v>1</v>
+      </c>
+      <c r="E68" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F68" s="61" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="86" t="s">
+        <v>180</v>
+      </c>
+      <c r="B69" s="23">
+        <v>43124</v>
+      </c>
+      <c r="C69" s="23">
+        <v>43124</v>
+      </c>
+      <c r="D69" s="24">
+        <v>1</v>
+      </c>
+      <c r="E69" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F69" s="61"/>
+    </row>
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="69" t="s">
+        <v>173</v>
+      </c>
+      <c r="B70" s="23">
+        <v>43122</v>
+      </c>
+      <c r="C70" s="23">
+        <v>43124</v>
+      </c>
+      <c r="D70" s="24">
+        <v>1</v>
+      </c>
+      <c r="E70" s="23">
+        <v>43125</v>
+      </c>
+      <c r="F70" s="61"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="50"/>
       <c r="B71" s="23"/>
       <c r="C71" s="23"/>
       <c r="D71" s="24"/>
       <c r="E71" s="23"/>
-      <c r="F71" s="62"/>
-    </row>
-    <row r="72" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A72" s="51"/>
+      <c r="F71" s="61"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="50"/>
       <c r="B72" s="23"/>
       <c r="C72" s="23"/>
       <c r="D72" s="24"/>
       <c r="E72" s="23"/>
-      <c r="F72" s="62"/>
-    </row>
-    <row r="73" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="F72" s="61"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="50"/>
       <c r="B73" s="23"/>
       <c r="C73" s="23"/>
       <c r="D73" s="24"/>
       <c r="E73" s="23"/>
-      <c r="F73" s="60"/>
-    </row>
-    <row r="74" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="75" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
+      <c r="F73" s="61"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" s="50"/>
+      <c r="B74" s="23"/>
+      <c r="C74" s="23"/>
+      <c r="D74" s="24"/>
+      <c r="E74" s="23"/>
+      <c r="F74" s="61"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" s="50"/>
+      <c r="B75" s="23"/>
+      <c r="C75" s="23"/>
+      <c r="D75" s="24"/>
+      <c r="E75" s="23"/>
+      <c r="F75" s="61"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" s="50"/>
+      <c r="B76" s="23"/>
+      <c r="C76" s="23"/>
+      <c r="D76" s="24"/>
+      <c r="E76" s="23"/>
+      <c r="F76" s="61"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" s="50"/>
+      <c r="B77" s="23"/>
+      <c r="C77" s="23"/>
+      <c r="D77" s="24"/>
+      <c r="E77" s="23"/>
+      <c r="F77" s="61"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" s="50"/>
+      <c r="B78" s="23"/>
+      <c r="C78" s="23"/>
+      <c r="D78" s="24"/>
+      <c r="E78" s="23"/>
+      <c r="F78" s="61"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" s="50"/>
+      <c r="B79" s="23"/>
+      <c r="C79" s="23"/>
+      <c r="D79" s="24"/>
+      <c r="E79" s="23"/>
+      <c r="F79" s="61"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" s="50"/>
+      <c r="B80" s="23"/>
+      <c r="C80" s="23"/>
+      <c r="D80" s="24"/>
+      <c r="E80" s="23"/>
+      <c r="F80" s="61"/>
+    </row>
+    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B81" s="23"/>
+      <c r="C81" s="23"/>
+      <c r="D81" s="24"/>
+      <c r="E81" s="23"/>
+      <c r="F81" s="59"/>
+    </row>
+    <row r="82" spans="2:6" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="83" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="84" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="85" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <conditionalFormatting sqref="D2:D73">
-    <cfRule type="iconSet" priority="14">
+  <conditionalFormatting sqref="D2:D81">
+    <cfRule type="iconSet" priority="16">
       <iconSet iconSet="5Quarters" showValue="0">
         <cfvo type="percent" val="0"/>
         <cfvo type="num" val="0.2"/>
@@ -4456,70 +4683,70 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.6" zeroHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="9" width="4.78515625" style="42" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" style="42" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" style="42" customWidth="1"/>
-    <col min="12" max="12" width="13.85546875" style="42" customWidth="1"/>
-    <col min="13" max="17" width="11.140625" style="42" customWidth="1"/>
-    <col min="18" max="16384" width="8.85546875" hidden="1"/>
+    <col min="1" max="9" width="4.77734375" style="42" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" style="42" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" style="42" customWidth="1"/>
+    <col min="12" max="12" width="13.88671875" style="42" customWidth="1"/>
+    <col min="13" max="17" width="11.109375" style="42" customWidth="1"/>
+    <col min="18" max="16384" width="8.88671875" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="74.150000000000006" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:17" ht="72.599999999999994" x14ac:dyDescent="0.3">
       <c r="A1" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="41" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="41" t="s">
-        <v>122</v>
-      </c>
-      <c r="C1" s="41" t="s">
+      <c r="E1" s="41" t="s">
+        <v>120</v>
+      </c>
+      <c r="F1" s="41" t="s">
         <v>106</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="G1" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="H1" s="41" t="s">
+        <v>108</v>
+      </c>
+      <c r="I1" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="J1" s="44" t="s">
+        <v>113</v>
+      </c>
+      <c r="K1" s="44" t="s">
         <v>112</v>
       </c>
-      <c r="E1" s="41" t="s">
-        <v>121</v>
-      </c>
-      <c r="F1" s="41" t="s">
-        <v>107</v>
-      </c>
-      <c r="G1" s="41" t="s">
-        <v>108</v>
-      </c>
-      <c r="H1" s="41" t="s">
-        <v>109</v>
-      </c>
-      <c r="I1" s="41" t="s">
-        <v>110</v>
-      </c>
-      <c r="J1" s="44" t="s">
+      <c r="L1" s="44" t="s">
         <v>114</v>
       </c>
-      <c r="K1" s="44" t="s">
-        <v>113</v>
-      </c>
-      <c r="L1" s="44" t="s">
+      <c r="M1" s="41" t="s">
         <v>115</v>
       </c>
-      <c r="M1" s="41" t="s">
+      <c r="N1" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="N1" s="41" t="s">
+      <c r="O1" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="O1" s="42" t="s">
+      <c r="P1" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="P1" s="42" t="s">
+      <c r="Q1" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="Q1" s="42" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="43">
         <v>1</v>
       </c>
@@ -4542,13 +4769,13 @@
         <v>0</v>
       </c>
       <c r="H2" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I2" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="43">
         <v>2</v>
       </c>
@@ -4571,13 +4798,13 @@
         <v>0</v>
       </c>
       <c r="H3" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I3" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="43">
         <v>3</v>
       </c>
@@ -4600,13 +4827,13 @@
         <v>0</v>
       </c>
       <c r="H4" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I4" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="43">
         <v>4</v>
       </c>
@@ -4629,13 +4856,13 @@
         <v>0</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I5" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="43">
         <v>5</v>
       </c>
@@ -4658,13 +4885,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I6" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="43">
         <v>6</v>
       </c>
@@ -4687,13 +4914,13 @@
         <v>0</v>
       </c>
       <c r="H7" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I7" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="43">
         <v>7</v>
       </c>
@@ -4716,13 +4943,13 @@
         <v>0</v>
       </c>
       <c r="H8" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I8" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="43">
         <v>8</v>
       </c>
@@ -4745,13 +4972,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I9" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="43">
         <v>9</v>
       </c>
@@ -4774,13 +5001,13 @@
         <v>0</v>
       </c>
       <c r="H10" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I10" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="43">
         <v>10</v>
       </c>
@@ -4803,13 +5030,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I11" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="43">
         <v>11</v>
       </c>
@@ -4832,13 +5059,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I12" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="43">
         <v>12</v>
       </c>
@@ -4861,13 +5088,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I13" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="43">
         <v>13</v>
       </c>
@@ -4890,13 +5117,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I14" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="43">
         <v>14</v>
       </c>
@@ -4919,13 +5146,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I15" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="43">
         <v>15</v>
       </c>
@@ -4948,13 +5175,13 @@
         <v>0</v>
       </c>
       <c r="H16" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I16" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="43">
         <v>16</v>
       </c>
@@ -4977,13 +5204,13 @@
         <v>0</v>
       </c>
       <c r="H17" s="42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I17" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="43">
         <v>17</v>
       </c>
@@ -5006,13 +5233,13 @@
         <v>0</v>
       </c>
       <c r="H18" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I18" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="43">
         <v>18</v>
       </c>
@@ -5035,13 +5262,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I19" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="43">
         <v>19</v>
       </c>
@@ -5064,13 +5291,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I20" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="43">
         <v>20</v>
       </c>
@@ -5093,13 +5320,13 @@
         <v>0</v>
       </c>
       <c r="H21" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I21" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="43">
         <v>21</v>
       </c>
@@ -5122,13 +5349,13 @@
         <v>0</v>
       </c>
       <c r="H22" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I22" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="43">
         <v>22</v>
       </c>
@@ -5151,13 +5378,13 @@
         <v>0</v>
       </c>
       <c r="H23" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I23" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="43">
         <v>23</v>
       </c>
@@ -5180,13 +5407,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I24" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="43">
         <v>24</v>
       </c>
@@ -5209,13 +5436,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I25" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="43">
         <v>25</v>
       </c>
@@ -5238,13 +5465,13 @@
         <v>0</v>
       </c>
       <c r="H26" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I26" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="43">
         <v>26</v>
       </c>
@@ -5267,13 +5494,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I27" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="43">
         <v>27</v>
       </c>
@@ -5296,13 +5523,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I28" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="43">
         <v>28</v>
       </c>
@@ -5325,13 +5552,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I29" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="43">
         <v>29</v>
       </c>
@@ -5354,13 +5581,13 @@
         <v>0</v>
       </c>
       <c r="H30" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I30" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="43">
         <v>30</v>
       </c>
@@ -5383,13 +5610,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I31" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="43">
         <v>31</v>
       </c>
@@ -5412,13 +5639,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I32" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="43">
         <v>32</v>
       </c>
@@ -5441,13 +5668,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="42" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I33" s="42">
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -5460,164 +5687,164 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.6" zeroHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.78515625" customWidth="1"/>
-    <col min="2" max="2" width="12.640625" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" customWidth="1"/>
-    <col min="4" max="4" width="53.5703125" customWidth="1"/>
-    <col min="5" max="16384" width="8.85546875" hidden="1"/>
+    <col min="1" max="1" width="11.77734375" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" customWidth="1"/>
+    <col min="4" max="4" width="53.5546875" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" t="s">
         <v>125</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D1" s="45" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>126</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D2" s="45" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" s="45" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D4" s="45" t="s">
         <v>134</v>
       </c>
-      <c r="D1" s="45" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D5" s="45" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" t="s">
         <v>127</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C6" t="s">
         <v>128</v>
       </c>
-      <c r="C2" t="s">
-        <v>129</v>
-      </c>
-      <c r="D2" s="45" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>129</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="D6" s="45"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C7" t="s">
         <v>128</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" s="45" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C4" t="s">
-        <v>130</v>
-      </c>
-      <c r="D4" s="45" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>138</v>
-      </c>
-      <c r="B5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D5" s="45" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>106</v>
-      </c>
-      <c r="B6" t="s">
-        <v>128</v>
-      </c>
-      <c r="C6" t="s">
-        <v>129</v>
-      </c>
-      <c r="D6" s="45"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
+      <c r="D7" s="45"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>141</v>
       </c>
-      <c r="B7" t="s">
-        <v>128</v>
-      </c>
-      <c r="C7" t="s">
-        <v>129</v>
-      </c>
-      <c r="D7" s="45"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
+      <c r="D8" s="45"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>142</v>
       </c>
-      <c r="D8" s="45"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
+      <c r="D9" s="45"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>143</v>
       </c>
-      <c r="D9" s="45"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
+      <c r="C10" t="s">
         <v>144</v>
       </c>
-      <c r="C10" t="s">
-        <v>145</v>
-      </c>
       <c r="D10" s="45"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D11" s="45"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D12" s="45"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D13" s="45"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D14" s="45"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D15" s="45"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D16" s="45"/>
     </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D17" s="45"/>
     </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D18" s="45"/>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D19" s="45"/>
     </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D20" s="45"/>
     </row>
-    <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="D21" s="45"/>
     </row>
-    <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="D22" s="45"/>
     </row>
-    <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="D23" s="45"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Getting started with SLURM...
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="8652" windowHeight="8448" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="8652" windowHeight="7644" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Project Planner" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="191">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -659,6 +659,27 @@
   <si>
     <t>Make find_next_minimum also return phipeak</t>
   </si>
+  <si>
+    <t>Pre-compute equi-potent instanton suppression</t>
+  </si>
+  <si>
+    <t>Determine if best case and Hawking-Moss bound the action for super-potent instantons</t>
+  </si>
+  <si>
+    <t>Expand flowchart</t>
+  </si>
+  <si>
+    <t>Get Python multiprocessing and SLURM to play nice</t>
+  </si>
+  <si>
+    <t>Pool vs. Process, issues with subprocess?</t>
+  </si>
+  <si>
+    <t>Make different cpus indepently random</t>
+  </si>
+  <si>
+    <t>Fix V(phi_metaMin) &lt;= V(phi_absMin)</t>
+  </si>
 </sst>
 </file>
 
@@ -668,13 +689,34 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="48" x14ac:knownFonts="1">
+  <fonts count="51" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1149,98 +1191,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="43" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="46" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="36" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="39" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="46" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="49" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="47" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="47" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="47" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="47" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="47" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="43" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="46" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="36" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="39" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="45" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="39" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="42" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="46" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="49" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -1258,25 +1300,28 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="43" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="46" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="43" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="46" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="33" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="36" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -1290,102 +1335,114 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="18" fontId="27" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="18" fontId="24" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -1401,9 +1458,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="20">
     <cellStyle name="% complete" xfId="16"/>
@@ -1428,148 +1482,6 @@
     <cellStyle name="Title" xfId="8" builtinId="15" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="31">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="9" tint="-0.24994659260841701"/>
-        </left>
-        <right style="thin">
-          <color theme="9" tint="-0.24994659260841701"/>
-        </right>
-        <bottom style="thin">
-          <color theme="7"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color theme="7"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="9" tint="-0.24994659260841701"/>
-        </left>
-        <right style="thin">
-          <color theme="9" tint="-0.24994659260841701"/>
-        </right>
-        <bottom style="thin">
-          <color theme="9" tint="0.59996337778862885"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp">
-          <fgColor theme="7"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp">
-          <fgColor theme="7"/>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp">
-          <fgColor theme="7"/>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1919,6 +1831,148 @@
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="9" tint="-0.24994659260841701"/>
+        </left>
+        <right style="thin">
+          <color theme="9" tint="-0.24994659260841701"/>
+        </right>
+        <bottom style="thin">
+          <color theme="7"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color theme="7"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="9" tint="-0.24994659260841701"/>
+        </left>
+        <right style="thin">
+          <color theme="9" tint="-0.24994659260841701"/>
+        </right>
+        <bottom style="thin">
+          <color theme="9" tint="0.59996337778862885"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor theme="7"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor theme="7"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor theme="7"/>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1950,13 +2004,13 @@
     </filterColumn>
   </autoFilter>
   <sortState ref="A30:F81">
-    <sortCondition descending="1" ref="C1:C81"/>
+    <sortCondition ref="C1:C81"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" name="Task"/>
     <tableColumn id="2" name="Assigned"/>
     <tableColumn id="3" name="Due"/>
-    <tableColumn id="6" name=" " dataDxfId="30"/>
+    <tableColumn id="6" name=" " dataDxfId="20"/>
     <tableColumn id="4" name="Review"/>
     <tableColumn id="5" name="Notes"/>
   </tableColumns>
@@ -1965,26 +2019,26 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:Q33" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:Q33" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="A1:Q33"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="Test ID" dataDxfId="27"/>
-    <tableColumn id="2" name="log10(mv)" dataDxfId="26"/>
-    <tableColumn id="3" name="mh" dataDxfId="25"/>
-    <tableColumn id="4" name="log10(n_iter)" dataDxfId="24"/>
-    <tableColumn id="5" name="lambda_screen" dataDxfId="23"/>
-    <tableColumn id="6" name="fix_Lambda" dataDxfId="22"/>
-    <tableColumn id="7" name="fix_Q" dataDxfId="21"/>
-    <tableColumn id="8" name="measure" dataDxfId="20"/>
-    <tableColumn id="9" name="n_tunnel_max" dataDxfId="19"/>
-    <tableColumn id="10" name="End Date" dataDxfId="18"/>
-    <tableColumn id="11" name="Runtime" dataDxfId="17"/>
-    <tableColumn id="12" name="File name" dataDxfId="16"/>
-    <tableColumn id="13" name="Column13" dataDxfId="15"/>
-    <tableColumn id="14" name="Column14" dataDxfId="14"/>
-    <tableColumn id="15" name="Column15" dataDxfId="13"/>
-    <tableColumn id="16" name="Column16" dataDxfId="12"/>
-    <tableColumn id="17" name="Column17" dataDxfId="11"/>
+    <tableColumn id="1" name="Test ID" dataDxfId="17"/>
+    <tableColumn id="2" name="log10(mv)" dataDxfId="16"/>
+    <tableColumn id="3" name="mh" dataDxfId="15"/>
+    <tableColumn id="4" name="log10(n_iter)" dataDxfId="14"/>
+    <tableColumn id="5" name="lambda_screen" dataDxfId="13"/>
+    <tableColumn id="6" name="fix_Lambda" dataDxfId="12"/>
+    <tableColumn id="7" name="fix_Q" dataDxfId="11"/>
+    <tableColumn id="8" name="measure" dataDxfId="10"/>
+    <tableColumn id="9" name="n_tunnel_max" dataDxfId="9"/>
+    <tableColumn id="10" name="End Date" dataDxfId="8"/>
+    <tableColumn id="11" name="Runtime" dataDxfId="7"/>
+    <tableColumn id="12" name="File name" dataDxfId="6"/>
+    <tableColumn id="13" name="Column13" dataDxfId="5"/>
+    <tableColumn id="14" name="Column14" dataDxfId="4"/>
+    <tableColumn id="15" name="Column15" dataDxfId="3"/>
+    <tableColumn id="16" name="Column16" dataDxfId="2"/>
+    <tableColumn id="17" name="Column17" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1997,7 +2051,7 @@
     <tableColumn id="1" name="Quantity"/>
     <tableColumn id="2" name="Dimensions"/>
     <tableColumn id="3" name="Units"/>
-    <tableColumn id="4" name="Description" dataDxfId="10"/>
+    <tableColumn id="4" name="Description" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2258,13 +2312,13 @@
       <c r="G1" s="10"/>
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
@@ -2272,66 +2326,66 @@
         <v>8</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="78" t="s">
+      <c r="K2" s="85" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="79"/>
-      <c r="M2" s="79"/>
-      <c r="N2" s="79"/>
-      <c r="O2" s="80"/>
+      <c r="L2" s="86"/>
+      <c r="M2" s="86"/>
+      <c r="N2" s="86"/>
+      <c r="O2" s="87"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="78" t="s">
+      <c r="Q2" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="81"/>
-      <c r="S2" s="81"/>
-      <c r="T2" s="80"/>
+      <c r="R2" s="88"/>
+      <c r="S2" s="88"/>
+      <c r="T2" s="87"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="70" t="s">
+      <c r="V2" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="71"/>
-      <c r="X2" s="71"/>
-      <c r="Y2" s="82"/>
+      <c r="W2" s="78"/>
+      <c r="X2" s="78"/>
+      <c r="Y2" s="89"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="83" t="s">
+      <c r="AA2" s="90" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="84"/>
-      <c r="AC2" s="84"/>
-      <c r="AD2" s="84"/>
-      <c r="AE2" s="84"/>
-      <c r="AF2" s="84"/>
-      <c r="AG2" s="85"/>
+      <c r="AB2" s="91"/>
+      <c r="AC2" s="91"/>
+      <c r="AD2" s="91"/>
+      <c r="AE2" s="91"/>
+      <c r="AF2" s="91"/>
+      <c r="AG2" s="92"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="70" t="s">
+      <c r="AI2" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="71"/>
-      <c r="AK2" s="71"/>
-      <c r="AL2" s="71"/>
-      <c r="AM2" s="71"/>
-      <c r="AN2" s="71"/>
-      <c r="AO2" s="71"/>
-      <c r="AP2" s="71"/>
+      <c r="AJ2" s="78"/>
+      <c r="AK2" s="78"/>
+      <c r="AL2" s="78"/>
+      <c r="AM2" s="78"/>
+      <c r="AN2" s="78"/>
+      <c r="AO2" s="78"/>
+      <c r="AP2" s="78"/>
     </row>
     <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="75" t="s">
+      <c r="B3" s="80" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="75" t="s">
+      <c r="D3" s="82" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="75" t="s">
+      <c r="E3" s="82" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="75" t="s">
+      <c r="F3" s="82" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="77" t="s">
+      <c r="G3" s="84" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -2460,12 +2514,12 @@
       <c r="AW3" s="18"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="74"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
+      <c r="B4" s="81"/>
+      <c r="C4" s="83"/>
+      <c r="D4" s="83"/>
+      <c r="E4" s="83"/>
+      <c r="F4" s="83"/>
+      <c r="G4" s="83"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -3184,38 +3238,38 @@
     <mergeCell ref="AA2:AG2"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:BO31">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="30" priority="1">
       <formula>PercentComplete</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="3">
+    <cfRule type="expression" dxfId="29" priority="3">
       <formula>PercentCompleteBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="4">
+    <cfRule type="expression" dxfId="28" priority="4">
       <formula>Actual</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="5">
+    <cfRule type="expression" dxfId="27" priority="5">
       <formula>ActualBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="6">
+    <cfRule type="expression" dxfId="26" priority="6">
       <formula>Plan</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="7">
+    <cfRule type="expression" dxfId="25" priority="7">
       <formula>H$4=period_selected</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="11">
+    <cfRule type="expression" dxfId="24" priority="11">
       <formula>MOD(COLUMN(),2)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="12">
+    <cfRule type="expression" dxfId="23" priority="12">
       <formula>MOD(COLUMN(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:BO32">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="22" priority="2">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:BO4">
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule type="expression" dxfId="21" priority="8">
       <formula>H$4=period_selected</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3258,7 +3312,7 @@
     <col min="3" max="3" width="10.5546875" style="21" customWidth="1"/>
     <col min="4" max="4" width="5.21875" style="21" customWidth="1"/>
     <col min="5" max="5" width="9.77734375" style="21" customWidth="1"/>
-    <col min="6" max="6" width="80.88671875" style="21" customWidth="1"/>
+    <col min="6" max="6" width="70.33203125" style="21" customWidth="1"/>
     <col min="7" max="7" width="0" style="21" hidden="1" customWidth="1"/>
     <col min="8" max="16384" width="8.88671875" style="21" hidden="1"/>
   </cols>
@@ -3813,24 +3867,22 @@
       <c r="F29" s="56"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="21" t="s">
-        <v>62</v>
+      <c r="A30" s="70" t="s">
+        <v>181</v>
       </c>
       <c r="B30" s="23">
         <v>43124</v>
       </c>
       <c r="C30" s="23">
-        <v>43130</v>
+        <v>43124</v>
       </c>
       <c r="D30" s="24">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E30" s="23">
         <v>43132</v>
       </c>
-      <c r="F30" s="59" t="s">
-        <v>63</v>
-      </c>
+      <c r="F30" s="61"/>
     </row>
     <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="26" t="s">
@@ -3873,75 +3925,73 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="21" t="s">
-        <v>58</v>
+      <c r="A33" s="70" t="s">
+        <v>177</v>
       </c>
       <c r="B33" s="23">
         <v>43124</v>
       </c>
       <c r="C33" s="23">
-        <v>43130</v>
+        <v>43125</v>
       </c>
       <c r="D33" s="24">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="E33" s="23">
         <v>43132</v>
       </c>
-      <c r="F33" s="57" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="67" t="s">
-        <v>168</v>
+      <c r="F33" s="71" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="70" t="s">
+        <v>175</v>
       </c>
       <c r="B34" s="23">
-        <v>43119</v>
+        <v>43124</v>
       </c>
       <c r="C34" s="23">
-        <v>43126</v>
+        <v>43124</v>
       </c>
       <c r="D34" s="24">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E34" s="23">
         <v>43125</v>
       </c>
       <c r="F34" s="61"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="21" t="s">
-        <v>61</v>
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="69" t="s">
+        <v>174</v>
       </c>
       <c r="B35" s="23">
-        <v>43124</v>
+        <v>43122</v>
       </c>
       <c r="C35" s="23">
-        <v>43126</v>
+        <v>43122</v>
       </c>
       <c r="D35" s="24">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E35" s="23">
         <v>43125</v>
       </c>
-      <c r="F35" s="61" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="86" t="s">
-        <v>182</v>
+      <c r="F35" s="61"/>
+    </row>
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="50" t="s">
+        <v>153</v>
       </c>
       <c r="B36" s="23">
-        <v>43124</v>
+        <v>43112</v>
       </c>
       <c r="C36" s="23">
-        <v>43125</v>
+        <v>43118</v>
       </c>
       <c r="D36" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="23">
         <v>43125</v>
@@ -3949,14 +3999,14 @@
       <c r="F36" s="61"/>
     </row>
     <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="86" t="s">
-        <v>175</v>
+      <c r="A37" s="55" t="s">
+        <v>162</v>
       </c>
       <c r="B37" s="23">
-        <v>43124</v>
+        <v>43117</v>
       </c>
       <c r="C37" s="23">
-        <v>43124</v>
+        <v>43117</v>
       </c>
       <c r="D37" s="24">
         <v>1</v>
@@ -3986,25 +4036,23 @@
         <v>152</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="86" t="s">
-        <v>177</v>
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="67" t="s">
+        <v>167</v>
       </c>
       <c r="B39" s="23">
-        <v>43124</v>
+        <v>43119</v>
       </c>
       <c r="C39" s="23">
-        <v>43125</v>
+        <v>43122</v>
       </c>
       <c r="D39" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E39" s="23">
         <v>43125</v>
       </c>
-      <c r="F39" s="87" t="s">
-        <v>176</v>
-      </c>
+      <c r="F39" s="61"/>
     </row>
     <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="47" t="s">
@@ -4024,24 +4072,21 @@
       </c>
       <c r="F40" s="33"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="40" t="s">
-        <v>104</v>
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="68" t="s">
+        <v>169</v>
       </c>
       <c r="B41" s="23">
-        <v>43124</v>
+        <v>43119</v>
       </c>
       <c r="C41" s="23">
-        <v>43124</v>
+        <v>43122</v>
       </c>
       <c r="D41" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" s="23">
         <v>43125</v>
-      </c>
-      <c r="F41" s="87" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
@@ -4050,7 +4095,7 @@
       </c>
       <c r="B42" s="23">
         <f ca="1">TODAY()</f>
-        <v>43124</v>
+        <v>43131</v>
       </c>
       <c r="C42" s="23">
         <v>43118</v>
@@ -4064,14 +4109,14 @@
       <c r="F42" s="33"/>
     </row>
     <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="69" t="s">
-        <v>174</v>
+      <c r="A43" s="67" t="s">
+        <v>170</v>
       </c>
       <c r="B43" s="23">
-        <v>43122</v>
+        <v>43119</v>
       </c>
       <c r="C43" s="23">
-        <v>43122</v>
+        <v>43119</v>
       </c>
       <c r="D43" s="24">
         <v>1</v>
@@ -4079,7 +4124,9 @@
       <c r="E43" s="23">
         <v>43125</v>
       </c>
-      <c r="F43" s="61"/>
+      <c r="F43" s="68" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="49" t="s">
@@ -4087,7 +4134,7 @@
       </c>
       <c r="B44" s="23">
         <f ca="1">TODAY()</f>
-        <v>43124</v>
+        <v>43131</v>
       </c>
       <c r="C44" s="23">
         <v>43118</v>
@@ -4106,7 +4153,7 @@
       </c>
       <c r="B45" s="23">
         <f ca="1">TODAY()</f>
-        <v>43124</v>
+        <v>43131</v>
       </c>
       <c r="C45" s="23">
         <v>43118</v>
@@ -4120,14 +4167,14 @@
       <c r="F45" s="33"/>
     </row>
     <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="50" t="s">
-        <v>153</v>
+      <c r="A46" s="69" t="s">
+        <v>172</v>
       </c>
       <c r="B46" s="23">
-        <v>43112</v>
+        <v>43122</v>
       </c>
       <c r="C46" s="23">
-        <v>43118</v>
+        <v>43122</v>
       </c>
       <c r="D46" s="24">
         <v>1</v>
@@ -4143,7 +4190,7 @@
       </c>
       <c r="B47" s="23">
         <f ca="1">TODAY()</f>
-        <v>43124</v>
+        <v>43131</v>
       </c>
       <c r="C47" s="23"/>
       <c r="D47" s="24">
@@ -4273,14 +4320,14 @@
       <c r="F54" s="33"/>
     </row>
     <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="55" t="s">
-        <v>162</v>
+      <c r="A55" s="49" t="s">
+        <v>149</v>
       </c>
       <c r="B55" s="23">
-        <v>43117</v>
+        <v>43112</v>
       </c>
       <c r="C55" s="23">
-        <v>43117</v>
+        <v>43118</v>
       </c>
       <c r="D55" s="24">
         <v>1</v>
@@ -4288,7 +4335,9 @@
       <c r="E55" s="23">
         <v>43125</v>
       </c>
-      <c r="F55" s="61"/>
+      <c r="F55" s="64" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="55" t="s">
@@ -4345,14 +4394,14 @@
       <c r="F58" s="61"/>
     </row>
     <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="67" t="s">
-        <v>167</v>
+      <c r="A59" s="70" t="s">
+        <v>183</v>
       </c>
       <c r="B59" s="23">
-        <v>43119</v>
+        <v>43124</v>
       </c>
       <c r="C59" s="23">
-        <v>43122</v>
+        <v>43124</v>
       </c>
       <c r="D59" s="24">
         <v>1</v>
@@ -4383,14 +4432,14 @@
       </c>
     </row>
     <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="68" t="s">
-        <v>169</v>
+      <c r="A61" s="70" t="s">
+        <v>179</v>
       </c>
       <c r="B61" s="23">
-        <v>43119</v>
+        <v>43124</v>
       </c>
       <c r="C61" s="23">
-        <v>43122</v>
+        <v>43124</v>
       </c>
       <c r="D61" s="24">
         <v>1</v>
@@ -4398,16 +4447,19 @@
       <c r="E61" s="23">
         <v>43125</v>
       </c>
+      <c r="F61" s="61" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="67" t="s">
-        <v>170</v>
+      <c r="A62" s="70" t="s">
+        <v>180</v>
       </c>
       <c r="B62" s="23">
-        <v>43119</v>
+        <v>43124</v>
       </c>
       <c r="C62" s="23">
-        <v>43119</v>
+        <v>43124</v>
       </c>
       <c r="D62" s="24">
         <v>1</v>
@@ -4415,19 +4467,17 @@
       <c r="E62" s="23">
         <v>43125</v>
       </c>
-      <c r="F62" s="68" t="s">
-        <v>171</v>
-      </c>
+      <c r="F62" s="61"/>
     </row>
     <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="69" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B63" s="23">
         <v>43122</v>
       </c>
       <c r="C63" s="23">
-        <v>43122</v>
+        <v>43124</v>
       </c>
       <c r="D63" s="24">
         <v>1</v>
@@ -4458,84 +4508,84 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="86" t="s">
-        <v>181</v>
+      <c r="A65" s="70" t="s">
+        <v>182</v>
       </c>
       <c r="B65" s="23">
         <v>43124</v>
       </c>
       <c r="C65" s="23">
+        <v>43125</v>
+      </c>
+      <c r="D65" s="24">
+        <v>0</v>
+      </c>
+      <c r="E65" s="23">
+        <v>43132</v>
+      </c>
+      <c r="F65" s="61"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B66" s="23">
         <v>43124</v>
       </c>
-      <c r="D65" s="24">
-        <v>0</v>
-      </c>
-      <c r="E65" s="23">
+      <c r="C66" s="23">
+        <v>43126</v>
+      </c>
+      <c r="D66" s="24">
+        <v>0.75</v>
+      </c>
+      <c r="E66" s="23">
+        <v>43132</v>
+      </c>
+      <c r="F66" s="61" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="73" t="s">
+        <v>184</v>
+      </c>
+      <c r="B67" s="23">
         <v>43125</v>
       </c>
-      <c r="F65" s="61"/>
-    </row>
-    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="49" t="s">
-        <v>149</v>
-      </c>
-      <c r="B66" s="23">
-        <v>43112</v>
-      </c>
-      <c r="C66" s="23">
-        <v>43118</v>
-      </c>
-      <c r="D66" s="24">
-        <v>1</v>
-      </c>
-      <c r="E66" s="23">
-        <v>43125</v>
-      </c>
-      <c r="F66" s="64" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="86" t="s">
-        <v>183</v>
-      </c>
-      <c r="B67" s="23">
-        <v>43124</v>
-      </c>
       <c r="C67" s="23">
-        <v>43124</v>
+        <v>43126</v>
       </c>
       <c r="D67" s="24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E67" s="23">
-        <v>43125</v>
-      </c>
-      <c r="F67" s="61"/>
-    </row>
-    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="86" t="s">
-        <v>179</v>
+        <v>43132</v>
+      </c>
+      <c r="F67" s="74" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="67" t="s">
+        <v>168</v>
       </c>
       <c r="B68" s="23">
-        <v>43124</v>
+        <v>43119</v>
       </c>
       <c r="C68" s="23">
-        <v>43124</v>
+        <v>43129</v>
       </c>
       <c r="D68" s="24">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E68" s="23">
-        <v>43125</v>
-      </c>
-      <c r="F68" s="61" t="s">
-        <v>86</v>
-      </c>
+        <v>43132</v>
+      </c>
+      <c r="F68" s="61"/>
     </row>
     <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="86" t="s">
-        <v>180</v>
+      <c r="A69" s="40" t="s">
+        <v>104</v>
       </c>
       <c r="B69" s="23">
         <v>43124</v>
@@ -4543,70 +4593,128 @@
       <c r="C69" s="23">
         <v>43124</v>
       </c>
-      <c r="D69" s="24">
-        <v>1</v>
+      <c r="D69" s="72">
+        <v>1.5</v>
       </c>
       <c r="E69" s="23">
         <v>43125</v>
       </c>
-      <c r="F69" s="61"/>
-    </row>
-    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="69" t="s">
-        <v>173</v>
+      <c r="F69" s="71" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="21" t="s">
+        <v>62</v>
       </c>
       <c r="B70" s="23">
-        <v>43122</v>
+        <v>43124</v>
       </c>
       <c r="C70" s="23">
+        <v>43130</v>
+      </c>
+      <c r="D70" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="E70" s="23">
+        <v>43132</v>
+      </c>
+      <c r="F70" s="59" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B71" s="23">
         <v>43124</v>
       </c>
-      <c r="D70" s="24">
-        <v>1</v>
-      </c>
-      <c r="E70" s="23">
+      <c r="C71" s="23">
+        <v>43130</v>
+      </c>
+      <c r="D71" s="24">
+        <v>0.75</v>
+      </c>
+      <c r="E71" s="23">
+        <v>43132</v>
+      </c>
+      <c r="F71" s="57" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="73" t="s">
+        <v>186</v>
+      </c>
+      <c r="B72" s="23">
         <v>43125</v>
       </c>
-      <c r="F70" s="61"/>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="50"/>
-      <c r="B71" s="23"/>
-      <c r="C71" s="23"/>
-      <c r="D71" s="24"/>
-      <c r="E71" s="23"/>
-      <c r="F71" s="61"/>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="50"/>
-      <c r="B72" s="23"/>
-      <c r="C72" s="23"/>
-      <c r="D72" s="24"/>
-      <c r="E72" s="23"/>
+      <c r="C72" s="23">
+        <v>43126</v>
+      </c>
+      <c r="D72" s="24">
+        <v>1</v>
+      </c>
+      <c r="E72" s="23">
+        <v>43132</v>
+      </c>
       <c r="F72" s="61"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="50"/>
-      <c r="B73" s="23"/>
-      <c r="C73" s="23"/>
-      <c r="D73" s="24"/>
-      <c r="E73" s="23"/>
-      <c r="F73" s="61"/>
+      <c r="A73" s="75" t="s">
+        <v>187</v>
+      </c>
+      <c r="B73" s="23">
+        <v>43129</v>
+      </c>
+      <c r="C73" s="23">
+        <v>43130</v>
+      </c>
+      <c r="D73" s="24">
+        <v>0</v>
+      </c>
+      <c r="E73" s="23">
+        <v>43132</v>
+      </c>
+      <c r="F73" s="76" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="50"/>
-      <c r="B74" s="23"/>
-      <c r="C74" s="23"/>
-      <c r="D74" s="24"/>
-      <c r="E74" s="23"/>
+      <c r="A74" s="93" t="s">
+        <v>189</v>
+      </c>
+      <c r="B74" s="23">
+        <v>43131</v>
+      </c>
+      <c r="C74" s="23">
+        <v>43131</v>
+      </c>
+      <c r="D74" s="24">
+        <v>1</v>
+      </c>
+      <c r="E74" s="23">
+        <v>43132</v>
+      </c>
       <c r="F74" s="61"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="50"/>
-      <c r="B75" s="23"/>
-      <c r="C75" s="23"/>
-      <c r="D75" s="24"/>
-      <c r="E75" s="23"/>
+      <c r="A75" s="93" t="s">
+        <v>190</v>
+      </c>
+      <c r="B75" s="23">
+        <v>43131</v>
+      </c>
+      <c r="C75" s="23">
+        <v>43131</v>
+      </c>
+      <c r="D75" s="24">
+        <v>0</v>
+      </c>
+      <c r="E75" s="23">
+        <v>43132</v>
+      </c>
       <c r="F75" s="61"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fixed shifting of V_min
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="8652" windowHeight="7644" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="8649" windowHeight="7646" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Project Planner" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="194">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -680,6 +680,15 @@
   <si>
     <t>Fix V(phi_metaMin) &lt;= V(phi_absMin)</t>
   </si>
+  <si>
+    <t>Check for nearby minima with V_min ~= 0</t>
+  </si>
+  <si>
+    <t>Add eternal inflation flags to output</t>
+  </si>
+  <si>
+    <t>Choose threshold for vacuum energy density</t>
+  </si>
 </sst>
 </file>
 
@@ -689,13 +698,20 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="51" x14ac:knownFonts="1">
+  <fonts count="52" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1191,98 +1207,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="46" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="47" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="39" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="40" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="46" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="49" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="50" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="48" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="48" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="48" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="48" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="48" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="46" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="47" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="39" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="40" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="46" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="42" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="43" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="49" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="50" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -1300,25 +1316,26 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="47" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="47" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="36" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="37" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -1334,23 +1351,23 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -1359,90 +1376,90 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="18" fontId="27" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="28" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -1997,14 +2014,13 @@
     <filterColumn colId="3">
       <filters blank="1">
         <filter val="0"/>
-        <filter val="0.25"/>
         <filter val="0.5"/>
         <filter val="0.75"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <sortState ref="A30:F81">
-    <sortCondition ref="C1:C81"/>
+    <sortCondition descending="1" ref="C1:C81"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" name="Task"/>
@@ -2289,19 +2305,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BO31"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="2" customWidth="1"/>
-    <col min="3" max="6" width="11.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" style="4" customWidth="1"/>
-    <col min="8" max="27" width="3.5546875" style="1" customWidth="1"/>
-    <col min="28" max="48" width="3.5546875" customWidth="1"/>
+    <col min="1" max="1" width="2.640625" customWidth="1"/>
+    <col min="2" max="2" width="15.640625" style="2" customWidth="1"/>
+    <col min="3" max="6" width="11.640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.640625" style="4" customWidth="1"/>
+    <col min="8" max="27" width="3.5703125" style="1" customWidth="1"/>
+    <col min="28" max="48" width="3.5703125" customWidth="1"/>
     <col min="49" max="67" width="0" hidden="1" customWidth="1"/>
-    <col min="68" max="16384" width="2.77734375" hidden="1"/>
+    <col min="68" max="16384" width="2.78515625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.05">
+    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.4">
       <c r="B1" s="11" t="s">
         <v>40</v>
       </c>
@@ -2311,14 +2327,14 @@
       <c r="F1" s="10"/>
       <c r="G1" s="10"/>
     </row>
-    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="79" t="s">
+    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B2" s="80" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
+      <c r="C2" s="80"/>
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="80"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
@@ -2326,66 +2342,66 @@
         <v>8</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="85" t="s">
+      <c r="K2" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="86"/>
-      <c r="M2" s="86"/>
-      <c r="N2" s="86"/>
-      <c r="O2" s="87"/>
+      <c r="L2" s="87"/>
+      <c r="M2" s="87"/>
+      <c r="N2" s="87"/>
+      <c r="O2" s="88"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="85" t="s">
+      <c r="Q2" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="88"/>
-      <c r="S2" s="88"/>
-      <c r="T2" s="87"/>
+      <c r="R2" s="89"/>
+      <c r="S2" s="89"/>
+      <c r="T2" s="88"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="77" t="s">
+      <c r="V2" s="78" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="78"/>
-      <c r="X2" s="78"/>
-      <c r="Y2" s="89"/>
+      <c r="W2" s="79"/>
+      <c r="X2" s="79"/>
+      <c r="Y2" s="90"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="90" t="s">
+      <c r="AA2" s="91" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="91"/>
-      <c r="AC2" s="91"/>
-      <c r="AD2" s="91"/>
-      <c r="AE2" s="91"/>
-      <c r="AF2" s="91"/>
-      <c r="AG2" s="92"/>
+      <c r="AB2" s="92"/>
+      <c r="AC2" s="92"/>
+      <c r="AD2" s="92"/>
+      <c r="AE2" s="92"/>
+      <c r="AF2" s="92"/>
+      <c r="AG2" s="93"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="77" t="s">
+      <c r="AI2" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="78"/>
-      <c r="AK2" s="78"/>
-      <c r="AL2" s="78"/>
-      <c r="AM2" s="78"/>
-      <c r="AN2" s="78"/>
-      <c r="AO2" s="78"/>
-      <c r="AP2" s="78"/>
-    </row>
-    <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="80" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="82" t="s">
+      <c r="AJ2" s="79"/>
+      <c r="AK2" s="79"/>
+      <c r="AL2" s="79"/>
+      <c r="AM2" s="79"/>
+      <c r="AN2" s="79"/>
+      <c r="AO2" s="79"/>
+      <c r="AP2" s="79"/>
+    </row>
+    <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="81" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="82" t="s">
+      <c r="D3" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="82" t="s">
+      <c r="E3" s="83" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="82" t="s">
+      <c r="F3" s="83" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="84" t="s">
+      <c r="G3" s="85" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -2513,13 +2529,13 @@
       </c>
       <c r="AW3" s="18"/>
     </row>
-    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="81"/>
-      <c r="C4" s="83"/>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
-      <c r="G4" s="83"/>
+    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="82"/>
+      <c r="C4" s="84"/>
+      <c r="D4" s="84"/>
+      <c r="E4" s="84"/>
+      <c r="F4" s="84"/>
+      <c r="G4" s="84"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -2663,7 +2679,7 @@
       <c r="BN4" s="3"/>
       <c r="BO4" s="3"/>
     </row>
-    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B5" s="6" t="s">
         <v>38</v>
       </c>
@@ -2686,7 +2702,7 @@
       <c r="X5" s="19"/>
       <c r="Y5" s="19"/>
     </row>
-    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="6" t="s">
         <v>35</v>
       </c>
@@ -2709,7 +2725,7 @@
       <c r="X6" s="19"/>
       <c r="Y6" s="19"/>
     </row>
-    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="6" t="s">
         <v>29</v>
       </c>
@@ -2732,7 +2748,7 @@
       <c r="X7" s="19"/>
       <c r="Y7" s="19"/>
     </row>
-    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="6" t="s">
         <v>32</v>
       </c>
@@ -2753,7 +2769,7 @@
       <c r="X8" s="19"/>
       <c r="Y8" s="19"/>
     </row>
-    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="6" t="s">
         <v>33</v>
       </c>
@@ -2774,7 +2790,7 @@
       <c r="X9" s="19"/>
       <c r="Y9" s="19"/>
     </row>
-    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B10" s="6" t="s">
         <v>34</v>
       </c>
@@ -2795,7 +2811,7 @@
       <c r="X10" s="19"/>
       <c r="Y10" s="19"/>
     </row>
-    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="6" t="s">
         <v>39</v>
       </c>
@@ -2816,7 +2832,7 @@
       <c r="X11" s="19"/>
       <c r="Y11" s="19"/>
     </row>
-    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
@@ -2839,7 +2855,7 @@
       <c r="X12" s="19"/>
       <c r="Y12" s="19"/>
     </row>
-    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B13" s="6" t="s">
         <v>31</v>
       </c>
@@ -2860,7 +2876,7 @@
       <c r="X13" s="19"/>
       <c r="Y13" s="19"/>
     </row>
-    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B14" s="6" t="s">
         <v>36</v>
       </c>
@@ -2881,7 +2897,7 @@
       <c r="X14" s="19"/>
       <c r="Y14" s="19"/>
     </row>
-    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B15" s="6" t="s">
         <v>37</v>
       </c>
@@ -2902,7 +2918,7 @@
       <c r="X15" s="19"/>
       <c r="Y15" s="19"/>
     </row>
-    <row r="16" spans="2:67" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:67" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B16" s="6" t="s">
         <v>1</v>
       </c>
@@ -2922,7 +2938,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B17" s="6" t="s">
         <v>2</v>
       </c>
@@ -2942,7 +2958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B18" s="6" t="s">
         <v>3</v>
       </c>
@@ -2962,7 +2978,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B19" s="6" t="s">
         <v>4</v>
       </c>
@@ -2982,7 +2998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B20" s="6" t="s">
         <v>5</v>
       </c>
@@ -3002,7 +3018,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B21" s="6" t="s">
         <v>6</v>
       </c>
@@ -3022,7 +3038,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B22" s="6" t="s">
         <v>7</v>
       </c>
@@ -3042,7 +3058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B23" s="6" t="s">
         <v>8</v>
       </c>
@@ -3062,7 +3078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B24" s="6" t="s">
         <v>9</v>
       </c>
@@ -3082,7 +3098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B25" s="6" t="s">
         <v>10</v>
       </c>
@@ -3102,7 +3118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B26" s="6" t="s">
         <v>11</v>
       </c>
@@ -3122,7 +3138,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B27" s="6" t="s">
         <v>12</v>
       </c>
@@ -3142,7 +3158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B28" s="6" t="s">
         <v>13</v>
       </c>
@@ -3162,7 +3178,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B29" s="6" t="s">
         <v>14</v>
       </c>
@@ -3182,7 +3198,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B30" s="6" t="s">
         <v>15</v>
       </c>
@@ -3202,7 +3218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B31" s="6" t="s">
         <v>16</v>
       </c>
@@ -3305,19 +3321,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G85"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="51.21875" style="21" customWidth="1"/>
-    <col min="2" max="2" width="9.77734375" style="21" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" style="21" customWidth="1"/>
-    <col min="4" max="4" width="5.21875" style="21" customWidth="1"/>
-    <col min="5" max="5" width="9.77734375" style="21" customWidth="1"/>
-    <col min="6" max="6" width="70.33203125" style="21" customWidth="1"/>
+    <col min="1" max="1" width="51.2109375" style="21" customWidth="1"/>
+    <col min="2" max="2" width="9.78515625" style="21" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" style="21" customWidth="1"/>
+    <col min="4" max="4" width="5.2109375" style="21" customWidth="1"/>
+    <col min="5" max="5" width="9.78515625" style="21" customWidth="1"/>
+    <col min="6" max="6" width="70.35546875" style="21" customWidth="1"/>
     <col min="7" max="7" width="0" style="21" hidden="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="21" hidden="1"/>
+    <col min="8" max="16384" width="8.85546875" style="21" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
       <c r="A1" s="21" t="s">
         <v>41</v>
       </c>
@@ -3337,7 +3353,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A2" s="29" t="s">
         <v>80</v>
       </c>
@@ -3357,7 +3373,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A3" s="26" t="s">
         <v>66</v>
       </c>
@@ -3377,7 +3393,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A4" s="21" t="s">
         <v>47</v>
       </c>
@@ -3394,7 +3410,7 @@
         <v>42984</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A5" s="21" t="s">
         <v>48</v>
       </c>
@@ -3414,7 +3430,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A6" s="21" t="s">
         <v>50</v>
       </c>
@@ -3431,7 +3447,7 @@
         <v>42984</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A7" s="21" t="s">
         <v>52</v>
       </c>
@@ -3451,7 +3467,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A8" s="21" t="s">
         <v>51</v>
       </c>
@@ -3468,7 +3484,7 @@
         <v>42990</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A9" s="21" t="s">
         <v>55</v>
       </c>
@@ -3488,7 +3504,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A10" s="30" t="s">
         <v>81</v>
       </c>
@@ -3508,7 +3524,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A11" s="21" t="s">
         <v>60</v>
       </c>
@@ -3528,7 +3544,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A12" s="21" t="s">
         <v>56</v>
       </c>
@@ -3548,7 +3564,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A13" s="27" t="s">
         <v>73</v>
       </c>
@@ -3568,7 +3584,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A14" s="31" t="s">
         <v>82</v>
       </c>
@@ -3585,7 +3601,7 @@
         <v>43006</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" s="21" t="s">
         <v>53</v>
       </c>
@@ -3605,7 +3621,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="21" t="s">
         <v>54</v>
       </c>
@@ -3625,7 +3641,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A17" s="33" t="s">
         <v>84</v>
       </c>
@@ -3642,7 +3658,7 @@
         <v>43027</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A18" s="33" t="s">
         <v>89</v>
       </c>
@@ -3660,7 +3676,7 @@
       </c>
       <c r="F18" s="33"/>
     </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A19" s="33" t="s">
         <v>90</v>
       </c>
@@ -3680,7 +3696,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A20" s="35" t="s">
         <v>95</v>
       </c>
@@ -3698,7 +3714,7 @@
       </c>
       <c r="F20" s="33"/>
     </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A21" s="35" t="s">
         <v>94</v>
       </c>
@@ -3716,7 +3732,7 @@
       </c>
       <c r="F21" s="33"/>
     </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A22" s="34" t="s">
         <v>92</v>
       </c>
@@ -3736,7 +3752,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A23" s="36" t="s">
         <v>98</v>
       </c>
@@ -3756,7 +3772,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A24" s="38" t="s">
         <v>100</v>
       </c>
@@ -3776,7 +3792,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A25" s="36" t="s">
         <v>97</v>
       </c>
@@ -3794,7 +3810,7 @@
       </c>
       <c r="F25" s="33"/>
     </row>
-    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A26" s="35" t="s">
         <v>96</v>
       </c>
@@ -3812,7 +3828,7 @@
       </c>
       <c r="F26" s="33"/>
     </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A27" s="46" t="s">
         <v>146</v>
       </c>
@@ -3830,7 +3846,7 @@
       </c>
       <c r="F27" s="33"/>
     </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A28" s="39" t="s">
         <v>102</v>
       </c>
@@ -3848,7 +3864,7 @@
       </c>
       <c r="F28" s="33"/>
     </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A29" s="28" t="s">
         <v>75</v>
       </c>
@@ -3866,7 +3882,7 @@
       </c>
       <c r="F29" s="56"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
       <c r="A30" s="70" t="s">
         <v>181</v>
       </c>
@@ -3874,17 +3890,17 @@
         <v>43124</v>
       </c>
       <c r="C30" s="23">
-        <v>43124</v>
+        <v>43138</v>
       </c>
       <c r="D30" s="24">
         <v>0</v>
       </c>
       <c r="E30" s="23">
-        <v>43132</v>
+        <v>43139</v>
       </c>
       <c r="F30" s="61"/>
     </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A31" s="26" t="s">
         <v>67</v>
       </c>
@@ -3904,7 +3920,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A32" s="29" t="s">
         <v>77</v>
       </c>
@@ -3924,7 +3940,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A33" s="70" t="s">
         <v>177</v>
       </c>
@@ -3935,7 +3951,7 @@
         <v>43125</v>
       </c>
       <c r="D33" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E33" s="23">
         <v>43132</v>
@@ -3944,7 +3960,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A34" s="70" t="s">
         <v>175</v>
       </c>
@@ -3962,7 +3978,7 @@
       </c>
       <c r="F34" s="61"/>
     </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A35" s="69" t="s">
         <v>174</v>
       </c>
@@ -3980,7 +3996,7 @@
       </c>
       <c r="F35" s="61"/>
     </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A36" s="50" t="s">
         <v>153</v>
       </c>
@@ -3998,7 +4014,7 @@
       </c>
       <c r="F36" s="61"/>
     </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A37" s="55" t="s">
         <v>162</v>
       </c>
@@ -4016,7 +4032,7 @@
       </c>
       <c r="F37" s="61"/>
     </row>
-    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A38" s="40" t="s">
         <v>103</v>
       </c>
@@ -4036,7 +4052,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A39" s="67" t="s">
         <v>167</v>
       </c>
@@ -4054,7 +4070,7 @@
       </c>
       <c r="F39" s="61"/>
     </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A40" s="47" t="s">
         <v>147</v>
       </c>
@@ -4072,7 +4088,7 @@
       </c>
       <c r="F40" s="33"/>
     </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A41" s="68" t="s">
         <v>169</v>
       </c>
@@ -4089,13 +4105,13 @@
         <v>43125</v>
       </c>
     </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A42" s="48" t="s">
         <v>148</v>
       </c>
       <c r="B42" s="23">
         <f ca="1">TODAY()</f>
-        <v>43131</v>
+        <v>43132</v>
       </c>
       <c r="C42" s="23">
         <v>43118</v>
@@ -4108,7 +4124,7 @@
       </c>
       <c r="F42" s="33"/>
     </row>
-    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A43" s="67" t="s">
         <v>170</v>
       </c>
@@ -4128,13 +4144,13 @@
         <v>171</v>
       </c>
     </row>
-    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A44" s="49" t="s">
         <v>150</v>
       </c>
       <c r="B44" s="23">
         <f ca="1">TODAY()</f>
-        <v>43131</v>
+        <v>43132</v>
       </c>
       <c r="C44" s="23">
         <v>43118</v>
@@ -4147,13 +4163,13 @@
       </c>
       <c r="F44" s="33"/>
     </row>
-    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A45" s="49" t="s">
         <v>151</v>
       </c>
       <c r="B45" s="23">
         <f ca="1">TODAY()</f>
-        <v>43131</v>
+        <v>43132</v>
       </c>
       <c r="C45" s="23">
         <v>43118</v>
@@ -4166,7 +4182,7 @@
       </c>
       <c r="F45" s="33"/>
     </row>
-    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A46" s="69" t="s">
         <v>172</v>
       </c>
@@ -4184,13 +4200,13 @@
       </c>
       <c r="F46" s="61"/>
     </row>
-    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A47" s="50" t="s">
         <v>154</v>
       </c>
       <c r="B47" s="23">
         <f ca="1">TODAY()</f>
-        <v>43131</v>
+        <v>43132</v>
       </c>
       <c r="C47" s="23"/>
       <c r="D47" s="24">
@@ -4201,7 +4217,7 @@
       </c>
       <c r="F47" s="33"/>
     </row>
-    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A48" s="50" t="s">
         <v>155</v>
       </c>
@@ -4215,7 +4231,7 @@
       </c>
       <c r="F48" s="33"/>
     </row>
-    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A49" s="51" t="s">
         <v>156</v>
       </c>
@@ -4233,7 +4249,7 @@
       </c>
       <c r="F49" s="33"/>
     </row>
-    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A50" s="52" t="s">
         <v>157</v>
       </c>
@@ -4253,7 +4269,7 @@
         <v>0.60416666666666663</v>
       </c>
     </row>
-    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A51" s="53" t="s">
         <v>158</v>
       </c>
@@ -4271,7 +4287,7 @@
       </c>
       <c r="F51" s="61"/>
     </row>
-    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A52" s="53" t="s">
         <v>159</v>
       </c>
@@ -4287,7 +4303,7 @@
       <c r="E52" s="23"/>
       <c r="F52" s="33"/>
     </row>
-    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A53" s="54" t="s">
         <v>160</v>
       </c>
@@ -4303,7 +4319,7 @@
       <c r="E53" s="23"/>
       <c r="F53" s="33"/>
     </row>
-    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A54" s="54" t="s">
         <v>161</v>
       </c>
@@ -4319,7 +4335,7 @@
       <c r="E54" s="23"/>
       <c r="F54" s="33"/>
     </row>
-    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A55" s="49" t="s">
         <v>149</v>
       </c>
@@ -4339,7 +4355,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A56" s="55" t="s">
         <v>163</v>
       </c>
@@ -4357,7 +4373,7 @@
       </c>
       <c r="F56" s="61"/>
     </row>
-    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A57" s="65" t="s">
         <v>165</v>
       </c>
@@ -4375,7 +4391,7 @@
       </c>
       <c r="F57" s="61"/>
     </row>
-    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A58" s="66" t="s">
         <v>166</v>
       </c>
@@ -4393,7 +4409,7 @@
       </c>
       <c r="F58" s="61"/>
     </row>
-    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A59" s="70" t="s">
         <v>183</v>
       </c>
@@ -4411,7 +4427,7 @@
       </c>
       <c r="F59" s="61"/>
     </row>
-    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A60" s="21" t="s">
         <v>59</v>
       </c>
@@ -4431,7 +4447,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A61" s="70" t="s">
         <v>179</v>
       </c>
@@ -4451,7 +4467,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A62" s="70" t="s">
         <v>180</v>
       </c>
@@ -4469,7 +4485,7 @@
       </c>
       <c r="F62" s="61"/>
     </row>
-    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A63" s="69" t="s">
         <v>173</v>
       </c>
@@ -4487,7 +4503,7 @@
       </c>
       <c r="F63" s="61"/>
     </row>
-    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A64" s="21" t="s">
         <v>64</v>
       </c>
@@ -4507,7 +4523,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A65" s="70" t="s">
         <v>182</v>
       </c>
@@ -4518,14 +4534,14 @@
         <v>43125</v>
       </c>
       <c r="D65" s="24">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E65" s="23">
         <v>43132</v>
       </c>
       <c r="F65" s="61"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A66" s="21" t="s">
         <v>61</v>
       </c>
@@ -4536,7 +4552,7 @@
         <v>43126</v>
       </c>
       <c r="D66" s="24">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E66" s="23">
         <v>43132</v>
@@ -4545,45 +4561,47 @@
         <v>88</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="73" t="s">
+    <row r="67" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A67" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B67" s="23">
+        <v>43124</v>
+      </c>
+      <c r="C67" s="23">
+        <v>43138</v>
+      </c>
+      <c r="D67" s="24">
+        <v>0.25</v>
+      </c>
+      <c r="E67" s="23">
+        <v>43139</v>
+      </c>
+      <c r="F67" s="57" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A68" s="73" t="s">
         <v>184</v>
       </c>
-      <c r="B67" s="23">
+      <c r="B68" s="23">
         <v>43125</v>
       </c>
-      <c r="C67" s="23">
-        <v>43126</v>
-      </c>
-      <c r="D67" s="24">
-        <v>0</v>
-      </c>
-      <c r="E67" s="23">
-        <v>43132</v>
-      </c>
-      <c r="F67" s="74" t="s">
+      <c r="C68" s="23">
+        <v>43136</v>
+      </c>
+      <c r="D68" s="24">
+        <v>0</v>
+      </c>
+      <c r="E68" s="23">
+        <v>43139</v>
+      </c>
+      <c r="F68" s="74" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="67" t="s">
-        <v>168</v>
-      </c>
-      <c r="B68" s="23">
-        <v>43119</v>
-      </c>
-      <c r="C68" s="23">
-        <v>43129</v>
-      </c>
-      <c r="D68" s="24">
-        <v>0.75</v>
-      </c>
-      <c r="E68" s="23">
-        <v>43132</v>
-      </c>
-      <c r="F68" s="61"/>
-    </row>
-    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A69" s="40" t="s">
         <v>104</v>
       </c>
@@ -4603,47 +4621,45 @@
         <v>178</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="21" t="s">
+    <row r="70" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A70" s="67" t="s">
+        <v>168</v>
+      </c>
+      <c r="B70" s="23">
+        <v>43119</v>
+      </c>
+      <c r="C70" s="23">
+        <v>43136</v>
+      </c>
+      <c r="D70" s="24">
+        <v>0.75</v>
+      </c>
+      <c r="E70" s="23">
+        <v>43139</v>
+      </c>
+      <c r="F70" s="61"/>
+    </row>
+    <row r="71" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A71" s="21" t="s">
         <v>62</v>
-      </c>
-      <c r="B70" s="23">
-        <v>43124</v>
-      </c>
-      <c r="C70" s="23">
-        <v>43130</v>
-      </c>
-      <c r="D70" s="24">
-        <v>0.5</v>
-      </c>
-      <c r="E70" s="23">
-        <v>43132</v>
-      </c>
-      <c r="F70" s="59" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="21" t="s">
-        <v>58</v>
       </c>
       <c r="B71" s="23">
         <v>43124</v>
       </c>
       <c r="C71" s="23">
-        <v>43130</v>
+        <v>43136</v>
       </c>
       <c r="D71" s="24">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="E71" s="23">
-        <v>43132</v>
-      </c>
-      <c r="F71" s="57" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+        <v>43139</v>
+      </c>
+      <c r="F71" s="59" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A72" s="73" t="s">
         <v>186</v>
       </c>
@@ -4661,7 +4677,7 @@
       </c>
       <c r="F72" s="61"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A73" s="75" t="s">
         <v>187</v>
       </c>
@@ -4669,10 +4685,10 @@
         <v>43129</v>
       </c>
       <c r="C73" s="23">
-        <v>43130</v>
+        <v>43133</v>
       </c>
       <c r="D73" s="24">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E73" s="23">
         <v>43132</v>
@@ -4681,8 +4697,8 @@
         <v>188</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="93" t="s">
+    <row r="74" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A74" s="77" t="s">
         <v>189</v>
       </c>
       <c r="B74" s="23">
@@ -4699,8 +4715,8 @@
       </c>
       <c r="F74" s="61"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="93" t="s">
+    <row r="75" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A75" s="77" t="s">
         <v>190</v>
       </c>
       <c r="B75" s="23">
@@ -4710,46 +4726,86 @@
         <v>43131</v>
       </c>
       <c r="D75" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E75" s="23">
         <v>43132</v>
       </c>
       <c r="F75" s="61"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="50"/>
-      <c r="B76" s="23"/>
-      <c r="C76" s="23"/>
-      <c r="D76" s="24"/>
-      <c r="E76" s="23"/>
+    <row r="76" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A76" s="77" t="s">
+        <v>191</v>
+      </c>
+      <c r="B76" s="23">
+        <v>43129</v>
+      </c>
+      <c r="C76" s="23">
+        <v>43137</v>
+      </c>
+      <c r="D76" s="24">
+        <v>1</v>
+      </c>
+      <c r="E76" s="23">
+        <v>43139</v>
+      </c>
       <c r="F76" s="61"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="50"/>
-      <c r="B77" s="23"/>
-      <c r="C77" s="23"/>
-      <c r="D77" s="24"/>
-      <c r="E77" s="23"/>
+    <row r="77" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A77" s="94" t="s">
+        <v>96</v>
+      </c>
+      <c r="B77" s="23">
+        <v>43132</v>
+      </c>
+      <c r="C77" s="23">
+        <v>43133</v>
+      </c>
+      <c r="D77" s="24">
+        <v>0</v>
+      </c>
+      <c r="E77" s="23">
+        <v>43139</v>
+      </c>
       <c r="F77" s="61"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="50"/>
-      <c r="B78" s="23"/>
-      <c r="C78" s="23"/>
-      <c r="D78" s="24"/>
-      <c r="E78" s="23"/>
+    <row r="78" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A78" s="94" t="s">
+        <v>192</v>
+      </c>
+      <c r="B78" s="23">
+        <v>43132</v>
+      </c>
+      <c r="C78" s="23">
+        <v>43133</v>
+      </c>
+      <c r="D78" s="24">
+        <v>0</v>
+      </c>
+      <c r="E78" s="23">
+        <v>43139</v>
+      </c>
       <c r="F78" s="61"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="50"/>
-      <c r="B79" s="23"/>
-      <c r="C79" s="23"/>
-      <c r="D79" s="24"/>
-      <c r="E79" s="23"/>
+    <row r="79" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A79" s="94" t="s">
+        <v>193</v>
+      </c>
+      <c r="B79" s="23">
+        <v>43132</v>
+      </c>
+      <c r="C79" s="23">
+        <v>43136</v>
+      </c>
+      <c r="D79" s="24">
+        <v>0</v>
+      </c>
+      <c r="E79" s="23">
+        <v>43139</v>
+      </c>
       <c r="F79" s="61"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
       <c r="A80" s="50"/>
       <c r="B80" s="23"/>
       <c r="C80" s="23"/>
@@ -4757,17 +4813,17 @@
       <c r="E80" s="23"/>
       <c r="F80" s="61"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:6" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B81" s="23"/>
       <c r="C81" s="23"/>
       <c r="D81" s="24"/>
       <c r="E81" s="23"/>
       <c r="F81" s="59"/>
     </row>
-    <row r="82" spans="2:6" hidden="1" x14ac:dyDescent="0.3"/>
-    <row r="83" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="84" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="85" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="82" spans="2:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="83" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="84" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="85" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <conditionalFormatting sqref="D2:D81">
     <cfRule type="iconSet" priority="16">
@@ -4791,17 +4847,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.6" zeroHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="9" width="4.77734375" style="42" customWidth="1"/>
-    <col min="10" max="10" width="12.109375" style="42" customWidth="1"/>
-    <col min="11" max="11" width="12.5546875" style="42" customWidth="1"/>
-    <col min="12" max="12" width="13.88671875" style="42" customWidth="1"/>
-    <col min="13" max="17" width="11.109375" style="42" customWidth="1"/>
-    <col min="18" max="16384" width="8.88671875" hidden="1"/>
+    <col min="1" max="9" width="4.78515625" style="42" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" style="42" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" style="42" customWidth="1"/>
+    <col min="12" max="12" width="13.85546875" style="42" customWidth="1"/>
+    <col min="13" max="17" width="11.140625" style="42" customWidth="1"/>
+    <col min="18" max="16384" width="8.85546875" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="72.599999999999994" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="74.599999999999994" x14ac:dyDescent="0.4">
       <c r="A1" s="41" t="s">
         <v>110</v>
       </c>
@@ -4854,7 +4910,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A2" s="43">
         <v>1</v>
       </c>
@@ -4883,7 +4939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A3" s="43">
         <v>2</v>
       </c>
@@ -4912,7 +4968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A4" s="43">
         <v>3</v>
       </c>
@@ -4941,7 +4997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" s="43">
         <v>4</v>
       </c>
@@ -4970,7 +5026,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A6" s="43">
         <v>5</v>
       </c>
@@ -4999,7 +5055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A7" s="43">
         <v>6</v>
       </c>
@@ -5028,7 +5084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A8" s="43">
         <v>7</v>
       </c>
@@ -5057,7 +5113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A9" s="43">
         <v>8</v>
       </c>
@@ -5086,7 +5142,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A10" s="43">
         <v>9</v>
       </c>
@@ -5115,7 +5171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A11" s="43">
         <v>10</v>
       </c>
@@ -5144,7 +5200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A12" s="43">
         <v>11</v>
       </c>
@@ -5173,7 +5229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A13" s="43">
         <v>12</v>
       </c>
@@ -5202,7 +5258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A14" s="43">
         <v>13</v>
       </c>
@@ -5231,7 +5287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A15" s="43">
         <v>14</v>
       </c>
@@ -5260,7 +5316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A16" s="43">
         <v>15</v>
       </c>
@@ -5289,7 +5345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A17" s="43">
         <v>16</v>
       </c>
@@ -5318,7 +5374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A18" s="43">
         <v>17</v>
       </c>
@@ -5347,7 +5403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A19" s="43">
         <v>18</v>
       </c>
@@ -5376,7 +5432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A20" s="43">
         <v>19</v>
       </c>
@@ -5405,7 +5461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A21" s="43">
         <v>20</v>
       </c>
@@ -5434,7 +5490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A22" s="43">
         <v>21</v>
       </c>
@@ -5463,7 +5519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A23" s="43">
         <v>22</v>
       </c>
@@ -5492,7 +5548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A24" s="43">
         <v>23</v>
       </c>
@@ -5521,7 +5577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A25" s="43">
         <v>24</v>
       </c>
@@ -5550,7 +5606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A26" s="43">
         <v>25</v>
       </c>
@@ -5579,7 +5635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A27" s="43">
         <v>26</v>
       </c>
@@ -5608,7 +5664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A28" s="43">
         <v>27</v>
       </c>
@@ -5637,7 +5693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A29" s="43">
         <v>28</v>
       </c>
@@ -5666,7 +5722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A30" s="43">
         <v>29</v>
       </c>
@@ -5695,7 +5751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A31" s="43">
         <v>30</v>
       </c>
@@ -5724,7 +5780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A32" s="43">
         <v>31</v>
       </c>
@@ -5753,7 +5809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A33" s="43">
         <v>32</v>
       </c>
@@ -5782,7 +5838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -5795,16 +5851,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.6" zeroHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.77734375" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" customWidth="1"/>
-    <col min="4" max="4" width="53.5546875" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" hidden="1"/>
+    <col min="1" max="1" width="11.78515625" customWidth="1"/>
+    <col min="2" max="2" width="12.640625" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
+    <col min="4" max="4" width="53.5703125" customWidth="1"/>
+    <col min="5" max="16384" width="8.85546875" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>124</v>
       </c>
@@ -5818,7 +5874,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>126</v>
       </c>
@@ -5832,7 +5888,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>128</v>
       </c>
@@ -5846,7 +5902,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>130</v>
       </c>
@@ -5860,7 +5916,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>137</v>
       </c>
@@ -5871,7 +5927,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>105</v>
       </c>
@@ -5883,7 +5939,7 @@
       </c>
       <c r="D6" s="45"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>140</v>
       </c>
@@ -5895,19 +5951,19 @@
       </c>
       <c r="D7" s="45"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>141</v>
       </c>
       <c r="D8" s="45"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>142</v>
       </c>
       <c r="D9" s="45"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>143</v>
       </c>
@@ -5916,43 +5972,43 @@
       </c>
       <c r="D10" s="45"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="D11" s="45"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="D12" s="45"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="D13" s="45"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="D14" s="45"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="D15" s="45"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="D16" s="45"/>
     </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.4">
       <c r="D17" s="45"/>
     </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.4">
       <c r="D18" s="45"/>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.4">
       <c r="D19" s="45"/>
     </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="4:4" x14ac:dyDescent="0.4">
       <c r="D20" s="45"/>
     </row>
-    <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="D21" s="45"/>
     </row>
-    <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="D22" s="45"/>
     </row>
-    <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.4">
       <c r="D23" s="45"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
First clone to hummingbird
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="8649" windowHeight="7646" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="8652" windowHeight="7644" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Project Planner" sheetId="1" r:id="rId1"/>
@@ -30,11 +30,12 @@
     <definedName name="TitleRegion..BO60">'Project Planner'!$B$3:$B$4</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="222">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -738,13 +739,40 @@
     <t>Only necessary for measure A</t>
   </si>
   <si>
-    <t>Not run as often as find_phistop</t>
-  </si>
-  <si>
     <t>Check NSinceStoch and numStochEpochs</t>
   </si>
   <si>
     <t>Allow potential minimum to be slightly negative</t>
+  </si>
+  <si>
+    <t>Impose lower bound on N for stochastic epoch</t>
+  </si>
+  <si>
+    <t>Fix stochastic bug</t>
+  </si>
+  <si>
+    <t>phistart is eternal, but phistart+delta is not - why? Measure A</t>
+  </si>
+  <si>
+    <t>Not run as often as find_phistop; back burner</t>
+  </si>
+  <si>
+    <t>Replaced with step search</t>
+  </si>
+  <si>
+    <t>Bad step size</t>
+  </si>
+  <si>
+    <t>Modify find_phistop MEX code</t>
+  </si>
+  <si>
+    <t>Write script to read output structure from file</t>
+  </si>
+  <si>
+    <t>Ask about second derivative check for stochastic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use thin wall for parke </t>
   </si>
 </sst>
 </file>
@@ -755,13 +783,20 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="59" x14ac:knownFonts="1">
+  <fonts count="60" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1313,98 +1348,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="54" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="55" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="47" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="48" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="54" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="57" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="58" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="56" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="56" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="56" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="56" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="56" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="54" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="55" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="47" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="48" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="54" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="50" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="51" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="57" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="58" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -1422,25 +1457,26 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="54" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="55" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="54" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="55" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="44" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="45" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -1456,23 +1492,23 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -1481,110 +1517,117 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="18" fontId="35" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="36" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -1599,7 +1642,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
   </cellXfs>
   <cellStyles count="20">
     <cellStyle name="% complete" xfId="16"/>
@@ -2134,19 +2176,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F100" totalsRowShown="0">
-  <autoFilter ref="A1:F100">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F108" totalsRowShown="0">
+  <autoFilter ref="A1:F108">
     <filterColumn colId="3">
       <filters blank="1">
-        <filter val="0"/>
         <filter val="0.25"/>
-        <filter val="0.5"/>
-        <filter val="0.75"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState ref="A30:F100">
-    <sortCondition descending="1" ref="C1:C100"/>
+  <sortState ref="A30:F108">
+    <sortCondition descending="1" ref="C1:C108"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" name="Task"/>
@@ -2431,19 +2470,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BO31"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.640625" customWidth="1"/>
-    <col min="2" max="2" width="15.640625" style="2" customWidth="1"/>
-    <col min="3" max="6" width="11.640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.640625" style="4" customWidth="1"/>
-    <col min="8" max="27" width="3.5703125" style="1" customWidth="1"/>
-    <col min="28" max="48" width="3.5703125" customWidth="1"/>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="2" customWidth="1"/>
+    <col min="3" max="6" width="11.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="4" customWidth="1"/>
+    <col min="8" max="27" width="3.5546875" style="1" customWidth="1"/>
+    <col min="28" max="48" width="3.5546875" customWidth="1"/>
     <col min="49" max="67" width="0" hidden="1" customWidth="1"/>
-    <col min="68" max="16384" width="2.78515625" hidden="1"/>
+    <col min="68" max="16384" width="2.77734375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.4">
+    <row r="1" spans="2:67" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.05">
       <c r="B1" s="11" t="s">
         <v>40</v>
       </c>
@@ -2453,14 +2492,14 @@
       <c r="F1" s="10"/>
       <c r="G1" s="10"/>
     </row>
-    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="91" t="s">
+    <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
@@ -2468,66 +2507,66 @@
         <v>8</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="97" t="s">
+      <c r="K2" s="101" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="98"/>
-      <c r="M2" s="98"/>
-      <c r="N2" s="98"/>
-      <c r="O2" s="99"/>
+      <c r="L2" s="102"/>
+      <c r="M2" s="102"/>
+      <c r="N2" s="102"/>
+      <c r="O2" s="103"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="97" t="s">
+      <c r="Q2" s="101" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="100"/>
-      <c r="S2" s="100"/>
-      <c r="T2" s="99"/>
+      <c r="R2" s="104"/>
+      <c r="S2" s="104"/>
+      <c r="T2" s="103"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="89" t="s">
+      <c r="V2" s="93" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="90"/>
-      <c r="X2" s="90"/>
-      <c r="Y2" s="101"/>
+      <c r="W2" s="94"/>
+      <c r="X2" s="94"/>
+      <c r="Y2" s="105"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="102" t="s">
+      <c r="AA2" s="106" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="103"/>
-      <c r="AC2" s="103"/>
-      <c r="AD2" s="103"/>
-      <c r="AE2" s="103"/>
-      <c r="AF2" s="103"/>
-      <c r="AG2" s="104"/>
+      <c r="AB2" s="107"/>
+      <c r="AC2" s="107"/>
+      <c r="AD2" s="107"/>
+      <c r="AE2" s="107"/>
+      <c r="AF2" s="107"/>
+      <c r="AG2" s="108"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="89" t="s">
+      <c r="AI2" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="90"/>
-      <c r="AK2" s="90"/>
-      <c r="AL2" s="90"/>
-      <c r="AM2" s="90"/>
-      <c r="AN2" s="90"/>
-      <c r="AO2" s="90"/>
-      <c r="AP2" s="90"/>
-    </row>
-    <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="92" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="94" t="s">
+      <c r="AJ2" s="94"/>
+      <c r="AK2" s="94"/>
+      <c r="AL2" s="94"/>
+      <c r="AM2" s="94"/>
+      <c r="AN2" s="94"/>
+      <c r="AO2" s="94"/>
+      <c r="AP2" s="94"/>
+    </row>
+    <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="96" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="98" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="94" t="s">
+      <c r="D3" s="98" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="94" t="s">
+      <c r="E3" s="98" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="94" t="s">
+      <c r="F3" s="98" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="96" t="s">
+      <c r="G3" s="100" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -2655,13 +2694,13 @@
       </c>
       <c r="AW3" s="18"/>
     </row>
-    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="93"/>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
+    <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="97"/>
+      <c r="C4" s="99"/>
+      <c r="D4" s="99"/>
+      <c r="E4" s="99"/>
+      <c r="F4" s="99"/>
+      <c r="G4" s="99"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -2805,7 +2844,7 @@
       <c r="BN4" s="3"/>
       <c r="BO4" s="3"/>
     </row>
-    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="6" t="s">
         <v>38</v>
       </c>
@@ -2828,7 +2867,7 @@
       <c r="X5" s="19"/>
       <c r="Y5" s="19"/>
     </row>
-    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>35</v>
       </c>
@@ -2851,7 +2890,7 @@
       <c r="X6" s="19"/>
       <c r="Y6" s="19"/>
     </row>
-    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="6" t="s">
         <v>29</v>
       </c>
@@ -2874,7 +2913,7 @@
       <c r="X7" s="19"/>
       <c r="Y7" s="19"/>
     </row>
-    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>32</v>
       </c>
@@ -2895,7 +2934,7 @@
       <c r="X8" s="19"/>
       <c r="Y8" s="19"/>
     </row>
-    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="6" t="s">
         <v>33</v>
       </c>
@@ -2916,7 +2955,7 @@
       <c r="X9" s="19"/>
       <c r="Y9" s="19"/>
     </row>
-    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="6" t="s">
         <v>34</v>
       </c>
@@ -2937,7 +2976,7 @@
       <c r="X10" s="19"/>
       <c r="Y10" s="19"/>
     </row>
-    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="6" t="s">
         <v>39</v>
       </c>
@@ -2958,7 +2997,7 @@
       <c r="X11" s="19"/>
       <c r="Y11" s="19"/>
     </row>
-    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
@@ -2981,7 +3020,7 @@
       <c r="X12" s="19"/>
       <c r="Y12" s="19"/>
     </row>
-    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="6" t="s">
         <v>31</v>
       </c>
@@ -3002,7 +3041,7 @@
       <c r="X13" s="19"/>
       <c r="Y13" s="19"/>
     </row>
-    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>36</v>
       </c>
@@ -3023,7 +3062,7 @@
       <c r="X14" s="19"/>
       <c r="Y14" s="19"/>
     </row>
-    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:67" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="6" t="s">
         <v>37</v>
       </c>
@@ -3044,7 +3083,7 @@
       <c r="X15" s="19"/>
       <c r="Y15" s="19"/>
     </row>
-    <row r="16" spans="2:67" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:67" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="6" t="s">
         <v>1</v>
       </c>
@@ -3064,7 +3103,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="6" t="s">
         <v>2</v>
       </c>
@@ -3084,7 +3123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="6" t="s">
         <v>3</v>
       </c>
@@ -3104,7 +3143,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="6" t="s">
         <v>4</v>
       </c>
@@ -3124,7 +3163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="6" t="s">
         <v>5</v>
       </c>
@@ -3144,7 +3183,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="6" t="s">
         <v>6</v>
       </c>
@@ -3164,7 +3203,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="6" t="s">
         <v>7</v>
       </c>
@@ -3184,7 +3223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="6" t="s">
         <v>8</v>
       </c>
@@ -3204,7 +3243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="6" t="s">
         <v>9</v>
       </c>
@@ -3224,7 +3263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="6" t="s">
         <v>10</v>
       </c>
@@ -3244,7 +3283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="6" t="s">
         <v>11</v>
       </c>
@@ -3264,7 +3303,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="6" t="s">
         <v>12</v>
       </c>
@@ -3284,7 +3323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="6" t="s">
         <v>13</v>
       </c>
@@ -3304,7 +3343,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="6" t="s">
         <v>14</v>
       </c>
@@ -3324,7 +3363,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="6" t="s">
         <v>15</v>
       </c>
@@ -3344,7 +3383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="6" t="s">
         <v>16</v>
       </c>
@@ -3446,20 +3485,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G104"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:G112"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="51.2109375" style="21" customWidth="1"/>
-    <col min="2" max="2" width="9.78515625" style="21" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" style="21" customWidth="1"/>
-    <col min="4" max="4" width="5.2109375" style="21" customWidth="1"/>
-    <col min="5" max="5" width="9.78515625" style="21" customWidth="1"/>
-    <col min="6" max="6" width="70.35546875" style="21" customWidth="1"/>
+    <col min="1" max="1" width="51.21875" style="21" customWidth="1"/>
+    <col min="2" max="2" width="9.77734375" style="21" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" style="21" customWidth="1"/>
+    <col min="4" max="4" width="5.21875" style="21" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" style="21" customWidth="1"/>
+    <col min="6" max="6" width="70.33203125" style="21" customWidth="1"/>
     <col min="7" max="7" width="0" style="21" hidden="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.85546875" style="21" hidden="1"/>
+    <col min="8" max="16384" width="8.88671875" style="21" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
         <v>41</v>
       </c>
@@ -3479,7 +3518,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>80</v>
       </c>
@@ -3499,7 +3538,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
         <v>66</v>
       </c>
@@ -3519,7 +3558,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>47</v>
       </c>
@@ -3536,7 +3575,7 @@
         <v>42984</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
         <v>48</v>
       </c>
@@ -3556,7 +3595,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
         <v>50</v>
       </c>
@@ -3573,7 +3612,7 @@
         <v>42984</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
         <v>52</v>
       </c>
@@ -3593,7 +3632,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="21" t="s">
         <v>51</v>
       </c>
@@ -3610,7 +3649,7 @@
         <v>42990</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
         <v>55</v>
       </c>
@@ -3630,7 +3669,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
         <v>81</v>
       </c>
@@ -3650,7 +3689,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
         <v>60</v>
       </c>
@@ -3670,7 +3709,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
         <v>56</v>
       </c>
@@ -3690,7 +3729,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="27" t="s">
         <v>73</v>
       </c>
@@ -3710,7 +3749,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="31" t="s">
         <v>82</v>
       </c>
@@ -3727,7 +3766,7 @@
         <v>43006</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
         <v>53</v>
       </c>
@@ -3747,7 +3786,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>54</v>
       </c>
@@ -3767,7 +3806,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
         <v>84</v>
       </c>
@@ -3784,7 +3823,7 @@
         <v>43027</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="33" t="s">
         <v>89</v>
       </c>
@@ -3802,7 +3841,7 @@
       </c>
       <c r="F18" s="33"/>
     </row>
-    <row r="19" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33" t="s">
         <v>90</v>
       </c>
@@ -3822,7 +3861,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="35" t="s">
         <v>95</v>
       </c>
@@ -3840,7 +3879,7 @@
       </c>
       <c r="F20" s="33"/>
     </row>
-    <row r="21" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="35" t="s">
         <v>94</v>
       </c>
@@ -3858,7 +3897,7 @@
       </c>
       <c r="F21" s="33"/>
     </row>
-    <row r="22" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="34" t="s">
         <v>92</v>
       </c>
@@ -3878,7 +3917,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="36" t="s">
         <v>98</v>
       </c>
@@ -3898,7 +3937,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="38" t="s">
         <v>100</v>
       </c>
@@ -3918,7 +3957,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="36" t="s">
         <v>97</v>
       </c>
@@ -3936,7 +3975,7 @@
       </c>
       <c r="F25" s="33"/>
     </row>
-    <row r="26" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="35" t="s">
         <v>96</v>
       </c>
@@ -3954,7 +3993,7 @@
       </c>
       <c r="F26" s="33"/>
     </row>
-    <row r="27" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="46" t="s">
         <v>146</v>
       </c>
@@ -3972,7 +4011,7 @@
       </c>
       <c r="F27" s="33"/>
     </row>
-    <row r="28" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="39" t="s">
         <v>102</v>
       </c>
@@ -3990,7 +4029,7 @@
       </c>
       <c r="F28" s="33"/>
     </row>
-    <row r="29" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="28" t="s">
         <v>75</v>
       </c>
@@ -4008,7 +4047,7 @@
       </c>
       <c r="F29" s="56"/>
     </row>
-    <row r="30" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="70" t="s">
         <v>181</v>
       </c>
@@ -4019,14 +4058,14 @@
         <v>43138</v>
       </c>
       <c r="D30" s="24">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E30" s="23">
         <v>43139</v>
       </c>
       <c r="F30" s="61"/>
     </row>
-    <row r="31" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="26" t="s">
         <v>67</v>
       </c>
@@ -4046,7 +4085,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="29" t="s">
         <v>77</v>
       </c>
@@ -4066,7 +4105,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="70" t="s">
         <v>177</v>
       </c>
@@ -4086,7 +4125,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="70" t="s">
         <v>175</v>
       </c>
@@ -4104,7 +4143,7 @@
       </c>
       <c r="F34" s="61"/>
     </row>
-    <row r="35" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="69" t="s">
         <v>174</v>
       </c>
@@ -4122,7 +4161,7 @@
       </c>
       <c r="F35" s="61"/>
     </row>
-    <row r="36" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="50" t="s">
         <v>153</v>
       </c>
@@ -4140,7 +4179,7 @@
       </c>
       <c r="F36" s="61"/>
     </row>
-    <row r="37" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="55" t="s">
         <v>162</v>
       </c>
@@ -4158,7 +4197,7 @@
       </c>
       <c r="F37" s="61"/>
     </row>
-    <row r="38" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="40" t="s">
         <v>103</v>
       </c>
@@ -4178,7 +4217,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="67" t="s">
         <v>167</v>
       </c>
@@ -4196,7 +4235,7 @@
       </c>
       <c r="F39" s="61"/>
     </row>
-    <row r="40" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="47" t="s">
         <v>147</v>
       </c>
@@ -4214,7 +4253,7 @@
       </c>
       <c r="F40" s="33"/>
     </row>
-    <row r="41" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="68" t="s">
         <v>169</v>
       </c>
@@ -4231,13 +4270,13 @@
         <v>43125</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="48" t="s">
         <v>148</v>
       </c>
       <c r="B42" s="23">
         <f ca="1">TODAY()</f>
-        <v>43137</v>
+        <v>43138</v>
       </c>
       <c r="C42" s="23">
         <v>43118</v>
@@ -4250,7 +4289,7 @@
       </c>
       <c r="F42" s="33"/>
     </row>
-    <row r="43" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="67" t="s">
         <v>170</v>
       </c>
@@ -4270,13 +4309,13 @@
         <v>171</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="49" t="s">
         <v>150</v>
       </c>
       <c r="B44" s="23">
         <f ca="1">TODAY()</f>
-        <v>43137</v>
+        <v>43138</v>
       </c>
       <c r="C44" s="23">
         <v>43118</v>
@@ -4289,13 +4328,13 @@
       </c>
       <c r="F44" s="33"/>
     </row>
-    <row r="45" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="49" t="s">
         <v>151</v>
       </c>
       <c r="B45" s="23">
         <f ca="1">TODAY()</f>
-        <v>43137</v>
+        <v>43138</v>
       </c>
       <c r="C45" s="23">
         <v>43118</v>
@@ -4308,7 +4347,7 @@
       </c>
       <c r="F45" s="33"/>
     </row>
-    <row r="46" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="69" t="s">
         <v>172</v>
       </c>
@@ -4326,13 +4365,13 @@
       </c>
       <c r="F46" s="61"/>
     </row>
-    <row r="47" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="50" t="s">
         <v>154</v>
       </c>
       <c r="B47" s="23">
         <f ca="1">TODAY()</f>
-        <v>43137</v>
+        <v>43138</v>
       </c>
       <c r="C47" s="23"/>
       <c r="D47" s="24">
@@ -4343,7 +4382,7 @@
       </c>
       <c r="F47" s="33"/>
     </row>
-    <row r="48" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="50" t="s">
         <v>155</v>
       </c>
@@ -4357,7 +4396,7 @@
       </c>
       <c r="F48" s="33"/>
     </row>
-    <row r="49" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="51" t="s">
         <v>156</v>
       </c>
@@ -4375,7 +4414,7 @@
       </c>
       <c r="F49" s="33"/>
     </row>
-    <row r="50" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="52" t="s">
         <v>157</v>
       </c>
@@ -4395,7 +4434,7 @@
         <v>0.60416666666666663</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="53" t="s">
         <v>158</v>
       </c>
@@ -4413,7 +4452,7 @@
       </c>
       <c r="F51" s="61"/>
     </row>
-    <row r="52" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="53" t="s">
         <v>159</v>
       </c>
@@ -4426,10 +4465,12 @@
       <c r="D52" s="24">
         <v>1</v>
       </c>
-      <c r="E52" s="23"/>
+      <c r="E52" s="23">
+        <v>43118</v>
+      </c>
       <c r="F52" s="33"/>
     </row>
-    <row r="53" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="54" t="s">
         <v>160</v>
       </c>
@@ -4442,10 +4483,12 @@
       <c r="D53" s="24">
         <v>1</v>
       </c>
-      <c r="E53" s="23"/>
+      <c r="E53" s="23">
+        <v>43118</v>
+      </c>
       <c r="F53" s="33"/>
     </row>
-    <row r="54" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="54" t="s">
         <v>161</v>
       </c>
@@ -4458,10 +4501,12 @@
       <c r="D54" s="24">
         <v>1</v>
       </c>
-      <c r="E54" s="23"/>
+      <c r="E54" s="23">
+        <v>43118</v>
+      </c>
       <c r="F54" s="33"/>
     </row>
-    <row r="55" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="49" t="s">
         <v>149</v>
       </c>
@@ -4481,7 +4526,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="55" t="s">
         <v>163</v>
       </c>
@@ -4499,7 +4544,7 @@
       </c>
       <c r="F56" s="61"/>
     </row>
-    <row r="57" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="65" t="s">
         <v>165</v>
       </c>
@@ -4517,7 +4562,7 @@
       </c>
       <c r="F57" s="61"/>
     </row>
-    <row r="58" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="66" t="s">
         <v>166</v>
       </c>
@@ -4535,7 +4580,7 @@
       </c>
       <c r="F58" s="61"/>
     </row>
-    <row r="59" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="70" t="s">
         <v>183</v>
       </c>
@@ -4553,7 +4598,7 @@
       </c>
       <c r="F59" s="61"/>
     </row>
-    <row r="60" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="21" t="s">
         <v>59</v>
       </c>
@@ -4573,7 +4618,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="70" t="s">
         <v>179</v>
       </c>
@@ -4593,7 +4638,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="70" t="s">
         <v>180</v>
       </c>
@@ -4611,7 +4656,7 @@
       </c>
       <c r="F62" s="61"/>
     </row>
-    <row r="63" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="69" t="s">
         <v>173</v>
       </c>
@@ -4629,7 +4674,7 @@
       </c>
       <c r="F63" s="61"/>
     </row>
-    <row r="64" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="21" t="s">
         <v>64</v>
       </c>
@@ -4649,7 +4694,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="70" t="s">
         <v>182</v>
       </c>
@@ -4667,7 +4712,7 @@
       </c>
       <c r="F65" s="61"/>
     </row>
-    <row r="66" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="21" t="s">
         <v>61</v>
       </c>
@@ -4687,7 +4732,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="21" t="s">
         <v>58</v>
       </c>
@@ -4707,7 +4752,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="73" t="s">
         <v>184</v>
       </c>
@@ -4718,7 +4763,7 @@
         <v>43136</v>
       </c>
       <c r="D68" s="24">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E68" s="23">
         <v>43139</v>
@@ -4727,7 +4772,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="40" t="s">
         <v>104</v>
       </c>
@@ -4747,7 +4792,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="67" t="s">
         <v>168</v>
       </c>
@@ -4758,14 +4803,14 @@
         <v>43136</v>
       </c>
       <c r="D70" s="24">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E70" s="23">
         <v>43139</v>
       </c>
       <c r="F70" s="61"/>
     </row>
-    <row r="71" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="21" t="s">
         <v>62</v>
       </c>
@@ -4776,7 +4821,7 @@
         <v>43136</v>
       </c>
       <c r="D71" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E71" s="23">
         <v>43139</v>
@@ -4785,7 +4830,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="73" t="s">
         <v>186</v>
       </c>
@@ -4803,7 +4848,7 @@
       </c>
       <c r="F72" s="61"/>
     </row>
-    <row r="73" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="75" t="s">
         <v>187</v>
       </c>
@@ -4811,19 +4856,19 @@
         <v>43129</v>
       </c>
       <c r="C73" s="23">
-        <v>43133</v>
+        <v>43143</v>
       </c>
       <c r="D73" s="24">
         <v>0.25</v>
       </c>
       <c r="E73" s="23">
-        <v>43132</v>
+        <v>43160</v>
       </c>
       <c r="F73" s="76" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="77" t="s">
         <v>189</v>
       </c>
@@ -4841,7 +4886,7 @@
       </c>
       <c r="F74" s="61"/>
     </row>
-    <row r="75" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="77" t="s">
         <v>190</v>
       </c>
@@ -4859,7 +4904,7 @@
       </c>
       <c r="F75" s="61"/>
     </row>
-    <row r="76" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="77" t="s">
         <v>191</v>
       </c>
@@ -4877,7 +4922,7 @@
       </c>
       <c r="F76" s="61"/>
     </row>
-    <row r="77" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="78" t="s">
         <v>96</v>
       </c>
@@ -4895,7 +4940,7 @@
       </c>
       <c r="F77" s="61"/>
     </row>
-    <row r="78" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="78" t="s">
         <v>192</v>
       </c>
@@ -4906,14 +4951,14 @@
         <v>43133</v>
       </c>
       <c r="D78" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E78" s="23">
         <v>43139</v>
       </c>
       <c r="F78" s="61"/>
     </row>
-    <row r="79" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="78" t="s">
         <v>193</v>
       </c>
@@ -4924,14 +4969,14 @@
         <v>43136</v>
       </c>
       <c r="D79" s="24">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E79" s="23">
         <v>43139</v>
       </c>
       <c r="F79" s="61"/>
     </row>
-    <row r="80" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="79" t="s">
         <v>194</v>
       </c>
@@ -4949,7 +4994,7 @@
       </c>
       <c r="F80" s="61"/>
     </row>
-    <row r="81" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="79" t="s">
         <v>195</v>
       </c>
@@ -4960,14 +5005,14 @@
         <v>43132</v>
       </c>
       <c r="D81" s="24">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E81" s="23">
         <v>43139</v>
       </c>
       <c r="F81" s="61"/>
     </row>
-    <row r="82" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="80" t="s">
         <v>196</v>
       </c>
@@ -4978,7 +5023,7 @@
         <v>43136</v>
       </c>
       <c r="D82" s="24">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E82" s="23">
         <v>43139</v>
@@ -4987,7 +5032,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="81" t="s">
         <v>197</v>
       </c>
@@ -4998,14 +5043,14 @@
         <v>43133</v>
       </c>
       <c r="D83" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E83" s="23">
         <v>43139</v>
       </c>
       <c r="F83" s="61"/>
     </row>
-    <row r="84" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="81" t="s">
         <v>198</v>
       </c>
@@ -5023,7 +5068,7 @@
       </c>
       <c r="F84" s="61"/>
     </row>
-    <row r="85" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="81" t="s">
         <v>199</v>
       </c>
@@ -5034,14 +5079,16 @@
         <v>43136</v>
       </c>
       <c r="D85" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E85" s="23">
         <v>43139</v>
       </c>
-      <c r="F85" s="61"/>
-    </row>
-    <row r="86" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="F85" s="90" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="84" t="s">
         <v>201</v>
       </c>
@@ -5061,7 +5108,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="84" t="s">
         <v>203</v>
       </c>
@@ -5079,7 +5126,7 @@
       </c>
       <c r="F87" s="61"/>
     </row>
-    <row r="88" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="86" t="s">
         <v>204</v>
       </c>
@@ -5097,7 +5144,7 @@
       </c>
       <c r="F88" s="61"/>
     </row>
-    <row r="89" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="86" t="s">
         <v>205</v>
       </c>
@@ -5115,7 +5162,7 @@
       </c>
       <c r="F89" s="61"/>
     </row>
-    <row r="90" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="86" t="s">
         <v>206</v>
       </c>
@@ -5126,16 +5173,16 @@
         <v>43136</v>
       </c>
       <c r="D90" s="24">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E90" s="23">
         <v>43139</v>
       </c>
-      <c r="F90" s="88" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="F90" s="90" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="86" t="s">
         <v>207</v>
       </c>
@@ -5146,14 +5193,16 @@
         <v>43137</v>
       </c>
       <c r="D91" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E91" s="23">
         <v>43139</v>
       </c>
-      <c r="F91" s="61"/>
-    </row>
-    <row r="92" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="F91" s="90" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="87" t="s">
         <v>208</v>
       </c>
@@ -5173,9 +5222,9 @@
         <v>209</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="87" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B93" s="23">
         <v>43137</v>
@@ -5184,16 +5233,16 @@
         <v>43137</v>
       </c>
       <c r="D93" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E93" s="23">
         <v>43139</v>
       </c>
       <c r="F93" s="61"/>
     </row>
-    <row r="94" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A94" s="105" t="s">
-        <v>212</v>
+    <row r="94" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="89" t="s">
+        <v>211</v>
       </c>
       <c r="B94" s="23">
         <v>43137</v>
@@ -5202,66 +5251,176 @@
         <v>43137</v>
       </c>
       <c r="D94" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E94" s="23">
         <v>43139</v>
       </c>
-      <c r="F94" s="61"/>
-    </row>
-    <row r="95" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A95" s="86"/>
-      <c r="B95" s="23"/>
-      <c r="C95" s="82"/>
-      <c r="D95" s="24"/>
-      <c r="E95" s="23"/>
+      <c r="F94" s="90" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="89" t="s">
+        <v>212</v>
+      </c>
+      <c r="B95" s="23">
+        <v>43137</v>
+      </c>
+      <c r="C95" s="82">
+        <v>43137</v>
+      </c>
+      <c r="D95" s="24">
+        <v>1</v>
+      </c>
+      <c r="E95" s="23">
+        <v>43139</v>
+      </c>
       <c r="F95" s="61"/>
     </row>
-    <row r="96" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A96" s="86"/>
-      <c r="B96" s="23"/>
-      <c r="C96" s="82"/>
-      <c r="D96" s="24"/>
-      <c r="E96" s="23"/>
-      <c r="F96" s="61"/>
-    </row>
-    <row r="97" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A97" s="86"/>
-      <c r="B97" s="23"/>
-      <c r="C97" s="82"/>
-      <c r="D97" s="24"/>
-      <c r="E97" s="23"/>
-      <c r="F97" s="61"/>
-    </row>
-    <row r="98" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A98" s="86"/>
-      <c r="B98" s="23"/>
-      <c r="C98" s="82"/>
-      <c r="D98" s="24"/>
-      <c r="E98" s="23"/>
-      <c r="F98" s="61"/>
-    </row>
-    <row r="99" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A99" s="86"/>
+    <row r="96" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="89" t="s">
+        <v>213</v>
+      </c>
+      <c r="B96" s="23">
+        <v>43137</v>
+      </c>
+      <c r="C96" s="82">
+        <v>43137</v>
+      </c>
+      <c r="D96" s="24">
+        <v>1</v>
+      </c>
+      <c r="E96" s="23">
+        <v>43139</v>
+      </c>
+      <c r="F96" s="90" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="91" t="s">
+        <v>219</v>
+      </c>
+      <c r="B97" s="23">
+        <v>43138</v>
+      </c>
+      <c r="C97" s="82">
+        <v>43139</v>
+      </c>
+      <c r="D97" s="24">
+        <v>1</v>
+      </c>
+      <c r="E97" s="23">
+        <v>43139</v>
+      </c>
+      <c r="F97" s="90"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" s="91" t="s">
+        <v>220</v>
+      </c>
+      <c r="B98" s="23">
+        <v>43138</v>
+      </c>
+      <c r="C98" s="82">
+        <v>43139</v>
+      </c>
+      <c r="D98" s="24">
+        <v>0</v>
+      </c>
+      <c r="E98" s="92">
+        <v>43139</v>
+      </c>
+      <c r="F98" s="90"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="91" t="s">
+        <v>221</v>
+      </c>
       <c r="B99" s="23"/>
       <c r="C99" s="82"/>
       <c r="D99" s="24"/>
       <c r="E99" s="23"/>
-      <c r="F99" s="61"/>
-    </row>
-    <row r="100" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="F99" s="90"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="91"/>
       <c r="B100" s="23"/>
-      <c r="C100" s="23"/>
+      <c r="C100" s="82"/>
       <c r="D100" s="24"/>
       <c r="E100" s="23"/>
-      <c r="F100" s="59"/>
-    </row>
-    <row r="101" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="102" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="103" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="104" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
+      <c r="F100" s="90"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="91"/>
+      <c r="B101" s="23"/>
+      <c r="C101" s="82"/>
+      <c r="D101" s="24"/>
+      <c r="E101" s="23"/>
+      <c r="F101" s="90"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="91"/>
+      <c r="B102" s="23"/>
+      <c r="C102" s="82"/>
+      <c r="D102" s="24"/>
+      <c r="E102" s="23"/>
+      <c r="F102" s="90"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" s="89"/>
+      <c r="B103" s="23"/>
+      <c r="C103" s="82"/>
+      <c r="D103" s="24"/>
+      <c r="E103" s="23"/>
+      <c r="F103" s="90"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="89"/>
+      <c r="B104" s="23"/>
+      <c r="C104" s="82"/>
+      <c r="D104" s="24"/>
+      <c r="E104" s="23"/>
+      <c r="F104" s="90"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" s="86"/>
+      <c r="B105" s="23"/>
+      <c r="C105" s="82"/>
+      <c r="D105" s="24"/>
+      <c r="E105" s="23"/>
+      <c r="F105" s="61"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="86"/>
+      <c r="B106" s="23"/>
+      <c r="C106" s="82"/>
+      <c r="D106" s="24"/>
+      <c r="E106" s="23"/>
+      <c r="F106" s="61"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107" s="86"/>
+      <c r="B107" s="23"/>
+      <c r="C107" s="82"/>
+      <c r="D107" s="24"/>
+      <c r="E107" s="23"/>
+      <c r="F107" s="61"/>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B108" s="23"/>
+      <c r="C108" s="23"/>
+      <c r="D108" s="24"/>
+      <c r="E108" s="23"/>
+      <c r="F108" s="59"/>
+    </row>
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="110" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="111" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="112" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <conditionalFormatting sqref="D2:D100">
+  <conditionalFormatting sqref="D2:D108">
     <cfRule type="iconSet" priority="16">
       <iconSet iconSet="5Quarters" showValue="0">
         <cfvo type="percent" val="0"/>
@@ -5283,17 +5442,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.6" zeroHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="9" width="4.78515625" style="42" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" style="42" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" style="42" customWidth="1"/>
-    <col min="12" max="12" width="13.85546875" style="42" customWidth="1"/>
-    <col min="13" max="17" width="11.140625" style="42" customWidth="1"/>
-    <col min="18" max="16384" width="8.85546875" hidden="1"/>
+    <col min="1" max="9" width="4.77734375" style="42" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" style="42" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" style="42" customWidth="1"/>
+    <col min="12" max="12" width="13.88671875" style="42" customWidth="1"/>
+    <col min="13" max="17" width="11.109375" style="42" customWidth="1"/>
+    <col min="18" max="16384" width="8.88671875" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="74.150000000000006" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:17" ht="72.599999999999994" x14ac:dyDescent="0.3">
       <c r="A1" s="41" t="s">
         <v>110</v>
       </c>
@@ -5346,7 +5505,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="43">
         <v>1</v>
       </c>
@@ -5375,7 +5534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="43">
         <v>2</v>
       </c>
@@ -5404,7 +5563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="43">
         <v>3</v>
       </c>
@@ -5433,7 +5592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="43">
         <v>4</v>
       </c>
@@ -5462,7 +5621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="43">
         <v>5</v>
       </c>
@@ -5491,7 +5650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="43">
         <v>6</v>
       </c>
@@ -5520,7 +5679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="43">
         <v>7</v>
       </c>
@@ -5549,7 +5708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="43">
         <v>8</v>
       </c>
@@ -5578,7 +5737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="43">
         <v>9</v>
       </c>
@@ -5607,7 +5766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="43">
         <v>10</v>
       </c>
@@ -5636,7 +5795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="43">
         <v>11</v>
       </c>
@@ -5665,7 +5824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="43">
         <v>12</v>
       </c>
@@ -5694,7 +5853,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="43">
         <v>13</v>
       </c>
@@ -5723,7 +5882,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="43">
         <v>14</v>
       </c>
@@ -5752,7 +5911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="43">
         <v>15</v>
       </c>
@@ -5781,7 +5940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="43">
         <v>16</v>
       </c>
@@ -5810,7 +5969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="43">
         <v>17</v>
       </c>
@@ -5839,7 +5998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="43">
         <v>18</v>
       </c>
@@ -5868,7 +6027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="43">
         <v>19</v>
       </c>
@@ -5897,7 +6056,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="43">
         <v>20</v>
       </c>
@@ -5926,7 +6085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="43">
         <v>21</v>
       </c>
@@ -5955,7 +6114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="43">
         <v>22</v>
       </c>
@@ -5984,7 +6143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="43">
         <v>23</v>
       </c>
@@ -6013,7 +6172,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="43">
         <v>24</v>
       </c>
@@ -6042,7 +6201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="43">
         <v>25</v>
       </c>
@@ -6071,7 +6230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="43">
         <v>26</v>
       </c>
@@ -6100,7 +6259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="43">
         <v>27</v>
       </c>
@@ -6129,7 +6288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="43">
         <v>28</v>
       </c>
@@ -6158,7 +6317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="43">
         <v>29</v>
       </c>
@@ -6187,7 +6346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="43">
         <v>30</v>
       </c>
@@ -6216,7 +6375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="43">
         <v>31</v>
       </c>
@@ -6245,7 +6404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="43">
         <v>32</v>
       </c>
@@ -6274,7 +6433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -6287,16 +6446,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.6" zeroHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.78515625" customWidth="1"/>
-    <col min="2" max="2" width="12.640625" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" customWidth="1"/>
-    <col min="4" max="4" width="53.5703125" customWidth="1"/>
-    <col min="5" max="16384" width="8.85546875" hidden="1"/>
+    <col min="1" max="1" width="11.77734375" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" customWidth="1"/>
+    <col min="4" max="4" width="53.5546875" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>124</v>
       </c>
@@ -6310,7 +6469,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>126</v>
       </c>
@@ -6324,7 +6483,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>128</v>
       </c>
@@ -6338,7 +6497,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>130</v>
       </c>
@@ -6352,7 +6511,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>137</v>
       </c>
@@ -6363,7 +6522,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>105</v>
       </c>
@@ -6375,7 +6534,7 @@
       </c>
       <c r="D6" s="45"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>140</v>
       </c>
@@ -6387,19 +6546,19 @@
       </c>
       <c r="D7" s="45"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>141</v>
       </c>
       <c r="D8" s="45"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>142</v>
       </c>
       <c r="D9" s="45"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>143</v>
       </c>
@@ -6408,43 +6567,43 @@
       </c>
       <c r="D10" s="45"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D11" s="45"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D12" s="45"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D13" s="45"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D14" s="45"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D15" s="45"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D16" s="45"/>
     </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D17" s="45"/>
     </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D18" s="45"/>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D19" s="45"/>
     </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D20" s="45"/>
     </row>
-    <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="D21" s="45"/>
     </row>
-    <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="D22" s="45"/>
     </row>
-    <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="D23" s="45"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add job array code for SLURM
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -30,12 +30,11 @@
     <definedName name="TitleRegion..BO60">'Project Planner'!$B$3:$B$4</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="223">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -772,7 +771,10 @@
     <t>Ask about second derivative check for stochastic</t>
   </si>
   <si>
-    <t xml:space="preserve">Use thin wall for parke </t>
+    <t>Get Matlab code running on hummingbird</t>
+  </si>
+  <si>
+    <t>Ask about integration failures in instanton calculation</t>
   </si>
 </sst>
 </file>
@@ -783,13 +785,20 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="60" x14ac:knownFonts="1">
+  <fonts count="61" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1348,98 +1357,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="55" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="56" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="48" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="49" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="58" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="59" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="57" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="57" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="57" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="57" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="57" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="55" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="56" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="48" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="49" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="51" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="52" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="58" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="59" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -1457,25 +1466,26 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="55" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="56" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="55" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="56" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="45" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="46" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -1491,23 +1501,23 @@
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -1516,118 +1526,118 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="18" fontId="36" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="37" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -2493,13 +2503,13 @@
       <c r="G1" s="10"/>
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="95" t="s">
+      <c r="B2" s="96" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
@@ -2507,66 +2517,66 @@
         <v>8</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="101" t="s">
+      <c r="K2" s="102" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="102"/>
-      <c r="M2" s="102"/>
-      <c r="N2" s="102"/>
-      <c r="O2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="103"/>
+      <c r="O2" s="104"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="101" t="s">
+      <c r="Q2" s="102" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="104"/>
-      <c r="S2" s="104"/>
-      <c r="T2" s="103"/>
+      <c r="R2" s="105"/>
+      <c r="S2" s="105"/>
+      <c r="T2" s="104"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="93" t="s">
+      <c r="V2" s="94" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="94"/>
-      <c r="X2" s="94"/>
-      <c r="Y2" s="105"/>
+      <c r="W2" s="95"/>
+      <c r="X2" s="95"/>
+      <c r="Y2" s="106"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="106" t="s">
+      <c r="AA2" s="107" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="107"/>
-      <c r="AC2" s="107"/>
-      <c r="AD2" s="107"/>
-      <c r="AE2" s="107"/>
-      <c r="AF2" s="107"/>
-      <c r="AG2" s="108"/>
+      <c r="AB2" s="108"/>
+      <c r="AC2" s="108"/>
+      <c r="AD2" s="108"/>
+      <c r="AE2" s="108"/>
+      <c r="AF2" s="108"/>
+      <c r="AG2" s="109"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="93" t="s">
+      <c r="AI2" s="94" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="94"/>
-      <c r="AK2" s="94"/>
-      <c r="AL2" s="94"/>
-      <c r="AM2" s="94"/>
-      <c r="AN2" s="94"/>
-      <c r="AO2" s="94"/>
-      <c r="AP2" s="94"/>
+      <c r="AJ2" s="95"/>
+      <c r="AK2" s="95"/>
+      <c r="AL2" s="95"/>
+      <c r="AM2" s="95"/>
+      <c r="AN2" s="95"/>
+      <c r="AO2" s="95"/>
+      <c r="AP2" s="95"/>
     </row>
     <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="96" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="98" t="s">
+      <c r="B3" s="97" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="99" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="98" t="s">
+      <c r="D3" s="99" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="98" t="s">
+      <c r="E3" s="99" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="98" t="s">
+      <c r="F3" s="99" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="100" t="s">
+      <c r="G3" s="101" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -2695,12 +2705,12 @@
       <c r="AW3" s="18"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="97"/>
-      <c r="C4" s="99"/>
-      <c r="D4" s="99"/>
-      <c r="E4" s="99"/>
-      <c r="F4" s="99"/>
-      <c r="G4" s="99"/>
+      <c r="B4" s="98"/>
+      <c r="C4" s="100"/>
+      <c r="D4" s="100"/>
+      <c r="E4" s="100"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="100"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -4055,7 +4065,7 @@
         <v>43124</v>
       </c>
       <c r="C30" s="23">
-        <v>43138</v>
+        <v>43142</v>
       </c>
       <c r="D30" s="24">
         <v>0.25</v>
@@ -4276,7 +4286,7 @@
       </c>
       <c r="B42" s="23">
         <f ca="1">TODAY()</f>
-        <v>43138</v>
+        <v>43139</v>
       </c>
       <c r="C42" s="23">
         <v>43118</v>
@@ -4315,7 +4325,7 @@
       </c>
       <c r="B44" s="23">
         <f ca="1">TODAY()</f>
-        <v>43138</v>
+        <v>43139</v>
       </c>
       <c r="C44" s="23">
         <v>43118</v>
@@ -4334,7 +4344,7 @@
       </c>
       <c r="B45" s="23">
         <f ca="1">TODAY()</f>
-        <v>43138</v>
+        <v>43139</v>
       </c>
       <c r="C45" s="23">
         <v>43118</v>
@@ -4371,7 +4381,7 @@
       </c>
       <c r="B47" s="23">
         <f ca="1">TODAY()</f>
-        <v>43138</v>
+        <v>43139</v>
       </c>
       <c r="C47" s="23"/>
       <c r="D47" s="24">
@@ -4740,7 +4750,7 @@
         <v>43124</v>
       </c>
       <c r="C67" s="23">
-        <v>43138</v>
+        <v>43142</v>
       </c>
       <c r="D67" s="24">
         <v>0.25</v>
@@ -5335,21 +5345,39 @@
       <c r="F98" s="90"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="91" t="s">
+      <c r="A99" s="93" t="s">
+        <v>222</v>
+      </c>
+      <c r="B99" s="23">
+        <v>43138</v>
+      </c>
+      <c r="C99" s="82">
+        <v>43139</v>
+      </c>
+      <c r="D99" s="24">
+        <v>0</v>
+      </c>
+      <c r="E99" s="23">
+        <v>43139</v>
+      </c>
+      <c r="F99" s="90"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="93" t="s">
         <v>221</v>
       </c>
-      <c r="B99" s="23"/>
-      <c r="C99" s="82"/>
-      <c r="D99" s="24"/>
-      <c r="E99" s="23"/>
-      <c r="F99" s="90"/>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="91"/>
-      <c r="B100" s="23"/>
-      <c r="C100" s="82"/>
-      <c r="D100" s="24"/>
-      <c r="E100" s="23"/>
+      <c r="B100" s="23">
+        <v>43138</v>
+      </c>
+      <c r="C100" s="82">
+        <v>43138</v>
+      </c>
+      <c r="D100" s="24">
+        <v>1</v>
+      </c>
+      <c r="E100" s="23">
+        <v>43139</v>
+      </c>
       <c r="F100" s="90"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
@@ -5452,7 +5480,7 @@
     <col min="18" max="16384" width="8.88671875" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="72.599999999999994" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="73.2" x14ac:dyDescent="0.3">
       <c r="A1" s="41" t="s">
         <v>110</v>
       </c>

</xml_diff>

<commit_message>
Fixed bad reference to obj.m_Pl
</commit_message>
<xml_diff>
--- a/ProjectPlanner.xlsx
+++ b/ProjectPlanner.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="390">
   <si>
     <t>ACTIVITY</t>
   </si>
@@ -1503,6 +1503,12 @@
   <si>
     <t>Get VBA to automate infile creation from run table</t>
   </si>
+  <si>
+    <t>Make B_cutoff an argument rather than a parameter</t>
+  </si>
+  <si>
+    <t>Measure B, but don't demand inflation at phistart, search for it downhill</t>
+  </si>
 </sst>
 </file>
 
@@ -1511,15 +1517,22 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
-    <numFmt numFmtId="169" formatCode="0000"/>
+    <numFmt numFmtId="166" formatCode="0000"/>
   </numFmts>
-  <fonts count="70" x14ac:knownFonts="1">
+  <fonts count="71" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1" tint="0.24994659260841701"/>
       <name val="Corbel"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2146,98 +2159,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="60" fillId="0" borderId="2" applyFill="0" applyProtection="0">
+    <xf numFmtId="3" fontId="61" fillId="0" borderId="2" applyFill="0" applyProtection="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="53" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="9" fontId="54" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="60" fillId="6" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" applyFill="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="63" fillId="6" borderId="1">
+    <xf numFmtId="1" fontId="64" fillId="6" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="62" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="62" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="62" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="62" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
+    <xf numFmtId="0" fontId="62" fillId="7" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="2">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="2">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="60" fillId="0" borderId="2" xfId="3">
+    <xf numFmtId="3" fontId="61" fillId="0" borderId="2" xfId="3">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="53" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="9" fontId="54" fillId="0" borderId="0" xfId="6">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="6" borderId="1" xfId="7">
+    <xf numFmtId="0" fontId="60" fillId="6" borderId="1" xfId="7">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="2" applyFont="1">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="2" applyFont="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="56" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="9" fontId="57" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="63" fillId="6" borderId="1" xfId="13">
+    <xf numFmtId="1" fontId="64" fillId="6" borderId="1" xfId="13">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="14" applyFont="1" applyAlignment="1">
@@ -2255,25 +2268,26 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="18" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="60" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="61" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="60" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="61" fillId="8" borderId="0" xfId="11" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="19"/>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="19"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="50" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="51" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -2289,20 +2303,20 @@
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="64" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="64" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="64" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="19" applyFont="1"/>
@@ -2311,104 +2325,116 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="19" applyAlignment="1">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="19" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="18" fontId="41" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="42" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="19" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="65" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="66" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="67" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="66" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="1" fontId="67" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="19" applyFont="1"/>
+    <xf numFmtId="0" fontId="70" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="70" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="70" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="60" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
@@ -2417,34 +2443,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="12">
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="12">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="9">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="9">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="2" xfId="9" applyBorder="1">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="2" xfId="9" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="10">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="10">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="2" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="2" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="5" xfId="10" applyBorder="1">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="5" xfId="10" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="5" applyFont="1">
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="5" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="5" applyFont="1" applyBorder="1">
@@ -2460,17 +2486,11 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1"/>
-    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="19" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="69" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="59" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="19" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="20">
@@ -2496,24 +2516,6 @@
     <cellStyle name="Title" xfId="8" builtinId="15" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="43">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2657,185 +2659,7 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="169" formatCode="0000"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="0.24994659260841701"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2922,9 +2746,6 @@
         <family val="3"/>
         <scheme val="none"/>
       </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -3179,6 +3000,205 @@
       </font>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0000"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="0.24994659260841701"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -3201,8 +3221,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F115" totalsRowShown="0">
-  <autoFilter ref="A1:F115">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F129" totalsRowShown="0">
+  <autoFilter ref="A1:F129">
     <filterColumn colId="3">
       <filters blank="1">
         <filter val="0"/>
@@ -3210,8 +3230,8 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState ref="A30:F115">
-    <sortCondition descending="1" ref="C1:C115"/>
+  <sortState ref="A30:F129">
+    <sortCondition descending="1" ref="C1:C129"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" name="Task"/>
@@ -3229,46 +3249,46 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:W33" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
   <autoFilter ref="A1:W33"/>
   <tableColumns count="23">
-    <tableColumn id="1" name="Test ID" dataDxfId="11"/>
-    <tableColumn id="18" name="n_iter" dataDxfId="12"/>
-    <tableColumn id="2" name="log10(mv)" dataDxfId="13"/>
-    <tableColumn id="3" name="mh" dataDxfId="39"/>
-    <tableColumn id="4" name="kmax" dataDxfId="38"/>
-    <tableColumn id="19" name="gamma" dataDxfId="20"/>
-    <tableColumn id="8" name="measure" dataDxfId="18"/>
-    <tableColumn id="9" name="n_tunnel_max" dataDxfId="17"/>
-    <tableColumn id="5" name="lambda_screen" dataDxfId="37"/>
-    <tableColumn id="6" name="rho_Lambda_thres" dataDxfId="36"/>
-    <tableColumn id="20" name="fixQ" dataDxfId="16"/>
-    <tableColumn id="21" name="Nafter" dataDxfId="15"/>
-    <tableColumn id="22" name="seed" dataDxfId="14"/>
-    <tableColumn id="7" name="n_recycle" dataDxfId="19"/>
-    <tableColumn id="10" name="Start Date" dataDxfId="35"/>
-    <tableColumn id="24" name="End Date" dataDxfId="0"/>
-    <tableColumn id="11" name="Runtime" dataDxfId="34"/>
-    <tableColumn id="12" name="File name" dataDxfId="33"/>
-    <tableColumn id="13" name="Column13" dataDxfId="32"/>
-    <tableColumn id="14" name="Column14" dataDxfId="31"/>
-    <tableColumn id="15" name="Column15" dataDxfId="30"/>
-    <tableColumn id="16" name="Column16" dataDxfId="29"/>
-    <tableColumn id="17" name="Column17" dataDxfId="28"/>
+    <tableColumn id="1" name="Test ID" dataDxfId="39"/>
+    <tableColumn id="18" name="n_iter" dataDxfId="38"/>
+    <tableColumn id="2" name="log10(mv)" dataDxfId="37"/>
+    <tableColumn id="3" name="mh" dataDxfId="36"/>
+    <tableColumn id="4" name="kmax" dataDxfId="35"/>
+    <tableColumn id="19" name="gamma" dataDxfId="34"/>
+    <tableColumn id="8" name="measure" dataDxfId="33"/>
+    <tableColumn id="9" name="n_tunnel_max" dataDxfId="32"/>
+    <tableColumn id="5" name="lambda_screen" dataDxfId="31"/>
+    <tableColumn id="6" name="rho_Lambda_thres" dataDxfId="30"/>
+    <tableColumn id="20" name="fixQ" dataDxfId="29"/>
+    <tableColumn id="21" name="Nafter" dataDxfId="28"/>
+    <tableColumn id="22" name="seed" dataDxfId="27"/>
+    <tableColumn id="7" name="n_recycle" dataDxfId="26"/>
+    <tableColumn id="10" name="Start Date" dataDxfId="25"/>
+    <tableColumn id="24" name="End Date" dataDxfId="24"/>
+    <tableColumn id="11" name="Runtime" dataDxfId="23"/>
+    <tableColumn id="12" name="File name" dataDxfId="22"/>
+    <tableColumn id="13" name="Column13" dataDxfId="21"/>
+    <tableColumn id="14" name="Column14" dataDxfId="20"/>
+    <tableColumn id="15" name="Column15" dataDxfId="19"/>
+    <tableColumn id="16" name="Column16" dataDxfId="18"/>
+    <tableColumn id="17" name="Column17" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table44" displayName="Table44" ref="A1:E117" totalsRowShown="0" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table44" displayName="Table44" ref="A1:E117" totalsRowShown="0" dataDxfId="16">
   <autoFilter ref="A1:E117"/>
   <sortState ref="A2:E117">
     <sortCondition ref="A1:A117"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" name="Class" dataDxfId="25"/>
-    <tableColumn id="2" name="Function" dataDxfId="24"/>
-    <tableColumn id="3" name="Line" dataDxfId="23"/>
-    <tableColumn id="5" name="Checked" dataDxfId="22"/>
-    <tableColumn id="4" name="Description" dataDxfId="21"/>
+    <tableColumn id="1" name="Class" dataDxfId="15"/>
+    <tableColumn id="2" name="Function" dataDxfId="14"/>
+    <tableColumn id="3" name="Line" dataDxfId="13"/>
+    <tableColumn id="5" name="Checked" dataDxfId="12"/>
+    <tableColumn id="4" name="Description" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3292,7 +3312,7 @@
     <tableColumn id="6" name="Quantity"/>
     <tableColumn id="2" name="Dimensions"/>
     <tableColumn id="3" name="Units"/>
-    <tableColumn id="4" name="Description" dataDxfId="27"/>
+    <tableColumn id="4" name="Description" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3553,13 +3573,13 @@
       <c r="G1" s="10"/>
     </row>
     <row r="2" spans="2:67" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="104" t="s">
+      <c r="B2" s="109" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="104"/>
-      <c r="D2" s="104"/>
-      <c r="E2" s="104"/>
-      <c r="F2" s="104"/>
+      <c r="C2" s="109"/>
+      <c r="D2" s="109"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
@@ -3567,66 +3587,66 @@
         <v>8</v>
       </c>
       <c r="J2" s="13"/>
-      <c r="K2" s="110" t="s">
+      <c r="K2" s="115" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="111"/>
-      <c r="M2" s="111"/>
-      <c r="N2" s="111"/>
-      <c r="O2" s="112"/>
+      <c r="L2" s="116"/>
+      <c r="M2" s="116"/>
+      <c r="N2" s="116"/>
+      <c r="O2" s="117"/>
       <c r="P2" s="14"/>
-      <c r="Q2" s="110" t="s">
+      <c r="Q2" s="115" t="s">
         <v>26</v>
       </c>
-      <c r="R2" s="113"/>
-      <c r="S2" s="113"/>
-      <c r="T2" s="112"/>
+      <c r="R2" s="118"/>
+      <c r="S2" s="118"/>
+      <c r="T2" s="117"/>
       <c r="U2" s="15"/>
-      <c r="V2" s="102" t="s">
+      <c r="V2" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="W2" s="103"/>
-      <c r="X2" s="103"/>
-      <c r="Y2" s="114"/>
+      <c r="W2" s="108"/>
+      <c r="X2" s="108"/>
+      <c r="Y2" s="119"/>
       <c r="Z2" s="16"/>
-      <c r="AA2" s="115" t="s">
+      <c r="AA2" s="120" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="116"/>
-      <c r="AC2" s="116"/>
-      <c r="AD2" s="116"/>
-      <c r="AE2" s="116"/>
-      <c r="AF2" s="116"/>
-      <c r="AG2" s="117"/>
+      <c r="AB2" s="121"/>
+      <c r="AC2" s="121"/>
+      <c r="AD2" s="121"/>
+      <c r="AE2" s="121"/>
+      <c r="AF2" s="121"/>
+      <c r="AG2" s="122"/>
       <c r="AH2" s="17"/>
-      <c r="AI2" s="102" t="s">
+      <c r="AI2" s="107" t="s">
         <v>19</v>
       </c>
-      <c r="AJ2" s="103"/>
-      <c r="AK2" s="103"/>
-      <c r="AL2" s="103"/>
-      <c r="AM2" s="103"/>
-      <c r="AN2" s="103"/>
-      <c r="AO2" s="103"/>
-      <c r="AP2" s="103"/>
+      <c r="AJ2" s="108"/>
+      <c r="AK2" s="108"/>
+      <c r="AL2" s="108"/>
+      <c r="AM2" s="108"/>
+      <c r="AN2" s="108"/>
+      <c r="AO2" s="108"/>
+      <c r="AP2" s="108"/>
     </row>
     <row r="3" spans="2:67" s="9" customFormat="1" ht="39.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="105" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="107" t="s">
+      <c r="B3" s="110" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="112" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="107" t="s">
+      <c r="D3" s="112" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="107" t="s">
+      <c r="E3" s="112" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="107" t="s">
+      <c r="F3" s="112" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="109" t="s">
+      <c r="G3" s="114" t="s">
         <v>25</v>
       </c>
       <c r="H3" s="18">
@@ -3755,12 +3775,12 @@
       <c r="AW3" s="18"/>
     </row>
     <row r="4" spans="2:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="106"/>
-      <c r="C4" s="108"/>
-      <c r="D4" s="108"/>
-      <c r="E4" s="108"/>
-      <c r="F4" s="108"/>
-      <c r="G4" s="108"/>
+      <c r="B4" s="111"/>
+      <c r="C4" s="113"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="113"/>
+      <c r="F4" s="113"/>
+      <c r="G4" s="113"/>
       <c r="H4" s="3">
         <v>1</v>
       </c>
@@ -4479,38 +4499,38 @@
     <mergeCell ref="AA2:AG2"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:BO31">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>PercentComplete</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="3">
+    <cfRule type="expression" dxfId="8" priority="3">
       <formula>PercentCompleteBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="4">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>Actual</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>ActualBeyond</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>Plan</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="7">
+    <cfRule type="expression" dxfId="4" priority="7">
       <formula>H$4=period_selected</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="11">
+    <cfRule type="expression" dxfId="3" priority="11">
       <formula>MOD(COLUMN(),2)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="12">
+    <cfRule type="expression" dxfId="2" priority="12">
       <formula>MOD(COLUMN(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:BO32">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:BO4">
-    <cfRule type="expression" dxfId="1" priority="8">
+    <cfRule type="expression" dxfId="0" priority="8">
       <formula>H$4=period_selected</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4545,7 +4565,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G119"/>
+  <dimension ref="A1:G133"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="51.2109375" style="21" customWidth="1"/>
@@ -5123,7 +5143,9 @@
       <c r="E30" s="23">
         <v>43160</v>
       </c>
-      <c r="F30" s="89"/>
+      <c r="F30" s="125" t="s">
+        <v>389</v>
+      </c>
     </row>
     <row r="31" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A31" s="26" t="s">
@@ -6487,7 +6509,7 @@
       <c r="F103" s="89"/>
     </row>
     <row r="104" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A104" s="118" t="s">
+      <c r="A104" s="102" t="s">
         <v>330</v>
       </c>
       <c r="B104" s="23">
@@ -6524,8 +6546,8 @@
       </c>
       <c r="F105" s="60"/>
     </row>
-    <row r="106" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A106" s="118" t="s">
+    <row r="106" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A106" s="102" t="s">
         <v>331</v>
       </c>
       <c r="B106" s="23">
@@ -6535,7 +6557,7 @@
         <v>43145</v>
       </c>
       <c r="D106" s="24">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E106" s="23">
         <v>43160</v>
@@ -6562,7 +6584,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
       <c r="A108" s="97" t="s">
         <v>325</v>
       </c>
@@ -6573,15 +6595,15 @@
         <v>43144</v>
       </c>
       <c r="D108" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E108" s="23">
         <v>43160</v>
       </c>
       <c r="F108" s="96"/>
     </row>
-    <row r="109" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A109" s="118" t="s">
+    <row r="109" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A109" s="102" t="s">
         <v>329</v>
       </c>
       <c r="B109" s="23">
@@ -6598,8 +6620,8 @@
       </c>
       <c r="F109" s="96"/>
     </row>
-    <row r="110" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A110" s="118" t="s">
+    <row r="110" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A110" s="102" t="s">
         <v>332</v>
       </c>
       <c r="B110" s="23">
@@ -6609,15 +6631,15 @@
         <v>43144</v>
       </c>
       <c r="D110" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E110" s="23">
         <v>43160</v>
       </c>
       <c r="F110" s="96"/>
     </row>
-    <row r="111" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A111" s="118" t="s">
+    <row r="111" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A111" s="102" t="s">
         <v>387</v>
       </c>
       <c r="B111" s="23">
@@ -6627,50 +6649,172 @@
         <v>43144</v>
       </c>
       <c r="D111" s="24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E111" s="23">
         <v>43160</v>
       </c>
       <c r="F111" s="96"/>
     </row>
-    <row r="112" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A112" s="97"/>
-      <c r="B112" s="23"/>
-      <c r="C112" s="81"/>
-      <c r="D112" s="24"/>
-      <c r="E112" s="23"/>
+    <row r="112" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A112" s="123" t="s">
+        <v>388</v>
+      </c>
+      <c r="B112" s="124">
+        <v>43144</v>
+      </c>
+      <c r="C112" s="81">
+        <v>43145</v>
+      </c>
+      <c r="D112" s="24">
+        <v>1</v>
+      </c>
+      <c r="E112" s="23">
+        <v>43160</v>
+      </c>
       <c r="F112" s="96"/>
     </row>
     <row r="113" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A113" s="97"/>
-      <c r="B113" s="23"/>
+      <c r="A113" s="123"/>
+      <c r="B113" s="124"/>
       <c r="C113" s="81"/>
       <c r="D113" s="24"/>
       <c r="E113" s="23"/>
       <c r="F113" s="96"/>
     </row>
     <row r="114" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="A114" s="85"/>
-      <c r="B114" s="23"/>
+      <c r="A114" s="123"/>
+      <c r="B114" s="124"/>
       <c r="C114" s="81"/>
       <c r="D114" s="24"/>
       <c r="E114" s="23"/>
-      <c r="F114" s="60"/>
+      <c r="F114" s="96"/>
     </row>
     <row r="115" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
-      <c r="B115" s="23"/>
-      <c r="C115" s="23"/>
+      <c r="A115" s="123"/>
+      <c r="B115" s="124"/>
+      <c r="C115" s="81"/>
       <c r="D115" s="24"/>
       <c r="E115" s="23"/>
-      <c r="F115" s="58"/>
-    </row>
-    <row r="116" spans="1:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="117" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="118" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="119" spans="1:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
+      <c r="F115" s="96"/>
+    </row>
+    <row r="116" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A116" s="123"/>
+      <c r="B116" s="124"/>
+      <c r="C116" s="81"/>
+      <c r="D116" s="24"/>
+      <c r="E116" s="23"/>
+      <c r="F116" s="96"/>
+    </row>
+    <row r="117" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A117" s="123"/>
+      <c r="B117" s="124"/>
+      <c r="C117" s="81"/>
+      <c r="D117" s="24"/>
+      <c r="E117" s="23"/>
+      <c r="F117" s="96"/>
+    </row>
+    <row r="118" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A118" s="123"/>
+      <c r="B118" s="124"/>
+      <c r="C118" s="81"/>
+      <c r="D118" s="24"/>
+      <c r="E118" s="23"/>
+      <c r="F118" s="96"/>
+    </row>
+    <row r="119" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A119" s="123"/>
+      <c r="B119" s="124"/>
+      <c r="C119" s="81"/>
+      <c r="D119" s="24"/>
+      <c r="E119" s="23"/>
+      <c r="F119" s="96"/>
+    </row>
+    <row r="120" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A120" s="123"/>
+      <c r="B120" s="124"/>
+      <c r="C120" s="81"/>
+      <c r="D120" s="24"/>
+      <c r="E120" s="23"/>
+      <c r="F120" s="96"/>
+    </row>
+    <row r="121" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A121" s="123"/>
+      <c r="B121" s="124"/>
+      <c r="C121" s="81"/>
+      <c r="D121" s="24"/>
+      <c r="E121" s="23"/>
+      <c r="F121" s="96"/>
+    </row>
+    <row r="122" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A122" s="123"/>
+      <c r="B122" s="124"/>
+      <c r="C122" s="81"/>
+      <c r="D122" s="24"/>
+      <c r="E122" s="23"/>
+      <c r="F122" s="96"/>
+    </row>
+    <row r="123" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A123" s="123"/>
+      <c r="B123" s="124"/>
+      <c r="C123" s="81"/>
+      <c r="D123" s="24"/>
+      <c r="E123" s="23"/>
+      <c r="F123" s="96"/>
+    </row>
+    <row r="124" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A124" s="123"/>
+      <c r="B124" s="124"/>
+      <c r="C124" s="81"/>
+      <c r="D124" s="24"/>
+      <c r="E124" s="23"/>
+      <c r="F124" s="96"/>
+    </row>
+    <row r="125" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A125" s="123"/>
+      <c r="B125" s="124"/>
+      <c r="C125" s="81"/>
+      <c r="D125" s="24"/>
+      <c r="E125" s="23"/>
+      <c r="F125" s="96"/>
+    </row>
+    <row r="126" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A126" s="123"/>
+      <c r="B126" s="124"/>
+      <c r="C126" s="81"/>
+      <c r="D126" s="24"/>
+      <c r="E126" s="23"/>
+      <c r="F126" s="96"/>
+    </row>
+    <row r="127" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A127" s="97"/>
+      <c r="B127" s="23"/>
+      <c r="C127" s="81"/>
+      <c r="D127" s="24"/>
+      <c r="E127" s="23"/>
+      <c r="F127" s="96"/>
+    </row>
+    <row r="128" spans="1:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="A128" s="85"/>
+      <c r="B128" s="23"/>
+      <c r="C128" s="81"/>
+      <c r="D128" s="24"/>
+      <c r="E128" s="23"/>
+      <c r="F128" s="60"/>
+    </row>
+    <row r="129" spans="2:6" ht="14.6" x14ac:dyDescent="0.4">
+      <c r="B129" s="23"/>
+      <c r="C129" s="23"/>
+      <c r="D129" s="24"/>
+      <c r="E129" s="23"/>
+      <c r="F129" s="58"/>
+    </row>
+    <row r="130" spans="2:6" ht="14.6" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="131" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="132" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="133" spans="2:6" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
-  <conditionalFormatting sqref="D2:D115">
+  <conditionalFormatting sqref="D2:D129">
     <cfRule type="iconSet" priority="16">
       <iconSet iconSet="5Quarters" showValue="0">
         <cfvo type="percent" val="0"/>
@@ -6704,7 +6848,7 @@
     <col min="21" max="25" width="11.140625" style="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="92.6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:25" ht="92.15" x14ac:dyDescent="0.4">
       <c r="A1" s="41" t="s">
         <v>107</v>
       </c>
@@ -6778,7 +6922,7 @@
       <c r="Y1"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A2" s="122">
+      <c r="A2" s="106">
         <v>1</v>
       </c>
       <c r="B2" s="42">
@@ -6827,7 +6971,7 @@
       <c r="Y2"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A3" s="122">
+      <c r="A3" s="106">
         <v>2</v>
       </c>
       <c r="B3" s="42">
@@ -6876,7 +7020,7 @@
       <c r="Y3"/>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A4" s="122">
+      <c r="A4" s="106">
         <v>3</v>
       </c>
       <c r="B4" s="42">
@@ -6925,7 +7069,7 @@
       <c r="Y4"/>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A5" s="122">
+      <c r="A5" s="106">
         <v>4</v>
       </c>
       <c r="B5" s="42">
@@ -6974,7 +7118,7 @@
       <c r="Y5"/>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A6" s="122">
+      <c r="A6" s="106">
         <v>5</v>
       </c>
       <c r="B6" s="42">
@@ -7023,7 +7167,7 @@
       <c r="Y6"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A7" s="122">
+      <c r="A7" s="106">
         <v>6</v>
       </c>
       <c r="B7" s="42">
@@ -7072,7 +7216,7 @@
       <c r="Y7"/>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A8" s="122">
+      <c r="A8" s="106">
         <v>7</v>
       </c>
       <c r="B8" s="42">
@@ -7121,7 +7265,7 @@
       <c r="Y8"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A9" s="122">
+      <c r="A9" s="106">
         <v>8</v>
       </c>
       <c r="B9" s="42">
@@ -7170,7 +7314,7 @@
       <c r="Y9"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A10" s="122">
+      <c r="A10" s="106">
         <v>9</v>
       </c>
       <c r="B10" s="42">
@@ -7219,7 +7363,7 @@
       <c r="Y10"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A11" s="122">
+      <c r="A11" s="106">
         <v>10</v>
       </c>
       <c r="B11" s="42">
@@ -7268,7 +7412,7 @@
       <c r="Y11"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A12" s="122">
+      <c r="A12" s="106">
         <v>11</v>
       </c>
       <c r="B12" s="42">
@@ -7317,7 +7461,7 @@
       <c r="Y12"/>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A13" s="122">
+      <c r="A13" s="106">
         <v>12</v>
       </c>
       <c r="B13" s="42">
@@ -7366,7 +7510,7 @@
       <c r="Y13"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A14" s="122">
+      <c r="A14" s="106">
         <v>13</v>
       </c>
       <c r="B14" s="42">
@@ -7415,7 +7559,7 @@
       <c r="Y14"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A15" s="122">
+      <c r="A15" s="106">
         <v>14</v>
       </c>
       <c r="B15" s="42">
@@ -7464,7 +7608,7 @@
       <c r="Y15"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A16" s="122">
+      <c r="A16" s="106">
         <v>15</v>
       </c>
       <c r="B16" s="42">
@@ -7513,7 +7657,7 @@
       <c r="Y16"/>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A17" s="122">
+      <c r="A17" s="106">
         <v>16</v>
       </c>
       <c r="B17" s="42">
@@ -7562,7 +7706,7 @@
       <c r="Y17"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A18" s="122">
+      <c r="A18" s="106">
         <v>17</v>
       </c>
       <c r="B18" s="42">
@@ -7611,7 +7755,7 @@
       <c r="Y18"/>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A19" s="122">
+      <c r="A19" s="106">
         <v>18</v>
       </c>
       <c r="B19" s="42">
@@ -7660,7 +7804,7 @@
       <c r="Y19"/>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A20" s="122">
+      <c r="A20" s="106">
         <v>19</v>
       </c>
       <c r="B20" s="42">
@@ -7709,7 +7853,7 @@
       <c r="Y20"/>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A21" s="122">
+      <c r="A21" s="106">
         <v>20</v>
       </c>
       <c r="B21" s="42">
@@ -7758,7 +7902,7 @@
       <c r="Y21"/>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A22" s="122">
+      <c r="A22" s="106">
         <v>21</v>
       </c>
       <c r="B22" s="42">
@@ -7807,7 +7951,7 @@
       <c r="Y22"/>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A23" s="122">
+      <c r="A23" s="106">
         <v>22</v>
       </c>
       <c r="B23" s="42">
@@ -7856,7 +8000,7 @@
       <c r="Y23"/>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A24" s="122">
+      <c r="A24" s="106">
         <v>23</v>
       </c>
       <c r="B24" s="42">
@@ -7905,7 +8049,7 @@
       <c r="Y24"/>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A25" s="122">
+      <c r="A25" s="106">
         <v>24</v>
       </c>
       <c r="B25" s="42">
@@ -7954,7 +8098,7 @@
       <c r="Y25"/>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A26" s="122">
+      <c r="A26" s="106">
         <v>25</v>
       </c>
       <c r="B26" s="42">
@@ -8003,7 +8147,7 @@
       <c r="Y26"/>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A27" s="122">
+      <c r="A27" s="106">
         <v>26</v>
       </c>
       <c r="B27" s="42">
@@ -8052,7 +8196,7 @@
       <c r="Y27"/>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A28" s="122">
+      <c r="A28" s="106">
         <v>27</v>
       </c>
       <c r="B28" s="42">
@@ -8101,7 +8245,7 @@
       <c r="Y28"/>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A29" s="122">
+      <c r="A29" s="106">
         <v>28</v>
       </c>
       <c r="B29" s="42">
@@ -8150,7 +8294,7 @@
       <c r="Y29"/>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A30" s="122">
+      <c r="A30" s="106">
         <v>29</v>
       </c>
       <c r="B30" s="42">
@@ -8199,7 +8343,7 @@
       <c r="Y30"/>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A31" s="122">
+      <c r="A31" s="106">
         <v>30</v>
       </c>
       <c r="B31" s="42">
@@ -8248,7 +8392,7 @@
       <c r="Y31"/>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A32" s="122">
+      <c r="A32" s="106">
         <v>31</v>
       </c>
       <c r="B32" s="42">
@@ -8297,7 +8441,7 @@
       <c r="Y32"/>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.4">
-      <c r="A33" s="122">
+      <c r="A33" s="106">
         <v>32</v>
       </c>
       <c r="B33" s="42">
@@ -10145,585 +10289,585 @@
       <c r="E5" s="44"/>
     </row>
     <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="119" t="s">
+      <c r="A6" s="103" t="s">
         <v>260</v>
       </c>
-      <c r="B6" s="119" t="s">
+      <c r="B6" s="103" t="s">
         <v>122</v>
       </c>
-      <c r="C6" s="119" t="s">
+      <c r="C6" s="103" t="s">
         <v>346</v>
       </c>
-      <c r="D6" s="119" t="s">
+      <c r="D6" s="103" t="s">
         <v>121</v>
       </c>
-      <c r="E6" s="120" t="s">
+      <c r="E6" s="104" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="119"/>
-      <c r="B7" s="119"/>
-      <c r="C7" s="119"/>
-      <c r="D7" s="119"/>
-      <c r="E7" s="120"/>
+      <c r="A7" s="103"/>
+      <c r="B7" s="103"/>
+      <c r="C7" s="103"/>
+      <c r="D7" s="103"/>
+      <c r="E7" s="104"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A8" s="119" t="s">
+      <c r="A8" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B8" s="119" t="s">
+      <c r="B8" s="103" t="s">
         <v>338</v>
       </c>
-      <c r="C8" s="119" t="s">
+      <c r="C8" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D8" s="119" t="s">
+      <c r="D8" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E8" s="120" t="s">
+      <c r="E8" s="104" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A9" s="119" t="s">
+      <c r="A9" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B9" s="119" t="s">
+      <c r="B9" s="103" t="s">
         <v>335</v>
       </c>
-      <c r="C9" s="119" t="s">
+      <c r="C9" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D9" s="119" t="s">
+      <c r="D9" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E9" s="120" t="s">
+      <c r="E9" s="104" t="s">
         <v>383</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A10" s="119" t="s">
+      <c r="A10" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B10" s="119" t="s">
+      <c r="B10" s="103" t="s">
         <v>334</v>
       </c>
-      <c r="C10" s="119" t="s">
+      <c r="C10" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D10" s="119" t="s">
+      <c r="D10" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E10" s="120" t="s">
+      <c r="E10" s="104" t="s">
         <v>382</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A11" s="119" t="s">
+      <c r="A11" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B11" s="119" t="s">
+      <c r="B11" s="103" t="s">
         <v>336</v>
       </c>
-      <c r="C11" s="119" t="s">
+      <c r="C11" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D11" s="119" t="s">
+      <c r="D11" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E11" s="120" t="s">
+      <c r="E11" s="104" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A12" s="119" t="s">
+      <c r="A12" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B12" s="119" t="s">
+      <c r="B12" s="103" t="s">
         <v>105</v>
       </c>
-      <c r="C12" s="119" t="s">
+      <c r="C12" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D12" s="119" t="s">
+      <c r="D12" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E12" s="121" t="s">
+      <c r="E12" s="105" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A13" s="119" t="s">
+      <c r="A13" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B13" s="119" t="s">
+      <c r="B13" s="103" t="s">
         <v>104</v>
       </c>
-      <c r="C13" s="119" t="s">
+      <c r="C13" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D13" s="119" t="s">
+      <c r="D13" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E13" s="120" t="s">
+      <c r="E13" s="104" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A14" s="119" t="s">
+      <c r="A14" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B14" s="119" t="s">
+      <c r="B14" s="103" t="s">
         <v>126</v>
       </c>
-      <c r="C14" s="119" t="s">
+      <c r="C14" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D14" s="119" t="s">
+      <c r="D14" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E14" s="120" t="s">
+      <c r="E14" s="104" t="s">
         <v>378</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A15" s="119" t="s">
+      <c r="A15" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B15" s="119" t="s">
+      <c r="B15" s="103" t="s">
         <v>333</v>
       </c>
-      <c r="C15" s="119" t="s">
+      <c r="C15" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D15" s="119" t="s">
+      <c r="D15" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E15" s="120" t="s">
+      <c r="E15" s="104" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A16" s="119" t="s">
+      <c r="A16" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B16" s="119" t="s">
+      <c r="B16" s="103" t="s">
         <v>341</v>
       </c>
-      <c r="C16" s="119" t="s">
+      <c r="C16" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D16" s="119" t="s">
+      <c r="D16" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E16" s="120" t="s">
+      <c r="E16" s="104" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A17" s="119" t="s">
+      <c r="A17" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B17" s="119" t="s">
+      <c r="B17" s="103" t="s">
         <v>106</v>
       </c>
-      <c r="C17" s="119" t="s">
+      <c r="C17" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D17" s="119" t="s">
+      <c r="D17" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E17" s="120" t="s">
+      <c r="E17" s="104" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A18" s="119" t="s">
+      <c r="A18" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B18" s="119" t="s">
+      <c r="B18" s="103" t="s">
         <v>339</v>
       </c>
-      <c r="C18" s="119" t="s">
+      <c r="C18" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D18" s="119" t="s">
+      <c r="D18" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E18" s="120" t="s">
+      <c r="E18" s="104" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A19" s="119" t="s">
+      <c r="A19" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B19" s="119" t="s">
+      <c r="B19" s="103" t="s">
         <v>337</v>
       </c>
-      <c r="C19" s="119" t="s">
+      <c r="C19" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D19" s="119" t="s">
+      <c r="D19" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E19" s="120" t="s">
+      <c r="E19" s="104" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A20" s="119" t="s">
+      <c r="A20" s="103" t="s">
         <v>258</v>
       </c>
-      <c r="B20" s="119" t="s">
+      <c r="B20" s="103" t="s">
         <v>340</v>
       </c>
-      <c r="C20" s="119" t="s">
+      <c r="C20" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D20" s="119" t="s">
+      <c r="D20" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E20" s="120" t="s">
+      <c r="E20" s="104" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A21" s="119" t="s">
+      <c r="A21" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B21" s="119" t="s">
+      <c r="B21" s="103" t="s">
         <v>345</v>
       </c>
-      <c r="C21" s="119" t="s">
+      <c r="C21" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D21" s="119" t="s">
+      <c r="D21" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E21" s="120" t="s">
+      <c r="E21" s="104" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A22" s="119" t="s">
+      <c r="A22" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B22" s="119" t="s">
+      <c r="B22" s="103" t="s">
         <v>348</v>
       </c>
-      <c r="C22" s="119"/>
-      <c r="D22" s="119"/>
-      <c r="E22" s="120" t="s">
+      <c r="C22" s="103"/>
+      <c r="D22" s="103"/>
+      <c r="E22" s="104" t="s">
         <v>385</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A23" s="119" t="s">
+      <c r="A23" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B23" s="119" t="s">
+      <c r="B23" s="103" t="s">
         <v>352</v>
       </c>
-      <c r="C23" s="119" t="s">
+      <c r="C23" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D23" s="119" t="s">
+      <c r="D23" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E23" s="120" t="s">
+      <c r="E23" s="104" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A24" s="119" t="s">
+      <c r="A24" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B24" s="119" t="s">
+      <c r="B24" s="103" t="s">
         <v>349</v>
       </c>
-      <c r="C24" s="119" t="s">
+      <c r="C24" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D24" s="119" t="s">
+      <c r="D24" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E24" s="120" t="s">
+      <c r="E24" s="104" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A25" s="119" t="s">
+      <c r="A25" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B25" s="119" t="s">
+      <c r="B25" s="103" t="s">
         <v>353</v>
       </c>
-      <c r="C25" s="119" t="s">
+      <c r="C25" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D25" s="119" t="s">
+      <c r="D25" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E25" s="120" t="s">
+      <c r="E25" s="104" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A26" s="119" t="s">
+      <c r="A26" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B26" s="119" t="s">
+      <c r="B26" s="103" t="s">
         <v>126</v>
       </c>
-      <c r="C26" s="119" t="s">
+      <c r="C26" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D26" s="119" t="s">
+      <c r="D26" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E26" s="120" t="s">
+      <c r="E26" s="104" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A27" s="119" t="s">
+      <c r="A27" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B27" s="119" t="s">
+      <c r="B27" s="103" t="s">
         <v>343</v>
       </c>
-      <c r="C27" s="119" t="s">
+      <c r="C27" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D27" s="119" t="s">
+      <c r="D27" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E27" s="120" t="s">
+      <c r="E27" s="104" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A28" s="119" t="s">
+      <c r="A28" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B28" s="119" t="s">
+      <c r="B28" s="103" t="s">
         <v>342</v>
       </c>
-      <c r="C28" s="119" t="s">
+      <c r="C28" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D28" s="119" t="s">
+      <c r="D28" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E28" s="120" t="s">
+      <c r="E28" s="104" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A29" s="119" t="s">
+      <c r="A29" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B29" s="119" t="s">
+      <c r="B29" s="103" t="s">
         <v>355</v>
       </c>
-      <c r="C29" s="119" t="s">
+      <c r="C29" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D29" s="119" t="s">
+      <c r="D29" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E29" s="120" t="s">
+      <c r="E29" s="104" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A30" s="119" t="s">
+      <c r="A30" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B30" s="119" t="s">
+      <c r="B30" s="103" t="s">
         <v>351</v>
       </c>
-      <c r="C30" s="119" t="s">
+      <c r="C30" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D30" s="119" t="s">
+      <c r="D30" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E30" s="120" t="s">
+      <c r="E30" s="104" t="s">
         <v>364</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A31" s="119" t="s">
+      <c r="A31" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B31" s="119" t="s">
+      <c r="B31" s="103" t="s">
         <v>354</v>
       </c>
-      <c r="C31" s="119" t="s">
+      <c r="C31" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D31" s="119" t="s">
+      <c r="D31" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E31" s="120" t="s">
+      <c r="E31" s="104" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A32" s="119" t="s">
+      <c r="A32" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B32" s="119" t="s">
+      <c r="B32" s="103" t="s">
         <v>356</v>
       </c>
-      <c r="C32" s="119" t="s">
+      <c r="C32" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D32" s="119" t="s">
+      <c r="D32" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E32" s="120" t="s">
+      <c r="E32" s="104" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A33" s="119" t="s">
+      <c r="A33" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B33" s="119" t="s">
+      <c r="B33" s="103" t="s">
         <v>127</v>
       </c>
-      <c r="C33" s="119" t="s">
+      <c r="C33" s="103" t="s">
         <v>220</v>
       </c>
-      <c r="D33" s="119"/>
-      <c r="E33" s="120" t="s">
+      <c r="D33" s="103"/>
+      <c r="E33" s="104" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A34" s="119" t="s">
+      <c r="A34" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B34" s="119" t="s">
+      <c r="B34" s="103" t="s">
         <v>344</v>
       </c>
-      <c r="C34" s="119" t="s">
+      <c r="C34" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D34" s="119" t="s">
+      <c r="D34" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E34" s="120" t="s">
+      <c r="E34" s="104" t="s">
         <v>362</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A35" s="119" t="s">
+      <c r="A35" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B35" s="119" t="s">
+      <c r="B35" s="103" t="s">
         <v>128</v>
       </c>
-      <c r="C35" s="119" t="s">
+      <c r="C35" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D35" s="119" t="s">
+      <c r="D35" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E35" s="120" t="s">
+      <c r="E35" s="104" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A36" s="119" t="s">
+      <c r="A36" s="103" t="s">
         <v>259</v>
       </c>
-      <c r="B36" s="119" t="s">
+      <c r="B36" s="103" t="s">
         <v>350</v>
       </c>
-      <c r="C36" s="119" t="s">
+      <c r="C36" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="D36" s="119" t="s">
+      <c r="D36" s="103" t="s">
         <v>347</v>
       </c>
-      <c r="E36" s="120" t="s">
+      <c r="E36" s="104" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="119"/>
-      <c r="B37" s="119"/>
-      <c r="C37" s="119"/>
-      <c r="D37" s="119"/>
-      <c r="E37" s="120"/>
+      <c r="A37" s="103"/>
+      <c r="B37" s="103"/>
+      <c r="C37" s="103"/>
+      <c r="D37" s="103"/>
+      <c r="E37" s="104"/>
     </row>
     <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="119"/>
-      <c r="B38" s="119"/>
-      <c r="C38" s="119"/>
-      <c r="D38" s="119"/>
-      <c r="E38" s="120"/>
+      <c r="A38" s="103"/>
+      <c r="B38" s="103"/>
+      <c r="C38" s="103"/>
+      <c r="D38" s="103"/>
+      <c r="E38" s="104"/>
     </row>
     <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="119"/>
-      <c r="B39" s="119"/>
-      <c r="C39" s="119"/>
-      <c r="D39" s="119"/>
-      <c r="E39" s="120"/>
+      <c r="A39" s="103"/>
+      <c r="B39" s="103"/>
+      <c r="C39" s="103"/>
+      <c r="D39" s="103"/>
+      <c r="E39" s="104"/>
     </row>
     <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="119"/>
-      <c r="B40" s="119"/>
-      <c r="C40" s="119"/>
-      <c r="D40" s="119"/>
-      <c r="E40" s="120"/>
+      <c r="A40" s="103"/>
+      <c r="B40" s="103"/>
+      <c r="C40" s="103"/>
+      <c r="D40" s="103"/>
+      <c r="E40" s="104"/>
     </row>
     <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="119"/>
-      <c r="B41" s="119"/>
-      <c r="C41" s="119"/>
-      <c r="D41" s="119"/>
-      <c r="E41" s="120"/>
+      <c r="A41" s="103"/>
+      <c r="B41" s="103"/>
+      <c r="C41" s="103"/>
+      <c r="D41" s="103"/>
+      <c r="E41" s="104"/>
     </row>
     <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="119"/>
-      <c r="B42" s="119"/>
-      <c r="C42" s="119"/>
-      <c r="D42" s="119"/>
-      <c r="E42" s="120"/>
+      <c r="A42" s="103"/>
+      <c r="B42" s="103"/>
+      <c r="C42" s="103"/>
+      <c r="D42" s="103"/>
+      <c r="E42" s="104"/>
     </row>
     <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="119"/>
-      <c r="B43" s="119"/>
-      <c r="C43" s="119"/>
-      <c r="D43" s="119"/>
-      <c r="E43" s="120"/>
+      <c r="A43" s="103"/>
+      <c r="B43" s="103"/>
+      <c r="C43" s="103"/>
+      <c r="D43" s="103"/>
+      <c r="E43" s="104"/>
     </row>
     <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="119"/>
-      <c r="B44" s="119"/>
-      <c r="C44" s="119"/>
-      <c r="D44" s="119"/>
-      <c r="E44" s="120"/>
+      <c r="A44" s="103"/>
+      <c r="B44" s="103"/>
+      <c r="C44" s="103"/>
+      <c r="D44" s="103"/>
+      <c r="E44" s="104"/>
     </row>
     <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A45" s="119"/>
-      <c r="B45" s="119"/>
-      <c r="C45" s="119"/>
-      <c r="D45" s="119"/>
-      <c r="E45" s="120"/>
+      <c r="A45" s="103"/>
+      <c r="B45" s="103"/>
+      <c r="C45" s="103"/>
+      <c r="D45" s="103"/>
+      <c r="E45" s="104"/>
     </row>
     <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A46" s="119"/>
-      <c r="B46" s="119"/>
-      <c r="C46" s="119"/>
-      <c r="D46" s="119"/>
-      <c r="E46" s="120"/>
+      <c r="A46" s="103"/>
+      <c r="B46" s="103"/>
+      <c r="C46" s="103"/>
+      <c r="D46" s="103"/>
+      <c r="E46" s="104"/>
     </row>
     <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.4">
       <c r="E47" s="44"/>

</xml_diff>